<commit_message>
Money Out now entered as negative numbers
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HQ5Ghz8CrBGJ5WjxLz3zBX
</commit_message>
<xml_diff>
--- a/Cash_and_Debtors_Tracker.xlsx
+++ b/Cash_and_Debtors_Tracker.xlsx
@@ -53,7 +53,7 @@
     <t xml:space="preserve">HOW TO USE (3 steps)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Cash Book: record every cash/bank movement. Money received goes in 'Money In', money paid goes in 'Money Out'. Balance updates itself.</t>
+    <t xml:space="preserve">1. Cash Book: record every cash/bank movement. Money received goes in 'Money In', money paid goes in 'Money Out' as a NEGATIVE number (rent of 200 = -200). Balance updates itself.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Invoices: when you sell on credit, record the invoice (client, amount, due date).</t>
@@ -149,7 +149,7 @@
     <t xml:space="preserve">Cash Book - money in and money out</t>
   </si>
   <si>
-    <t xml:space="preserve">Type in yellow columns only. Balance is automatic.</t>
+    <t xml:space="preserve">Type in yellow columns only. Money In = positive, Money Out = negative (e.g. -200). Balance is automatic.</t>
   </si>
   <si>
     <t xml:space="preserve">Date</t>
@@ -164,7 +164,8 @@
     <t xml:space="preserve">Money In</t>
   </si>
   <si>
-    <t xml:space="preserve">Money Out</t>
+    <t xml:space="preserve">Money Out
+(enter as -)</t>
   </si>
   <si>
     <t xml:space="preserve">Balance</t>
@@ -1023,7 +1024,7 @@
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">SUM('Cash Book'!E5:E504)</f>
-        <v>300</v>
+        <v>-300</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1031,7 +1032,7 @@
         <v>31</v>
       </c>
       <c r="B7" s="11" t="n">
-        <f aca="false">B4+B5-B6</f>
+        <f aca="false">B4+B5+B6</f>
         <v>200</v>
       </c>
     </row>
@@ -1089,7 +1090,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="16" t="n">
-        <f aca="false">B14-C14</f>
+        <f aca="false">B14+C14</f>
         <v>0</v>
       </c>
     </row>
@@ -1107,7 +1108,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="16" t="n">
-        <f aca="false">B15-C15</f>
+        <f aca="false">B15+C15</f>
         <v>0</v>
       </c>
     </row>
@@ -1125,7 +1126,7 @@
         <v>0</v>
       </c>
       <c r="D16" s="16" t="n">
-        <f aca="false">B16-C16</f>
+        <f aca="false">B16+C16</f>
         <v>0</v>
       </c>
     </row>
@@ -1143,7 +1144,7 @@
         <v>0</v>
       </c>
       <c r="D17" s="16" t="n">
-        <f aca="false">B17-C17</f>
+        <f aca="false">B17+C17</f>
         <v>0</v>
       </c>
     </row>
@@ -1161,7 +1162,7 @@
         <v>0</v>
       </c>
       <c r="D18" s="16" t="n">
-        <f aca="false">B18-C18</f>
+        <f aca="false">B18+C18</f>
         <v>0</v>
       </c>
     </row>
@@ -1179,7 +1180,7 @@
         <v>0</v>
       </c>
       <c r="D19" s="16" t="n">
-        <f aca="false">B19-C19</f>
+        <f aca="false">B19+C19</f>
         <v>0</v>
       </c>
     </row>
@@ -1197,7 +1198,7 @@
         <v>0</v>
       </c>
       <c r="D20" s="16" t="n">
-        <f aca="false">B20-C20</f>
+        <f aca="false">B20+C20</f>
         <v>0</v>
       </c>
     </row>
@@ -1215,7 +1216,7 @@
         <v>0</v>
       </c>
       <c r="D21" s="16" t="n">
-        <f aca="false">B21-C21</f>
+        <f aca="false">B21+C21</f>
         <v>0</v>
       </c>
     </row>
@@ -1233,7 +1234,7 @@
         <v>0</v>
       </c>
       <c r="D22" s="16" t="n">
-        <f aca="false">B22-C22</f>
+        <f aca="false">B22+C22</f>
         <v>0</v>
       </c>
     </row>
@@ -1248,10 +1249,10 @@
       </c>
       <c r="C23" s="16" t="n">
         <f aca="false">SUMIFS('Cash Book'!$E$5:$E$504,'Cash Book'!$A$5:$A$504,"&gt;="&amp;$A23,'Cash Book'!$A$5:$A$504,"&lt;"&amp;DATE($B$11,11,1))</f>
-        <v>300</v>
+        <v>-300</v>
       </c>
       <c r="D23" s="16" t="n">
-        <f aca="false">B23-C23</f>
+        <f aca="false">B23+C23</f>
         <v>200</v>
       </c>
     </row>
@@ -1269,7 +1270,7 @@
         <v>0</v>
       </c>
       <c r="D24" s="16" t="n">
-        <f aca="false">B24-C24</f>
+        <f aca="false">B24+C24</f>
         <v>0</v>
       </c>
     </row>
@@ -1287,7 +1288,7 @@
         <v>0</v>
       </c>
       <c r="D25" s="16" t="n">
-        <f aca="false">B25-C25</f>
+        <f aca="false">B25+C25</f>
         <v>0</v>
       </c>
     </row>
@@ -1301,7 +1302,7 @@
       </c>
       <c r="C26" s="17" t="n">
         <f aca="false">SUM(C14:C25)</f>
-        <v>300</v>
+        <v>-300</v>
       </c>
       <c r="D26" s="17" t="n">
         <f aca="false">SUM(D14:D25)</f>
@@ -1388,7 +1389,7 @@
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="20" t="n">
-        <f aca="false">IF(AND(D5="",E5=""),"",'Start Here'!$B$4+SUM($D$5:D5)-SUM($E$5:E5))</f>
+        <f aca="false">IF(AND(D5="",E5=""),"",'Start Here'!$B$4+SUM($D$5:D5)+SUM($E$5:E5))</f>
         <v>500</v>
       </c>
       <c r="G5" s="5" t="s">
@@ -1407,10 +1408,10 @@
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4" t="n">
-        <v>300</v>
+        <v>-300</v>
       </c>
       <c r="F6" s="20" t="n">
-        <f aca="false">IF(AND(D6="",E6=""),"",'Start Here'!$B$4+SUM($D$5:D6)-SUM($E$5:E6))</f>
+        <f aca="false">IF(AND(D6="",E6=""),"",'Start Here'!$B$4+SUM($D$5:D6)+SUM($E$5:E6))</f>
         <v>200</v>
       </c>
       <c r="G6" s="5"/>
@@ -1422,7 +1423,7 @@
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="F7" s="20" t="str">
-        <f aca="false">IF(AND(D7="",E7=""),"",'Start Here'!$B$4+SUM($D$5:D7)-SUM($E$5:E7))</f>
+        <f aca="false">IF(AND(D7="",E7=""),"",'Start Here'!$B$4+SUM($D$5:D7)+SUM($E$5:E7))</f>
         <v/>
       </c>
       <c r="G7" s="5"/>
@@ -1434,7 +1435,7 @@
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
       <c r="F8" s="20" t="str">
-        <f aca="false">IF(AND(D8="",E8=""),"",'Start Here'!$B$4+SUM($D$5:D8)-SUM($E$5:E8))</f>
+        <f aca="false">IF(AND(D8="",E8=""),"",'Start Here'!$B$4+SUM($D$5:D8)+SUM($E$5:E8))</f>
         <v/>
       </c>
       <c r="G8" s="5"/>
@@ -1446,7 +1447,7 @@
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
       <c r="F9" s="20" t="str">
-        <f aca="false">IF(AND(D9="",E9=""),"",'Start Here'!$B$4+SUM($D$5:D9)-SUM($E$5:E9))</f>
+        <f aca="false">IF(AND(D9="",E9=""),"",'Start Here'!$B$4+SUM($D$5:D9)+SUM($E$5:E9))</f>
         <v/>
       </c>
       <c r="G9" s="5"/>
@@ -1458,7 +1459,7 @@
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
       <c r="F10" s="20" t="str">
-        <f aca="false">IF(AND(D10="",E10=""),"",'Start Here'!$B$4+SUM($D$5:D10)-SUM($E$5:E10))</f>
+        <f aca="false">IF(AND(D10="",E10=""),"",'Start Here'!$B$4+SUM($D$5:D10)+SUM($E$5:E10))</f>
         <v/>
       </c>
       <c r="G10" s="5"/>
@@ -1470,7 +1471,7 @@
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
       <c r="F11" s="20" t="str">
-        <f aca="false">IF(AND(D11="",E11=""),"",'Start Here'!$B$4+SUM($D$5:D11)-SUM($E$5:E11))</f>
+        <f aca="false">IF(AND(D11="",E11=""),"",'Start Here'!$B$4+SUM($D$5:D11)+SUM($E$5:E11))</f>
         <v/>
       </c>
       <c r="G11" s="5"/>
@@ -1482,7 +1483,7 @@
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
       <c r="F12" s="20" t="str">
-        <f aca="false">IF(AND(D12="",E12=""),"",'Start Here'!$B$4+SUM($D$5:D12)-SUM($E$5:E12))</f>
+        <f aca="false">IF(AND(D12="",E12=""),"",'Start Here'!$B$4+SUM($D$5:D12)+SUM($E$5:E12))</f>
         <v/>
       </c>
       <c r="G12" s="5"/>
@@ -1494,7 +1495,7 @@
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
       <c r="F13" s="20" t="str">
-        <f aca="false">IF(AND(D13="",E13=""),"",'Start Here'!$B$4+SUM($D$5:D13)-SUM($E$5:E13))</f>
+        <f aca="false">IF(AND(D13="",E13=""),"",'Start Here'!$B$4+SUM($D$5:D13)+SUM($E$5:E13))</f>
         <v/>
       </c>
       <c r="G13" s="5"/>
@@ -1506,7 +1507,7 @@
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
       <c r="F14" s="20" t="str">
-        <f aca="false">IF(AND(D14="",E14=""),"",'Start Here'!$B$4+SUM($D$5:D14)-SUM($E$5:E14))</f>
+        <f aca="false">IF(AND(D14="",E14=""),"",'Start Here'!$B$4+SUM($D$5:D14)+SUM($E$5:E14))</f>
         <v/>
       </c>
       <c r="G14" s="5"/>
@@ -1518,7 +1519,7 @@
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
       <c r="F15" s="20" t="str">
-        <f aca="false">IF(AND(D15="",E15=""),"",'Start Here'!$B$4+SUM($D$5:D15)-SUM($E$5:E15))</f>
+        <f aca="false">IF(AND(D15="",E15=""),"",'Start Here'!$B$4+SUM($D$5:D15)+SUM($E$5:E15))</f>
         <v/>
       </c>
       <c r="G15" s="5"/>
@@ -1530,7 +1531,7 @@
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="20" t="str">
-        <f aca="false">IF(AND(D16="",E16=""),"",'Start Here'!$B$4+SUM($D$5:D16)-SUM($E$5:E16))</f>
+        <f aca="false">IF(AND(D16="",E16=""),"",'Start Here'!$B$4+SUM($D$5:D16)+SUM($E$5:E16))</f>
         <v/>
       </c>
       <c r="G16" s="5"/>
@@ -1542,7 +1543,7 @@
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="20" t="str">
-        <f aca="false">IF(AND(D17="",E17=""),"",'Start Here'!$B$4+SUM($D$5:D17)-SUM($E$5:E17))</f>
+        <f aca="false">IF(AND(D17="",E17=""),"",'Start Here'!$B$4+SUM($D$5:D17)+SUM($E$5:E17))</f>
         <v/>
       </c>
       <c r="G17" s="5"/>
@@ -1554,7 +1555,7 @@
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
       <c r="F18" s="20" t="str">
-        <f aca="false">IF(AND(D18="",E18=""),"",'Start Here'!$B$4+SUM($D$5:D18)-SUM($E$5:E18))</f>
+        <f aca="false">IF(AND(D18="",E18=""),"",'Start Here'!$B$4+SUM($D$5:D18)+SUM($E$5:E18))</f>
         <v/>
       </c>
       <c r="G18" s="5"/>
@@ -1566,7 +1567,7 @@
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
       <c r="F19" s="20" t="str">
-        <f aca="false">IF(AND(D19="",E19=""),"",'Start Here'!$B$4+SUM($D$5:D19)-SUM($E$5:E19))</f>
+        <f aca="false">IF(AND(D19="",E19=""),"",'Start Here'!$B$4+SUM($D$5:D19)+SUM($E$5:E19))</f>
         <v/>
       </c>
       <c r="G19" s="5"/>
@@ -1578,7 +1579,7 @@
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
       <c r="F20" s="20" t="str">
-        <f aca="false">IF(AND(D20="",E20=""),"",'Start Here'!$B$4+SUM($D$5:D20)-SUM($E$5:E20))</f>
+        <f aca="false">IF(AND(D20="",E20=""),"",'Start Here'!$B$4+SUM($D$5:D20)+SUM($E$5:E20))</f>
         <v/>
       </c>
       <c r="G20" s="5"/>
@@ -1590,7 +1591,7 @@
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
       <c r="F21" s="20" t="str">
-        <f aca="false">IF(AND(D21="",E21=""),"",'Start Here'!$B$4+SUM($D$5:D21)-SUM($E$5:E21))</f>
+        <f aca="false">IF(AND(D21="",E21=""),"",'Start Here'!$B$4+SUM($D$5:D21)+SUM($E$5:E21))</f>
         <v/>
       </c>
       <c r="G21" s="5"/>
@@ -1602,7 +1603,7 @@
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
       <c r="F22" s="20" t="str">
-        <f aca="false">IF(AND(D22="",E22=""),"",'Start Here'!$B$4+SUM($D$5:D22)-SUM($E$5:E22))</f>
+        <f aca="false">IF(AND(D22="",E22=""),"",'Start Here'!$B$4+SUM($D$5:D22)+SUM($E$5:E22))</f>
         <v/>
       </c>
       <c r="G22" s="5"/>
@@ -1614,7 +1615,7 @@
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
       <c r="F23" s="20" t="str">
-        <f aca="false">IF(AND(D23="",E23=""),"",'Start Here'!$B$4+SUM($D$5:D23)-SUM($E$5:E23))</f>
+        <f aca="false">IF(AND(D23="",E23=""),"",'Start Here'!$B$4+SUM($D$5:D23)+SUM($E$5:E23))</f>
         <v/>
       </c>
       <c r="G23" s="5"/>
@@ -1626,7 +1627,7 @@
       <c r="D24" s="4"/>
       <c r="E24" s="4"/>
       <c r="F24" s="20" t="str">
-        <f aca="false">IF(AND(D24="",E24=""),"",'Start Here'!$B$4+SUM($D$5:D24)-SUM($E$5:E24))</f>
+        <f aca="false">IF(AND(D24="",E24=""),"",'Start Here'!$B$4+SUM($D$5:D24)+SUM($E$5:E24))</f>
         <v/>
       </c>
       <c r="G24" s="5"/>
@@ -1638,7 +1639,7 @@
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
       <c r="F25" s="20" t="str">
-        <f aca="false">IF(AND(D25="",E25=""),"",'Start Here'!$B$4+SUM($D$5:D25)-SUM($E$5:E25))</f>
+        <f aca="false">IF(AND(D25="",E25=""),"",'Start Here'!$B$4+SUM($D$5:D25)+SUM($E$5:E25))</f>
         <v/>
       </c>
       <c r="G25" s="5"/>
@@ -1650,7 +1651,7 @@
       <c r="D26" s="4"/>
       <c r="E26" s="4"/>
       <c r="F26" s="20" t="str">
-        <f aca="false">IF(AND(D26="",E26=""),"",'Start Here'!$B$4+SUM($D$5:D26)-SUM($E$5:E26))</f>
+        <f aca="false">IF(AND(D26="",E26=""),"",'Start Here'!$B$4+SUM($D$5:D26)+SUM($E$5:E26))</f>
         <v/>
       </c>
       <c r="G26" s="5"/>
@@ -1662,7 +1663,7 @@
       <c r="D27" s="4"/>
       <c r="E27" s="4"/>
       <c r="F27" s="20" t="str">
-        <f aca="false">IF(AND(D27="",E27=""),"",'Start Here'!$B$4+SUM($D$5:D27)-SUM($E$5:E27))</f>
+        <f aca="false">IF(AND(D27="",E27=""),"",'Start Here'!$B$4+SUM($D$5:D27)+SUM($E$5:E27))</f>
         <v/>
       </c>
       <c r="G27" s="5"/>
@@ -1674,7 +1675,7 @@
       <c r="D28" s="4"/>
       <c r="E28" s="4"/>
       <c r="F28" s="20" t="str">
-        <f aca="false">IF(AND(D28="",E28=""),"",'Start Here'!$B$4+SUM($D$5:D28)-SUM($E$5:E28))</f>
+        <f aca="false">IF(AND(D28="",E28=""),"",'Start Here'!$B$4+SUM($D$5:D28)+SUM($E$5:E28))</f>
         <v/>
       </c>
       <c r="G28" s="5"/>
@@ -1686,7 +1687,7 @@
       <c r="D29" s="4"/>
       <c r="E29" s="4"/>
       <c r="F29" s="20" t="str">
-        <f aca="false">IF(AND(D29="",E29=""),"",'Start Here'!$B$4+SUM($D$5:D29)-SUM($E$5:E29))</f>
+        <f aca="false">IF(AND(D29="",E29=""),"",'Start Here'!$B$4+SUM($D$5:D29)+SUM($E$5:E29))</f>
         <v/>
       </c>
       <c r="G29" s="5"/>
@@ -1698,7 +1699,7 @@
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
       <c r="F30" s="20" t="str">
-        <f aca="false">IF(AND(D30="",E30=""),"",'Start Here'!$B$4+SUM($D$5:D30)-SUM($E$5:E30))</f>
+        <f aca="false">IF(AND(D30="",E30=""),"",'Start Here'!$B$4+SUM($D$5:D30)+SUM($E$5:E30))</f>
         <v/>
       </c>
       <c r="G30" s="5"/>
@@ -1710,7 +1711,7 @@
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
       <c r="F31" s="20" t="str">
-        <f aca="false">IF(AND(D31="",E31=""),"",'Start Here'!$B$4+SUM($D$5:D31)-SUM($E$5:E31))</f>
+        <f aca="false">IF(AND(D31="",E31=""),"",'Start Here'!$B$4+SUM($D$5:D31)+SUM($E$5:E31))</f>
         <v/>
       </c>
       <c r="G31" s="5"/>
@@ -1722,7 +1723,7 @@
       <c r="D32" s="4"/>
       <c r="E32" s="4"/>
       <c r="F32" s="20" t="str">
-        <f aca="false">IF(AND(D32="",E32=""),"",'Start Here'!$B$4+SUM($D$5:D32)-SUM($E$5:E32))</f>
+        <f aca="false">IF(AND(D32="",E32=""),"",'Start Here'!$B$4+SUM($D$5:D32)+SUM($E$5:E32))</f>
         <v/>
       </c>
       <c r="G32" s="5"/>
@@ -1734,7 +1735,7 @@
       <c r="D33" s="4"/>
       <c r="E33" s="4"/>
       <c r="F33" s="20" t="str">
-        <f aca="false">IF(AND(D33="",E33=""),"",'Start Here'!$B$4+SUM($D$5:D33)-SUM($E$5:E33))</f>
+        <f aca="false">IF(AND(D33="",E33=""),"",'Start Here'!$B$4+SUM($D$5:D33)+SUM($E$5:E33))</f>
         <v/>
       </c>
       <c r="G33" s="5"/>
@@ -1746,7 +1747,7 @@
       <c r="D34" s="4"/>
       <c r="E34" s="4"/>
       <c r="F34" s="20" t="str">
-        <f aca="false">IF(AND(D34="",E34=""),"",'Start Here'!$B$4+SUM($D$5:D34)-SUM($E$5:E34))</f>
+        <f aca="false">IF(AND(D34="",E34=""),"",'Start Here'!$B$4+SUM($D$5:D34)+SUM($E$5:E34))</f>
         <v/>
       </c>
       <c r="G34" s="5"/>
@@ -1758,7 +1759,7 @@
       <c r="D35" s="4"/>
       <c r="E35" s="4"/>
       <c r="F35" s="20" t="str">
-        <f aca="false">IF(AND(D35="",E35=""),"",'Start Here'!$B$4+SUM($D$5:D35)-SUM($E$5:E35))</f>
+        <f aca="false">IF(AND(D35="",E35=""),"",'Start Here'!$B$4+SUM($D$5:D35)+SUM($E$5:E35))</f>
         <v/>
       </c>
       <c r="G35" s="5"/>
@@ -1770,7 +1771,7 @@
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
       <c r="F36" s="20" t="str">
-        <f aca="false">IF(AND(D36="",E36=""),"",'Start Here'!$B$4+SUM($D$5:D36)-SUM($E$5:E36))</f>
+        <f aca="false">IF(AND(D36="",E36=""),"",'Start Here'!$B$4+SUM($D$5:D36)+SUM($E$5:E36))</f>
         <v/>
       </c>
       <c r="G36" s="5"/>
@@ -1782,7 +1783,7 @@
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
       <c r="F37" s="20" t="str">
-        <f aca="false">IF(AND(D37="",E37=""),"",'Start Here'!$B$4+SUM($D$5:D37)-SUM($E$5:E37))</f>
+        <f aca="false">IF(AND(D37="",E37=""),"",'Start Here'!$B$4+SUM($D$5:D37)+SUM($E$5:E37))</f>
         <v/>
       </c>
       <c r="G37" s="5"/>
@@ -1794,7 +1795,7 @@
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
       <c r="F38" s="20" t="str">
-        <f aca="false">IF(AND(D38="",E38=""),"",'Start Here'!$B$4+SUM($D$5:D38)-SUM($E$5:E38))</f>
+        <f aca="false">IF(AND(D38="",E38=""),"",'Start Here'!$B$4+SUM($D$5:D38)+SUM($E$5:E38))</f>
         <v/>
       </c>
       <c r="G38" s="5"/>
@@ -1806,7 +1807,7 @@
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
       <c r="F39" s="20" t="str">
-        <f aca="false">IF(AND(D39="",E39=""),"",'Start Here'!$B$4+SUM($D$5:D39)-SUM($E$5:E39))</f>
+        <f aca="false">IF(AND(D39="",E39=""),"",'Start Here'!$B$4+SUM($D$5:D39)+SUM($E$5:E39))</f>
         <v/>
       </c>
       <c r="G39" s="5"/>
@@ -1818,7 +1819,7 @@
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
       <c r="F40" s="20" t="str">
-        <f aca="false">IF(AND(D40="",E40=""),"",'Start Here'!$B$4+SUM($D$5:D40)-SUM($E$5:E40))</f>
+        <f aca="false">IF(AND(D40="",E40=""),"",'Start Here'!$B$4+SUM($D$5:D40)+SUM($E$5:E40))</f>
         <v/>
       </c>
       <c r="G40" s="5"/>
@@ -1830,7 +1831,7 @@
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
       <c r="F41" s="20" t="str">
-        <f aca="false">IF(AND(D41="",E41=""),"",'Start Here'!$B$4+SUM($D$5:D41)-SUM($E$5:E41))</f>
+        <f aca="false">IF(AND(D41="",E41=""),"",'Start Here'!$B$4+SUM($D$5:D41)+SUM($E$5:E41))</f>
         <v/>
       </c>
       <c r="G41" s="5"/>
@@ -1842,7 +1843,7 @@
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
       <c r="F42" s="20" t="str">
-        <f aca="false">IF(AND(D42="",E42=""),"",'Start Here'!$B$4+SUM($D$5:D42)-SUM($E$5:E42))</f>
+        <f aca="false">IF(AND(D42="",E42=""),"",'Start Here'!$B$4+SUM($D$5:D42)+SUM($E$5:E42))</f>
         <v/>
       </c>
       <c r="G42" s="5"/>
@@ -1854,7 +1855,7 @@
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>
       <c r="F43" s="20" t="str">
-        <f aca="false">IF(AND(D43="",E43=""),"",'Start Here'!$B$4+SUM($D$5:D43)-SUM($E$5:E43))</f>
+        <f aca="false">IF(AND(D43="",E43=""),"",'Start Here'!$B$4+SUM($D$5:D43)+SUM($E$5:E43))</f>
         <v/>
       </c>
       <c r="G43" s="5"/>
@@ -1866,7 +1867,7 @@
       <c r="D44" s="4"/>
       <c r="E44" s="4"/>
       <c r="F44" s="20" t="str">
-        <f aca="false">IF(AND(D44="",E44=""),"",'Start Here'!$B$4+SUM($D$5:D44)-SUM($E$5:E44))</f>
+        <f aca="false">IF(AND(D44="",E44=""),"",'Start Here'!$B$4+SUM($D$5:D44)+SUM($E$5:E44))</f>
         <v/>
       </c>
       <c r="G44" s="5"/>
@@ -1878,7 +1879,7 @@
       <c r="D45" s="4"/>
       <c r="E45" s="4"/>
       <c r="F45" s="20" t="str">
-        <f aca="false">IF(AND(D45="",E45=""),"",'Start Here'!$B$4+SUM($D$5:D45)-SUM($E$5:E45))</f>
+        <f aca="false">IF(AND(D45="",E45=""),"",'Start Here'!$B$4+SUM($D$5:D45)+SUM($E$5:E45))</f>
         <v/>
       </c>
       <c r="G45" s="5"/>
@@ -1890,7 +1891,7 @@
       <c r="D46" s="4"/>
       <c r="E46" s="4"/>
       <c r="F46" s="20" t="str">
-        <f aca="false">IF(AND(D46="",E46=""),"",'Start Here'!$B$4+SUM($D$5:D46)-SUM($E$5:E46))</f>
+        <f aca="false">IF(AND(D46="",E46=""),"",'Start Here'!$B$4+SUM($D$5:D46)+SUM($E$5:E46))</f>
         <v/>
       </c>
       <c r="G46" s="5"/>
@@ -1902,7 +1903,7 @@
       <c r="D47" s="4"/>
       <c r="E47" s="4"/>
       <c r="F47" s="20" t="str">
-        <f aca="false">IF(AND(D47="",E47=""),"",'Start Here'!$B$4+SUM($D$5:D47)-SUM($E$5:E47))</f>
+        <f aca="false">IF(AND(D47="",E47=""),"",'Start Here'!$B$4+SUM($D$5:D47)+SUM($E$5:E47))</f>
         <v/>
       </c>
       <c r="G47" s="5"/>
@@ -1914,7 +1915,7 @@
       <c r="D48" s="4"/>
       <c r="E48" s="4"/>
       <c r="F48" s="20" t="str">
-        <f aca="false">IF(AND(D48="",E48=""),"",'Start Here'!$B$4+SUM($D$5:D48)-SUM($E$5:E48))</f>
+        <f aca="false">IF(AND(D48="",E48=""),"",'Start Here'!$B$4+SUM($D$5:D48)+SUM($E$5:E48))</f>
         <v/>
       </c>
       <c r="G48" s="5"/>
@@ -1926,7 +1927,7 @@
       <c r="D49" s="4"/>
       <c r="E49" s="4"/>
       <c r="F49" s="20" t="str">
-        <f aca="false">IF(AND(D49="",E49=""),"",'Start Here'!$B$4+SUM($D$5:D49)-SUM($E$5:E49))</f>
+        <f aca="false">IF(AND(D49="",E49=""),"",'Start Here'!$B$4+SUM($D$5:D49)+SUM($E$5:E49))</f>
         <v/>
       </c>
       <c r="G49" s="5"/>
@@ -1938,7 +1939,7 @@
       <c r="D50" s="4"/>
       <c r="E50" s="4"/>
       <c r="F50" s="20" t="str">
-        <f aca="false">IF(AND(D50="",E50=""),"",'Start Here'!$B$4+SUM($D$5:D50)-SUM($E$5:E50))</f>
+        <f aca="false">IF(AND(D50="",E50=""),"",'Start Here'!$B$4+SUM($D$5:D50)+SUM($E$5:E50))</f>
         <v/>
       </c>
       <c r="G50" s="5"/>
@@ -1950,7 +1951,7 @@
       <c r="D51" s="4"/>
       <c r="E51" s="4"/>
       <c r="F51" s="20" t="str">
-        <f aca="false">IF(AND(D51="",E51=""),"",'Start Here'!$B$4+SUM($D$5:D51)-SUM($E$5:E51))</f>
+        <f aca="false">IF(AND(D51="",E51=""),"",'Start Here'!$B$4+SUM($D$5:D51)+SUM($E$5:E51))</f>
         <v/>
       </c>
       <c r="G51" s="5"/>
@@ -1962,7 +1963,7 @@
       <c r="D52" s="4"/>
       <c r="E52" s="4"/>
       <c r="F52" s="20" t="str">
-        <f aca="false">IF(AND(D52="",E52=""),"",'Start Here'!$B$4+SUM($D$5:D52)-SUM($E$5:E52))</f>
+        <f aca="false">IF(AND(D52="",E52=""),"",'Start Here'!$B$4+SUM($D$5:D52)+SUM($E$5:E52))</f>
         <v/>
       </c>
       <c r="G52" s="5"/>
@@ -1974,7 +1975,7 @@
       <c r="D53" s="4"/>
       <c r="E53" s="4"/>
       <c r="F53" s="20" t="str">
-        <f aca="false">IF(AND(D53="",E53=""),"",'Start Here'!$B$4+SUM($D$5:D53)-SUM($E$5:E53))</f>
+        <f aca="false">IF(AND(D53="",E53=""),"",'Start Here'!$B$4+SUM($D$5:D53)+SUM($E$5:E53))</f>
         <v/>
       </c>
       <c r="G53" s="5"/>
@@ -1986,7 +1987,7 @@
       <c r="D54" s="4"/>
       <c r="E54" s="4"/>
       <c r="F54" s="20" t="str">
-        <f aca="false">IF(AND(D54="",E54=""),"",'Start Here'!$B$4+SUM($D$5:D54)-SUM($E$5:E54))</f>
+        <f aca="false">IF(AND(D54="",E54=""),"",'Start Here'!$B$4+SUM($D$5:D54)+SUM($E$5:E54))</f>
         <v/>
       </c>
       <c r="G54" s="5"/>
@@ -1998,7 +1999,7 @@
       <c r="D55" s="4"/>
       <c r="E55" s="4"/>
       <c r="F55" s="20" t="str">
-        <f aca="false">IF(AND(D55="",E55=""),"",'Start Here'!$B$4+SUM($D$5:D55)-SUM($E$5:E55))</f>
+        <f aca="false">IF(AND(D55="",E55=""),"",'Start Here'!$B$4+SUM($D$5:D55)+SUM($E$5:E55))</f>
         <v/>
       </c>
       <c r="G55" s="5"/>
@@ -2010,7 +2011,7 @@
       <c r="D56" s="4"/>
       <c r="E56" s="4"/>
       <c r="F56" s="20" t="str">
-        <f aca="false">IF(AND(D56="",E56=""),"",'Start Here'!$B$4+SUM($D$5:D56)-SUM($E$5:E56))</f>
+        <f aca="false">IF(AND(D56="",E56=""),"",'Start Here'!$B$4+SUM($D$5:D56)+SUM($E$5:E56))</f>
         <v/>
       </c>
       <c r="G56" s="5"/>
@@ -2022,7 +2023,7 @@
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
       <c r="F57" s="20" t="str">
-        <f aca="false">IF(AND(D57="",E57=""),"",'Start Here'!$B$4+SUM($D$5:D57)-SUM($E$5:E57))</f>
+        <f aca="false">IF(AND(D57="",E57=""),"",'Start Here'!$B$4+SUM($D$5:D57)+SUM($E$5:E57))</f>
         <v/>
       </c>
       <c r="G57" s="5"/>
@@ -2034,7 +2035,7 @@
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
       <c r="F58" s="20" t="str">
-        <f aca="false">IF(AND(D58="",E58=""),"",'Start Here'!$B$4+SUM($D$5:D58)-SUM($E$5:E58))</f>
+        <f aca="false">IF(AND(D58="",E58=""),"",'Start Here'!$B$4+SUM($D$5:D58)+SUM($E$5:E58))</f>
         <v/>
       </c>
       <c r="G58" s="5"/>
@@ -2046,7 +2047,7 @@
       <c r="D59" s="4"/>
       <c r="E59" s="4"/>
       <c r="F59" s="20" t="str">
-        <f aca="false">IF(AND(D59="",E59=""),"",'Start Here'!$B$4+SUM($D$5:D59)-SUM($E$5:E59))</f>
+        <f aca="false">IF(AND(D59="",E59=""),"",'Start Here'!$B$4+SUM($D$5:D59)+SUM($E$5:E59))</f>
         <v/>
       </c>
       <c r="G59" s="5"/>
@@ -2058,7 +2059,7 @@
       <c r="D60" s="4"/>
       <c r="E60" s="4"/>
       <c r="F60" s="20" t="str">
-        <f aca="false">IF(AND(D60="",E60=""),"",'Start Here'!$B$4+SUM($D$5:D60)-SUM($E$5:E60))</f>
+        <f aca="false">IF(AND(D60="",E60=""),"",'Start Here'!$B$4+SUM($D$5:D60)+SUM($E$5:E60))</f>
         <v/>
       </c>
       <c r="G60" s="5"/>
@@ -2070,7 +2071,7 @@
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
       <c r="F61" s="20" t="str">
-        <f aca="false">IF(AND(D61="",E61=""),"",'Start Here'!$B$4+SUM($D$5:D61)-SUM($E$5:E61))</f>
+        <f aca="false">IF(AND(D61="",E61=""),"",'Start Here'!$B$4+SUM($D$5:D61)+SUM($E$5:E61))</f>
         <v/>
       </c>
       <c r="G61" s="5"/>
@@ -2082,7 +2083,7 @@
       <c r="D62" s="4"/>
       <c r="E62" s="4"/>
       <c r="F62" s="20" t="str">
-        <f aca="false">IF(AND(D62="",E62=""),"",'Start Here'!$B$4+SUM($D$5:D62)-SUM($E$5:E62))</f>
+        <f aca="false">IF(AND(D62="",E62=""),"",'Start Here'!$B$4+SUM($D$5:D62)+SUM($E$5:E62))</f>
         <v/>
       </c>
       <c r="G62" s="5"/>
@@ -2094,7 +2095,7 @@
       <c r="D63" s="4"/>
       <c r="E63" s="4"/>
       <c r="F63" s="20" t="str">
-        <f aca="false">IF(AND(D63="",E63=""),"",'Start Here'!$B$4+SUM($D$5:D63)-SUM($E$5:E63))</f>
+        <f aca="false">IF(AND(D63="",E63=""),"",'Start Here'!$B$4+SUM($D$5:D63)+SUM($E$5:E63))</f>
         <v/>
       </c>
       <c r="G63" s="5"/>
@@ -2106,7 +2107,7 @@
       <c r="D64" s="4"/>
       <c r="E64" s="4"/>
       <c r="F64" s="20" t="str">
-        <f aca="false">IF(AND(D64="",E64=""),"",'Start Here'!$B$4+SUM($D$5:D64)-SUM($E$5:E64))</f>
+        <f aca="false">IF(AND(D64="",E64=""),"",'Start Here'!$B$4+SUM($D$5:D64)+SUM($E$5:E64))</f>
         <v/>
       </c>
       <c r="G64" s="5"/>
@@ -2118,7 +2119,7 @@
       <c r="D65" s="4"/>
       <c r="E65" s="4"/>
       <c r="F65" s="20" t="str">
-        <f aca="false">IF(AND(D65="",E65=""),"",'Start Here'!$B$4+SUM($D$5:D65)-SUM($E$5:E65))</f>
+        <f aca="false">IF(AND(D65="",E65=""),"",'Start Here'!$B$4+SUM($D$5:D65)+SUM($E$5:E65))</f>
         <v/>
       </c>
       <c r="G65" s="5"/>
@@ -2130,7 +2131,7 @@
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
       <c r="F66" s="20" t="str">
-        <f aca="false">IF(AND(D66="",E66=""),"",'Start Here'!$B$4+SUM($D$5:D66)-SUM($E$5:E66))</f>
+        <f aca="false">IF(AND(D66="",E66=""),"",'Start Here'!$B$4+SUM($D$5:D66)+SUM($E$5:E66))</f>
         <v/>
       </c>
       <c r="G66" s="5"/>
@@ -2142,7 +2143,7 @@
       <c r="D67" s="4"/>
       <c r="E67" s="4"/>
       <c r="F67" s="20" t="str">
-        <f aca="false">IF(AND(D67="",E67=""),"",'Start Here'!$B$4+SUM($D$5:D67)-SUM($E$5:E67))</f>
+        <f aca="false">IF(AND(D67="",E67=""),"",'Start Here'!$B$4+SUM($D$5:D67)+SUM($E$5:E67))</f>
         <v/>
       </c>
       <c r="G67" s="5"/>
@@ -2154,7 +2155,7 @@
       <c r="D68" s="4"/>
       <c r="E68" s="4"/>
       <c r="F68" s="20" t="str">
-        <f aca="false">IF(AND(D68="",E68=""),"",'Start Here'!$B$4+SUM($D$5:D68)-SUM($E$5:E68))</f>
+        <f aca="false">IF(AND(D68="",E68=""),"",'Start Here'!$B$4+SUM($D$5:D68)+SUM($E$5:E68))</f>
         <v/>
       </c>
       <c r="G68" s="5"/>
@@ -2166,7 +2167,7 @@
       <c r="D69" s="4"/>
       <c r="E69" s="4"/>
       <c r="F69" s="20" t="str">
-        <f aca="false">IF(AND(D69="",E69=""),"",'Start Here'!$B$4+SUM($D$5:D69)-SUM($E$5:E69))</f>
+        <f aca="false">IF(AND(D69="",E69=""),"",'Start Here'!$B$4+SUM($D$5:D69)+SUM($E$5:E69))</f>
         <v/>
       </c>
       <c r="G69" s="5"/>
@@ -2178,7 +2179,7 @@
       <c r="D70" s="4"/>
       <c r="E70" s="4"/>
       <c r="F70" s="20" t="str">
-        <f aca="false">IF(AND(D70="",E70=""),"",'Start Here'!$B$4+SUM($D$5:D70)-SUM($E$5:E70))</f>
+        <f aca="false">IF(AND(D70="",E70=""),"",'Start Here'!$B$4+SUM($D$5:D70)+SUM($E$5:E70))</f>
         <v/>
       </c>
       <c r="G70" s="5"/>
@@ -2190,7 +2191,7 @@
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
       <c r="F71" s="20" t="str">
-        <f aca="false">IF(AND(D71="",E71=""),"",'Start Here'!$B$4+SUM($D$5:D71)-SUM($E$5:E71))</f>
+        <f aca="false">IF(AND(D71="",E71=""),"",'Start Here'!$B$4+SUM($D$5:D71)+SUM($E$5:E71))</f>
         <v/>
       </c>
       <c r="G71" s="5"/>
@@ -2202,7 +2203,7 @@
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
       <c r="F72" s="20" t="str">
-        <f aca="false">IF(AND(D72="",E72=""),"",'Start Here'!$B$4+SUM($D$5:D72)-SUM($E$5:E72))</f>
+        <f aca="false">IF(AND(D72="",E72=""),"",'Start Here'!$B$4+SUM($D$5:D72)+SUM($E$5:E72))</f>
         <v/>
       </c>
       <c r="G72" s="5"/>
@@ -2214,7 +2215,7 @@
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>
       <c r="F73" s="20" t="str">
-        <f aca="false">IF(AND(D73="",E73=""),"",'Start Here'!$B$4+SUM($D$5:D73)-SUM($E$5:E73))</f>
+        <f aca="false">IF(AND(D73="",E73=""),"",'Start Here'!$B$4+SUM($D$5:D73)+SUM($E$5:E73))</f>
         <v/>
       </c>
       <c r="G73" s="5"/>
@@ -2226,7 +2227,7 @@
       <c r="D74" s="4"/>
       <c r="E74" s="4"/>
       <c r="F74" s="20" t="str">
-        <f aca="false">IF(AND(D74="",E74=""),"",'Start Here'!$B$4+SUM($D$5:D74)-SUM($E$5:E74))</f>
+        <f aca="false">IF(AND(D74="",E74=""),"",'Start Here'!$B$4+SUM($D$5:D74)+SUM($E$5:E74))</f>
         <v/>
       </c>
       <c r="G74" s="5"/>
@@ -2238,7 +2239,7 @@
       <c r="D75" s="4"/>
       <c r="E75" s="4"/>
       <c r="F75" s="20" t="str">
-        <f aca="false">IF(AND(D75="",E75=""),"",'Start Here'!$B$4+SUM($D$5:D75)-SUM($E$5:E75))</f>
+        <f aca="false">IF(AND(D75="",E75=""),"",'Start Here'!$B$4+SUM($D$5:D75)+SUM($E$5:E75))</f>
         <v/>
       </c>
       <c r="G75" s="5"/>
@@ -2250,7 +2251,7 @@
       <c r="D76" s="4"/>
       <c r="E76" s="4"/>
       <c r="F76" s="20" t="str">
-        <f aca="false">IF(AND(D76="",E76=""),"",'Start Here'!$B$4+SUM($D$5:D76)-SUM($E$5:E76))</f>
+        <f aca="false">IF(AND(D76="",E76=""),"",'Start Here'!$B$4+SUM($D$5:D76)+SUM($E$5:E76))</f>
         <v/>
       </c>
       <c r="G76" s="5"/>
@@ -2262,7 +2263,7 @@
       <c r="D77" s="4"/>
       <c r="E77" s="4"/>
       <c r="F77" s="20" t="str">
-        <f aca="false">IF(AND(D77="",E77=""),"",'Start Here'!$B$4+SUM($D$5:D77)-SUM($E$5:E77))</f>
+        <f aca="false">IF(AND(D77="",E77=""),"",'Start Here'!$B$4+SUM($D$5:D77)+SUM($E$5:E77))</f>
         <v/>
       </c>
       <c r="G77" s="5"/>
@@ -2274,7 +2275,7 @@
       <c r="D78" s="4"/>
       <c r="E78" s="4"/>
       <c r="F78" s="20" t="str">
-        <f aca="false">IF(AND(D78="",E78=""),"",'Start Here'!$B$4+SUM($D$5:D78)-SUM($E$5:E78))</f>
+        <f aca="false">IF(AND(D78="",E78=""),"",'Start Here'!$B$4+SUM($D$5:D78)+SUM($E$5:E78))</f>
         <v/>
       </c>
       <c r="G78" s="5"/>
@@ -2286,7 +2287,7 @@
       <c r="D79" s="4"/>
       <c r="E79" s="4"/>
       <c r="F79" s="20" t="str">
-        <f aca="false">IF(AND(D79="",E79=""),"",'Start Here'!$B$4+SUM($D$5:D79)-SUM($E$5:E79))</f>
+        <f aca="false">IF(AND(D79="",E79=""),"",'Start Here'!$B$4+SUM($D$5:D79)+SUM($E$5:E79))</f>
         <v/>
       </c>
       <c r="G79" s="5"/>
@@ -2298,7 +2299,7 @@
       <c r="D80" s="4"/>
       <c r="E80" s="4"/>
       <c r="F80" s="20" t="str">
-        <f aca="false">IF(AND(D80="",E80=""),"",'Start Here'!$B$4+SUM($D$5:D80)-SUM($E$5:E80))</f>
+        <f aca="false">IF(AND(D80="",E80=""),"",'Start Here'!$B$4+SUM($D$5:D80)+SUM($E$5:E80))</f>
         <v/>
       </c>
       <c r="G80" s="5"/>
@@ -2310,7 +2311,7 @@
       <c r="D81" s="4"/>
       <c r="E81" s="4"/>
       <c r="F81" s="20" t="str">
-        <f aca="false">IF(AND(D81="",E81=""),"",'Start Here'!$B$4+SUM($D$5:D81)-SUM($E$5:E81))</f>
+        <f aca="false">IF(AND(D81="",E81=""),"",'Start Here'!$B$4+SUM($D$5:D81)+SUM($E$5:E81))</f>
         <v/>
       </c>
       <c r="G81" s="5"/>
@@ -2322,7 +2323,7 @@
       <c r="D82" s="4"/>
       <c r="E82" s="4"/>
       <c r="F82" s="20" t="str">
-        <f aca="false">IF(AND(D82="",E82=""),"",'Start Here'!$B$4+SUM($D$5:D82)-SUM($E$5:E82))</f>
+        <f aca="false">IF(AND(D82="",E82=""),"",'Start Here'!$B$4+SUM($D$5:D82)+SUM($E$5:E82))</f>
         <v/>
       </c>
       <c r="G82" s="5"/>
@@ -2334,7 +2335,7 @@
       <c r="D83" s="4"/>
       <c r="E83" s="4"/>
       <c r="F83" s="20" t="str">
-        <f aca="false">IF(AND(D83="",E83=""),"",'Start Here'!$B$4+SUM($D$5:D83)-SUM($E$5:E83))</f>
+        <f aca="false">IF(AND(D83="",E83=""),"",'Start Here'!$B$4+SUM($D$5:D83)+SUM($E$5:E83))</f>
         <v/>
       </c>
       <c r="G83" s="5"/>
@@ -2346,7 +2347,7 @@
       <c r="D84" s="4"/>
       <c r="E84" s="4"/>
       <c r="F84" s="20" t="str">
-        <f aca="false">IF(AND(D84="",E84=""),"",'Start Here'!$B$4+SUM($D$5:D84)-SUM($E$5:E84))</f>
+        <f aca="false">IF(AND(D84="",E84=""),"",'Start Here'!$B$4+SUM($D$5:D84)+SUM($E$5:E84))</f>
         <v/>
       </c>
       <c r="G84" s="5"/>
@@ -2358,7 +2359,7 @@
       <c r="D85" s="4"/>
       <c r="E85" s="4"/>
       <c r="F85" s="20" t="str">
-        <f aca="false">IF(AND(D85="",E85=""),"",'Start Here'!$B$4+SUM($D$5:D85)-SUM($E$5:E85))</f>
+        <f aca="false">IF(AND(D85="",E85=""),"",'Start Here'!$B$4+SUM($D$5:D85)+SUM($E$5:E85))</f>
         <v/>
       </c>
       <c r="G85" s="5"/>
@@ -2370,7 +2371,7 @@
       <c r="D86" s="4"/>
       <c r="E86" s="4"/>
       <c r="F86" s="20" t="str">
-        <f aca="false">IF(AND(D86="",E86=""),"",'Start Here'!$B$4+SUM($D$5:D86)-SUM($E$5:E86))</f>
+        <f aca="false">IF(AND(D86="",E86=""),"",'Start Here'!$B$4+SUM($D$5:D86)+SUM($E$5:E86))</f>
         <v/>
       </c>
       <c r="G86" s="5"/>
@@ -2382,7 +2383,7 @@
       <c r="D87" s="4"/>
       <c r="E87" s="4"/>
       <c r="F87" s="20" t="str">
-        <f aca="false">IF(AND(D87="",E87=""),"",'Start Here'!$B$4+SUM($D$5:D87)-SUM($E$5:E87))</f>
+        <f aca="false">IF(AND(D87="",E87=""),"",'Start Here'!$B$4+SUM($D$5:D87)+SUM($E$5:E87))</f>
         <v/>
       </c>
       <c r="G87" s="5"/>
@@ -2394,7 +2395,7 @@
       <c r="D88" s="4"/>
       <c r="E88" s="4"/>
       <c r="F88" s="20" t="str">
-        <f aca="false">IF(AND(D88="",E88=""),"",'Start Here'!$B$4+SUM($D$5:D88)-SUM($E$5:E88))</f>
+        <f aca="false">IF(AND(D88="",E88=""),"",'Start Here'!$B$4+SUM($D$5:D88)+SUM($E$5:E88))</f>
         <v/>
       </c>
       <c r="G88" s="5"/>
@@ -2406,7 +2407,7 @@
       <c r="D89" s="4"/>
       <c r="E89" s="4"/>
       <c r="F89" s="20" t="str">
-        <f aca="false">IF(AND(D89="",E89=""),"",'Start Here'!$B$4+SUM($D$5:D89)-SUM($E$5:E89))</f>
+        <f aca="false">IF(AND(D89="",E89=""),"",'Start Here'!$B$4+SUM($D$5:D89)+SUM($E$5:E89))</f>
         <v/>
       </c>
       <c r="G89" s="5"/>
@@ -2418,7 +2419,7 @@
       <c r="D90" s="4"/>
       <c r="E90" s="4"/>
       <c r="F90" s="20" t="str">
-        <f aca="false">IF(AND(D90="",E90=""),"",'Start Here'!$B$4+SUM($D$5:D90)-SUM($E$5:E90))</f>
+        <f aca="false">IF(AND(D90="",E90=""),"",'Start Here'!$B$4+SUM($D$5:D90)+SUM($E$5:E90))</f>
         <v/>
       </c>
       <c r="G90" s="5"/>
@@ -2430,7 +2431,7 @@
       <c r="D91" s="4"/>
       <c r="E91" s="4"/>
       <c r="F91" s="20" t="str">
-        <f aca="false">IF(AND(D91="",E91=""),"",'Start Here'!$B$4+SUM($D$5:D91)-SUM($E$5:E91))</f>
+        <f aca="false">IF(AND(D91="",E91=""),"",'Start Here'!$B$4+SUM($D$5:D91)+SUM($E$5:E91))</f>
         <v/>
       </c>
       <c r="G91" s="5"/>
@@ -2442,7 +2443,7 @@
       <c r="D92" s="4"/>
       <c r="E92" s="4"/>
       <c r="F92" s="20" t="str">
-        <f aca="false">IF(AND(D92="",E92=""),"",'Start Here'!$B$4+SUM($D$5:D92)-SUM($E$5:E92))</f>
+        <f aca="false">IF(AND(D92="",E92=""),"",'Start Here'!$B$4+SUM($D$5:D92)+SUM($E$5:E92))</f>
         <v/>
       </c>
       <c r="G92" s="5"/>
@@ -2454,7 +2455,7 @@
       <c r="D93" s="4"/>
       <c r="E93" s="4"/>
       <c r="F93" s="20" t="str">
-        <f aca="false">IF(AND(D93="",E93=""),"",'Start Here'!$B$4+SUM($D$5:D93)-SUM($E$5:E93))</f>
+        <f aca="false">IF(AND(D93="",E93=""),"",'Start Here'!$B$4+SUM($D$5:D93)+SUM($E$5:E93))</f>
         <v/>
       </c>
       <c r="G93" s="5"/>
@@ -2466,7 +2467,7 @@
       <c r="D94" s="4"/>
       <c r="E94" s="4"/>
       <c r="F94" s="20" t="str">
-        <f aca="false">IF(AND(D94="",E94=""),"",'Start Here'!$B$4+SUM($D$5:D94)-SUM($E$5:E94))</f>
+        <f aca="false">IF(AND(D94="",E94=""),"",'Start Here'!$B$4+SUM($D$5:D94)+SUM($E$5:E94))</f>
         <v/>
       </c>
       <c r="G94" s="5"/>
@@ -2478,7 +2479,7 @@
       <c r="D95" s="4"/>
       <c r="E95" s="4"/>
       <c r="F95" s="20" t="str">
-        <f aca="false">IF(AND(D95="",E95=""),"",'Start Here'!$B$4+SUM($D$5:D95)-SUM($E$5:E95))</f>
+        <f aca="false">IF(AND(D95="",E95=""),"",'Start Here'!$B$4+SUM($D$5:D95)+SUM($E$5:E95))</f>
         <v/>
       </c>
       <c r="G95" s="5"/>
@@ -2490,7 +2491,7 @@
       <c r="D96" s="4"/>
       <c r="E96" s="4"/>
       <c r="F96" s="20" t="str">
-        <f aca="false">IF(AND(D96="",E96=""),"",'Start Here'!$B$4+SUM($D$5:D96)-SUM($E$5:E96))</f>
+        <f aca="false">IF(AND(D96="",E96=""),"",'Start Here'!$B$4+SUM($D$5:D96)+SUM($E$5:E96))</f>
         <v/>
       </c>
       <c r="G96" s="5"/>
@@ -2502,7 +2503,7 @@
       <c r="D97" s="4"/>
       <c r="E97" s="4"/>
       <c r="F97" s="20" t="str">
-        <f aca="false">IF(AND(D97="",E97=""),"",'Start Here'!$B$4+SUM($D$5:D97)-SUM($E$5:E97))</f>
+        <f aca="false">IF(AND(D97="",E97=""),"",'Start Here'!$B$4+SUM($D$5:D97)+SUM($E$5:E97))</f>
         <v/>
       </c>
       <c r="G97" s="5"/>
@@ -2514,7 +2515,7 @@
       <c r="D98" s="4"/>
       <c r="E98" s="4"/>
       <c r="F98" s="20" t="str">
-        <f aca="false">IF(AND(D98="",E98=""),"",'Start Here'!$B$4+SUM($D$5:D98)-SUM($E$5:E98))</f>
+        <f aca="false">IF(AND(D98="",E98=""),"",'Start Here'!$B$4+SUM($D$5:D98)+SUM($E$5:E98))</f>
         <v/>
       </c>
       <c r="G98" s="5"/>
@@ -2526,7 +2527,7 @@
       <c r="D99" s="4"/>
       <c r="E99" s="4"/>
       <c r="F99" s="20" t="str">
-        <f aca="false">IF(AND(D99="",E99=""),"",'Start Here'!$B$4+SUM($D$5:D99)-SUM($E$5:E99))</f>
+        <f aca="false">IF(AND(D99="",E99=""),"",'Start Here'!$B$4+SUM($D$5:D99)+SUM($E$5:E99))</f>
         <v/>
       </c>
       <c r="G99" s="5"/>
@@ -2538,7 +2539,7 @@
       <c r="D100" s="4"/>
       <c r="E100" s="4"/>
       <c r="F100" s="20" t="str">
-        <f aca="false">IF(AND(D100="",E100=""),"",'Start Here'!$B$4+SUM($D$5:D100)-SUM($E$5:E100))</f>
+        <f aca="false">IF(AND(D100="",E100=""),"",'Start Here'!$B$4+SUM($D$5:D100)+SUM($E$5:E100))</f>
         <v/>
       </c>
       <c r="G100" s="5"/>
@@ -2550,7 +2551,7 @@
       <c r="D101" s="4"/>
       <c r="E101" s="4"/>
       <c r="F101" s="20" t="str">
-        <f aca="false">IF(AND(D101="",E101=""),"",'Start Here'!$B$4+SUM($D$5:D101)-SUM($E$5:E101))</f>
+        <f aca="false">IF(AND(D101="",E101=""),"",'Start Here'!$B$4+SUM($D$5:D101)+SUM($E$5:E101))</f>
         <v/>
       </c>
       <c r="G101" s="5"/>
@@ -2562,7 +2563,7 @@
       <c r="D102" s="4"/>
       <c r="E102" s="4"/>
       <c r="F102" s="20" t="str">
-        <f aca="false">IF(AND(D102="",E102=""),"",'Start Here'!$B$4+SUM($D$5:D102)-SUM($E$5:E102))</f>
+        <f aca="false">IF(AND(D102="",E102=""),"",'Start Here'!$B$4+SUM($D$5:D102)+SUM($E$5:E102))</f>
         <v/>
       </c>
       <c r="G102" s="5"/>
@@ -2574,7 +2575,7 @@
       <c r="D103" s="4"/>
       <c r="E103" s="4"/>
       <c r="F103" s="20" t="str">
-        <f aca="false">IF(AND(D103="",E103=""),"",'Start Here'!$B$4+SUM($D$5:D103)-SUM($E$5:E103))</f>
+        <f aca="false">IF(AND(D103="",E103=""),"",'Start Here'!$B$4+SUM($D$5:D103)+SUM($E$5:E103))</f>
         <v/>
       </c>
       <c r="G103" s="5"/>
@@ -2586,7 +2587,7 @@
       <c r="D104" s="4"/>
       <c r="E104" s="4"/>
       <c r="F104" s="20" t="str">
-        <f aca="false">IF(AND(D104="",E104=""),"",'Start Here'!$B$4+SUM($D$5:D104)-SUM($E$5:E104))</f>
+        <f aca="false">IF(AND(D104="",E104=""),"",'Start Here'!$B$4+SUM($D$5:D104)+SUM($E$5:E104))</f>
         <v/>
       </c>
       <c r="G104" s="5"/>
@@ -2598,7 +2599,7 @@
       <c r="D105" s="4"/>
       <c r="E105" s="4"/>
       <c r="F105" s="20" t="str">
-        <f aca="false">IF(AND(D105="",E105=""),"",'Start Here'!$B$4+SUM($D$5:D105)-SUM($E$5:E105))</f>
+        <f aca="false">IF(AND(D105="",E105=""),"",'Start Here'!$B$4+SUM($D$5:D105)+SUM($E$5:E105))</f>
         <v/>
       </c>
       <c r="G105" s="5"/>
@@ -2610,7 +2611,7 @@
       <c r="D106" s="4"/>
       <c r="E106" s="4"/>
       <c r="F106" s="20" t="str">
-        <f aca="false">IF(AND(D106="",E106=""),"",'Start Here'!$B$4+SUM($D$5:D106)-SUM($E$5:E106))</f>
+        <f aca="false">IF(AND(D106="",E106=""),"",'Start Here'!$B$4+SUM($D$5:D106)+SUM($E$5:E106))</f>
         <v/>
       </c>
       <c r="G106" s="5"/>
@@ -2622,7 +2623,7 @@
       <c r="D107" s="4"/>
       <c r="E107" s="4"/>
       <c r="F107" s="20" t="str">
-        <f aca="false">IF(AND(D107="",E107=""),"",'Start Here'!$B$4+SUM($D$5:D107)-SUM($E$5:E107))</f>
+        <f aca="false">IF(AND(D107="",E107=""),"",'Start Here'!$B$4+SUM($D$5:D107)+SUM($E$5:E107))</f>
         <v/>
       </c>
       <c r="G107" s="5"/>
@@ -2634,7 +2635,7 @@
       <c r="D108" s="4"/>
       <c r="E108" s="4"/>
       <c r="F108" s="20" t="str">
-        <f aca="false">IF(AND(D108="",E108=""),"",'Start Here'!$B$4+SUM($D$5:D108)-SUM($E$5:E108))</f>
+        <f aca="false">IF(AND(D108="",E108=""),"",'Start Here'!$B$4+SUM($D$5:D108)+SUM($E$5:E108))</f>
         <v/>
       </c>
       <c r="G108" s="5"/>
@@ -2646,7 +2647,7 @@
       <c r="D109" s="4"/>
       <c r="E109" s="4"/>
       <c r="F109" s="20" t="str">
-        <f aca="false">IF(AND(D109="",E109=""),"",'Start Here'!$B$4+SUM($D$5:D109)-SUM($E$5:E109))</f>
+        <f aca="false">IF(AND(D109="",E109=""),"",'Start Here'!$B$4+SUM($D$5:D109)+SUM($E$5:E109))</f>
         <v/>
       </c>
       <c r="G109" s="5"/>
@@ -2658,7 +2659,7 @@
       <c r="D110" s="4"/>
       <c r="E110" s="4"/>
       <c r="F110" s="20" t="str">
-        <f aca="false">IF(AND(D110="",E110=""),"",'Start Here'!$B$4+SUM($D$5:D110)-SUM($E$5:E110))</f>
+        <f aca="false">IF(AND(D110="",E110=""),"",'Start Here'!$B$4+SUM($D$5:D110)+SUM($E$5:E110))</f>
         <v/>
       </c>
       <c r="G110" s="5"/>
@@ -2670,7 +2671,7 @@
       <c r="D111" s="4"/>
       <c r="E111" s="4"/>
       <c r="F111" s="20" t="str">
-        <f aca="false">IF(AND(D111="",E111=""),"",'Start Here'!$B$4+SUM($D$5:D111)-SUM($E$5:E111))</f>
+        <f aca="false">IF(AND(D111="",E111=""),"",'Start Here'!$B$4+SUM($D$5:D111)+SUM($E$5:E111))</f>
         <v/>
       </c>
       <c r="G111" s="5"/>
@@ -2682,7 +2683,7 @@
       <c r="D112" s="4"/>
       <c r="E112" s="4"/>
       <c r="F112" s="20" t="str">
-        <f aca="false">IF(AND(D112="",E112=""),"",'Start Here'!$B$4+SUM($D$5:D112)-SUM($E$5:E112))</f>
+        <f aca="false">IF(AND(D112="",E112=""),"",'Start Here'!$B$4+SUM($D$5:D112)+SUM($E$5:E112))</f>
         <v/>
       </c>
       <c r="G112" s="5"/>
@@ -2694,7 +2695,7 @@
       <c r="D113" s="4"/>
       <c r="E113" s="4"/>
       <c r="F113" s="20" t="str">
-        <f aca="false">IF(AND(D113="",E113=""),"",'Start Here'!$B$4+SUM($D$5:D113)-SUM($E$5:E113))</f>
+        <f aca="false">IF(AND(D113="",E113=""),"",'Start Here'!$B$4+SUM($D$5:D113)+SUM($E$5:E113))</f>
         <v/>
       </c>
       <c r="G113" s="5"/>
@@ -2706,7 +2707,7 @@
       <c r="D114" s="4"/>
       <c r="E114" s="4"/>
       <c r="F114" s="20" t="str">
-        <f aca="false">IF(AND(D114="",E114=""),"",'Start Here'!$B$4+SUM($D$5:D114)-SUM($E$5:E114))</f>
+        <f aca="false">IF(AND(D114="",E114=""),"",'Start Here'!$B$4+SUM($D$5:D114)+SUM($E$5:E114))</f>
         <v/>
       </c>
       <c r="G114" s="5"/>
@@ -2718,7 +2719,7 @@
       <c r="D115" s="4"/>
       <c r="E115" s="4"/>
       <c r="F115" s="20" t="str">
-        <f aca="false">IF(AND(D115="",E115=""),"",'Start Here'!$B$4+SUM($D$5:D115)-SUM($E$5:E115))</f>
+        <f aca="false">IF(AND(D115="",E115=""),"",'Start Here'!$B$4+SUM($D$5:D115)+SUM($E$5:E115))</f>
         <v/>
       </c>
       <c r="G115" s="5"/>
@@ -2730,7 +2731,7 @@
       <c r="D116" s="4"/>
       <c r="E116" s="4"/>
       <c r="F116" s="20" t="str">
-        <f aca="false">IF(AND(D116="",E116=""),"",'Start Here'!$B$4+SUM($D$5:D116)-SUM($E$5:E116))</f>
+        <f aca="false">IF(AND(D116="",E116=""),"",'Start Here'!$B$4+SUM($D$5:D116)+SUM($E$5:E116))</f>
         <v/>
       </c>
       <c r="G116" s="5"/>
@@ -2742,7 +2743,7 @@
       <c r="D117" s="4"/>
       <c r="E117" s="4"/>
       <c r="F117" s="20" t="str">
-        <f aca="false">IF(AND(D117="",E117=""),"",'Start Here'!$B$4+SUM($D$5:D117)-SUM($E$5:E117))</f>
+        <f aca="false">IF(AND(D117="",E117=""),"",'Start Here'!$B$4+SUM($D$5:D117)+SUM($E$5:E117))</f>
         <v/>
       </c>
       <c r="G117" s="5"/>
@@ -2754,7 +2755,7 @@
       <c r="D118" s="4"/>
       <c r="E118" s="4"/>
       <c r="F118" s="20" t="str">
-        <f aca="false">IF(AND(D118="",E118=""),"",'Start Here'!$B$4+SUM($D$5:D118)-SUM($E$5:E118))</f>
+        <f aca="false">IF(AND(D118="",E118=""),"",'Start Here'!$B$4+SUM($D$5:D118)+SUM($E$5:E118))</f>
         <v/>
       </c>
       <c r="G118" s="5"/>
@@ -2766,7 +2767,7 @@
       <c r="D119" s="4"/>
       <c r="E119" s="4"/>
       <c r="F119" s="20" t="str">
-        <f aca="false">IF(AND(D119="",E119=""),"",'Start Here'!$B$4+SUM($D$5:D119)-SUM($E$5:E119))</f>
+        <f aca="false">IF(AND(D119="",E119=""),"",'Start Here'!$B$4+SUM($D$5:D119)+SUM($E$5:E119))</f>
         <v/>
       </c>
       <c r="G119" s="5"/>
@@ -2778,7 +2779,7 @@
       <c r="D120" s="4"/>
       <c r="E120" s="4"/>
       <c r="F120" s="20" t="str">
-        <f aca="false">IF(AND(D120="",E120=""),"",'Start Here'!$B$4+SUM($D$5:D120)-SUM($E$5:E120))</f>
+        <f aca="false">IF(AND(D120="",E120=""),"",'Start Here'!$B$4+SUM($D$5:D120)+SUM($E$5:E120))</f>
         <v/>
       </c>
       <c r="G120" s="5"/>
@@ -2790,7 +2791,7 @@
       <c r="D121" s="4"/>
       <c r="E121" s="4"/>
       <c r="F121" s="20" t="str">
-        <f aca="false">IF(AND(D121="",E121=""),"",'Start Here'!$B$4+SUM($D$5:D121)-SUM($E$5:E121))</f>
+        <f aca="false">IF(AND(D121="",E121=""),"",'Start Here'!$B$4+SUM($D$5:D121)+SUM($E$5:E121))</f>
         <v/>
       </c>
       <c r="G121" s="5"/>
@@ -2802,7 +2803,7 @@
       <c r="D122" s="4"/>
       <c r="E122" s="4"/>
       <c r="F122" s="20" t="str">
-        <f aca="false">IF(AND(D122="",E122=""),"",'Start Here'!$B$4+SUM($D$5:D122)-SUM($E$5:E122))</f>
+        <f aca="false">IF(AND(D122="",E122=""),"",'Start Here'!$B$4+SUM($D$5:D122)+SUM($E$5:E122))</f>
         <v/>
       </c>
       <c r="G122" s="5"/>
@@ -2814,7 +2815,7 @@
       <c r="D123" s="4"/>
       <c r="E123" s="4"/>
       <c r="F123" s="20" t="str">
-        <f aca="false">IF(AND(D123="",E123=""),"",'Start Here'!$B$4+SUM($D$5:D123)-SUM($E$5:E123))</f>
+        <f aca="false">IF(AND(D123="",E123=""),"",'Start Here'!$B$4+SUM($D$5:D123)+SUM($E$5:E123))</f>
         <v/>
       </c>
       <c r="G123" s="5"/>
@@ -2826,7 +2827,7 @@
       <c r="D124" s="4"/>
       <c r="E124" s="4"/>
       <c r="F124" s="20" t="str">
-        <f aca="false">IF(AND(D124="",E124=""),"",'Start Here'!$B$4+SUM($D$5:D124)-SUM($E$5:E124))</f>
+        <f aca="false">IF(AND(D124="",E124=""),"",'Start Here'!$B$4+SUM($D$5:D124)+SUM($E$5:E124))</f>
         <v/>
       </c>
       <c r="G124" s="5"/>
@@ -2838,7 +2839,7 @@
       <c r="D125" s="4"/>
       <c r="E125" s="4"/>
       <c r="F125" s="20" t="str">
-        <f aca="false">IF(AND(D125="",E125=""),"",'Start Here'!$B$4+SUM($D$5:D125)-SUM($E$5:E125))</f>
+        <f aca="false">IF(AND(D125="",E125=""),"",'Start Here'!$B$4+SUM($D$5:D125)+SUM($E$5:E125))</f>
         <v/>
       </c>
       <c r="G125" s="5"/>
@@ -2850,7 +2851,7 @@
       <c r="D126" s="4"/>
       <c r="E126" s="4"/>
       <c r="F126" s="20" t="str">
-        <f aca="false">IF(AND(D126="",E126=""),"",'Start Here'!$B$4+SUM($D$5:D126)-SUM($E$5:E126))</f>
+        <f aca="false">IF(AND(D126="",E126=""),"",'Start Here'!$B$4+SUM($D$5:D126)+SUM($E$5:E126))</f>
         <v/>
       </c>
       <c r="G126" s="5"/>
@@ -2862,7 +2863,7 @@
       <c r="D127" s="4"/>
       <c r="E127" s="4"/>
       <c r="F127" s="20" t="str">
-        <f aca="false">IF(AND(D127="",E127=""),"",'Start Here'!$B$4+SUM($D$5:D127)-SUM($E$5:E127))</f>
+        <f aca="false">IF(AND(D127="",E127=""),"",'Start Here'!$B$4+SUM($D$5:D127)+SUM($E$5:E127))</f>
         <v/>
       </c>
       <c r="G127" s="5"/>
@@ -2874,7 +2875,7 @@
       <c r="D128" s="4"/>
       <c r="E128" s="4"/>
       <c r="F128" s="20" t="str">
-        <f aca="false">IF(AND(D128="",E128=""),"",'Start Here'!$B$4+SUM($D$5:D128)-SUM($E$5:E128))</f>
+        <f aca="false">IF(AND(D128="",E128=""),"",'Start Here'!$B$4+SUM($D$5:D128)+SUM($E$5:E128))</f>
         <v/>
       </c>
       <c r="G128" s="5"/>
@@ -2886,7 +2887,7 @@
       <c r="D129" s="4"/>
       <c r="E129" s="4"/>
       <c r="F129" s="20" t="str">
-        <f aca="false">IF(AND(D129="",E129=""),"",'Start Here'!$B$4+SUM($D$5:D129)-SUM($E$5:E129))</f>
+        <f aca="false">IF(AND(D129="",E129=""),"",'Start Here'!$B$4+SUM($D$5:D129)+SUM($E$5:E129))</f>
         <v/>
       </c>
       <c r="G129" s="5"/>
@@ -2898,7 +2899,7 @@
       <c r="D130" s="4"/>
       <c r="E130" s="4"/>
       <c r="F130" s="20" t="str">
-        <f aca="false">IF(AND(D130="",E130=""),"",'Start Here'!$B$4+SUM($D$5:D130)-SUM($E$5:E130))</f>
+        <f aca="false">IF(AND(D130="",E130=""),"",'Start Here'!$B$4+SUM($D$5:D130)+SUM($E$5:E130))</f>
         <v/>
       </c>
       <c r="G130" s="5"/>
@@ -2910,7 +2911,7 @@
       <c r="D131" s="4"/>
       <c r="E131" s="4"/>
       <c r="F131" s="20" t="str">
-        <f aca="false">IF(AND(D131="",E131=""),"",'Start Here'!$B$4+SUM($D$5:D131)-SUM($E$5:E131))</f>
+        <f aca="false">IF(AND(D131="",E131=""),"",'Start Here'!$B$4+SUM($D$5:D131)+SUM($E$5:E131))</f>
         <v/>
       </c>
       <c r="G131" s="5"/>
@@ -2922,7 +2923,7 @@
       <c r="D132" s="4"/>
       <c r="E132" s="4"/>
       <c r="F132" s="20" t="str">
-        <f aca="false">IF(AND(D132="",E132=""),"",'Start Here'!$B$4+SUM($D$5:D132)-SUM($E$5:E132))</f>
+        <f aca="false">IF(AND(D132="",E132=""),"",'Start Here'!$B$4+SUM($D$5:D132)+SUM($E$5:E132))</f>
         <v/>
       </c>
       <c r="G132" s="5"/>
@@ -2934,7 +2935,7 @@
       <c r="D133" s="4"/>
       <c r="E133" s="4"/>
       <c r="F133" s="20" t="str">
-        <f aca="false">IF(AND(D133="",E133=""),"",'Start Here'!$B$4+SUM($D$5:D133)-SUM($E$5:E133))</f>
+        <f aca="false">IF(AND(D133="",E133=""),"",'Start Here'!$B$4+SUM($D$5:D133)+SUM($E$5:E133))</f>
         <v/>
       </c>
       <c r="G133" s="5"/>
@@ -2946,7 +2947,7 @@
       <c r="D134" s="4"/>
       <c r="E134" s="4"/>
       <c r="F134" s="20" t="str">
-        <f aca="false">IF(AND(D134="",E134=""),"",'Start Here'!$B$4+SUM($D$5:D134)-SUM($E$5:E134))</f>
+        <f aca="false">IF(AND(D134="",E134=""),"",'Start Here'!$B$4+SUM($D$5:D134)+SUM($E$5:E134))</f>
         <v/>
       </c>
       <c r="G134" s="5"/>
@@ -2958,7 +2959,7 @@
       <c r="D135" s="4"/>
       <c r="E135" s="4"/>
       <c r="F135" s="20" t="str">
-        <f aca="false">IF(AND(D135="",E135=""),"",'Start Here'!$B$4+SUM($D$5:D135)-SUM($E$5:E135))</f>
+        <f aca="false">IF(AND(D135="",E135=""),"",'Start Here'!$B$4+SUM($D$5:D135)+SUM($E$5:E135))</f>
         <v/>
       </c>
       <c r="G135" s="5"/>
@@ -2970,7 +2971,7 @@
       <c r="D136" s="4"/>
       <c r="E136" s="4"/>
       <c r="F136" s="20" t="str">
-        <f aca="false">IF(AND(D136="",E136=""),"",'Start Here'!$B$4+SUM($D$5:D136)-SUM($E$5:E136))</f>
+        <f aca="false">IF(AND(D136="",E136=""),"",'Start Here'!$B$4+SUM($D$5:D136)+SUM($E$5:E136))</f>
         <v/>
       </c>
       <c r="G136" s="5"/>
@@ -2982,7 +2983,7 @@
       <c r="D137" s="4"/>
       <c r="E137" s="4"/>
       <c r="F137" s="20" t="str">
-        <f aca="false">IF(AND(D137="",E137=""),"",'Start Here'!$B$4+SUM($D$5:D137)-SUM($E$5:E137))</f>
+        <f aca="false">IF(AND(D137="",E137=""),"",'Start Here'!$B$4+SUM($D$5:D137)+SUM($E$5:E137))</f>
         <v/>
       </c>
       <c r="G137" s="5"/>
@@ -2994,7 +2995,7 @@
       <c r="D138" s="4"/>
       <c r="E138" s="4"/>
       <c r="F138" s="20" t="str">
-        <f aca="false">IF(AND(D138="",E138=""),"",'Start Here'!$B$4+SUM($D$5:D138)-SUM($E$5:E138))</f>
+        <f aca="false">IF(AND(D138="",E138=""),"",'Start Here'!$B$4+SUM($D$5:D138)+SUM($E$5:E138))</f>
         <v/>
       </c>
       <c r="G138" s="5"/>
@@ -3006,7 +3007,7 @@
       <c r="D139" s="4"/>
       <c r="E139" s="4"/>
       <c r="F139" s="20" t="str">
-        <f aca="false">IF(AND(D139="",E139=""),"",'Start Here'!$B$4+SUM($D$5:D139)-SUM($E$5:E139))</f>
+        <f aca="false">IF(AND(D139="",E139=""),"",'Start Here'!$B$4+SUM($D$5:D139)+SUM($E$5:E139))</f>
         <v/>
       </c>
       <c r="G139" s="5"/>
@@ -3018,7 +3019,7 @@
       <c r="D140" s="4"/>
       <c r="E140" s="4"/>
       <c r="F140" s="20" t="str">
-        <f aca="false">IF(AND(D140="",E140=""),"",'Start Here'!$B$4+SUM($D$5:D140)-SUM($E$5:E140))</f>
+        <f aca="false">IF(AND(D140="",E140=""),"",'Start Here'!$B$4+SUM($D$5:D140)+SUM($E$5:E140))</f>
         <v/>
       </c>
       <c r="G140" s="5"/>
@@ -3030,7 +3031,7 @@
       <c r="D141" s="4"/>
       <c r="E141" s="4"/>
       <c r="F141" s="20" t="str">
-        <f aca="false">IF(AND(D141="",E141=""),"",'Start Here'!$B$4+SUM($D$5:D141)-SUM($E$5:E141))</f>
+        <f aca="false">IF(AND(D141="",E141=""),"",'Start Here'!$B$4+SUM($D$5:D141)+SUM($E$5:E141))</f>
         <v/>
       </c>
       <c r="G141" s="5"/>
@@ -3042,7 +3043,7 @@
       <c r="D142" s="4"/>
       <c r="E142" s="4"/>
       <c r="F142" s="20" t="str">
-        <f aca="false">IF(AND(D142="",E142=""),"",'Start Here'!$B$4+SUM($D$5:D142)-SUM($E$5:E142))</f>
+        <f aca="false">IF(AND(D142="",E142=""),"",'Start Here'!$B$4+SUM($D$5:D142)+SUM($E$5:E142))</f>
         <v/>
       </c>
       <c r="G142" s="5"/>
@@ -3054,7 +3055,7 @@
       <c r="D143" s="4"/>
       <c r="E143" s="4"/>
       <c r="F143" s="20" t="str">
-        <f aca="false">IF(AND(D143="",E143=""),"",'Start Here'!$B$4+SUM($D$5:D143)-SUM($E$5:E143))</f>
+        <f aca="false">IF(AND(D143="",E143=""),"",'Start Here'!$B$4+SUM($D$5:D143)+SUM($E$5:E143))</f>
         <v/>
       </c>
       <c r="G143" s="5"/>
@@ -3066,7 +3067,7 @@
       <c r="D144" s="4"/>
       <c r="E144" s="4"/>
       <c r="F144" s="20" t="str">
-        <f aca="false">IF(AND(D144="",E144=""),"",'Start Here'!$B$4+SUM($D$5:D144)-SUM($E$5:E144))</f>
+        <f aca="false">IF(AND(D144="",E144=""),"",'Start Here'!$B$4+SUM($D$5:D144)+SUM($E$5:E144))</f>
         <v/>
       </c>
       <c r="G144" s="5"/>
@@ -3078,7 +3079,7 @@
       <c r="D145" s="4"/>
       <c r="E145" s="4"/>
       <c r="F145" s="20" t="str">
-        <f aca="false">IF(AND(D145="",E145=""),"",'Start Here'!$B$4+SUM($D$5:D145)-SUM($E$5:E145))</f>
+        <f aca="false">IF(AND(D145="",E145=""),"",'Start Here'!$B$4+SUM($D$5:D145)+SUM($E$5:E145))</f>
         <v/>
       </c>
       <c r="G145" s="5"/>
@@ -3090,7 +3091,7 @@
       <c r="D146" s="4"/>
       <c r="E146" s="4"/>
       <c r="F146" s="20" t="str">
-        <f aca="false">IF(AND(D146="",E146=""),"",'Start Here'!$B$4+SUM($D$5:D146)-SUM($E$5:E146))</f>
+        <f aca="false">IF(AND(D146="",E146=""),"",'Start Here'!$B$4+SUM($D$5:D146)+SUM($E$5:E146))</f>
         <v/>
       </c>
       <c r="G146" s="5"/>
@@ -3102,7 +3103,7 @@
       <c r="D147" s="4"/>
       <c r="E147" s="4"/>
       <c r="F147" s="20" t="str">
-        <f aca="false">IF(AND(D147="",E147=""),"",'Start Here'!$B$4+SUM($D$5:D147)-SUM($E$5:E147))</f>
+        <f aca="false">IF(AND(D147="",E147=""),"",'Start Here'!$B$4+SUM($D$5:D147)+SUM($E$5:E147))</f>
         <v/>
       </c>
       <c r="G147" s="5"/>
@@ -3114,7 +3115,7 @@
       <c r="D148" s="4"/>
       <c r="E148" s="4"/>
       <c r="F148" s="20" t="str">
-        <f aca="false">IF(AND(D148="",E148=""),"",'Start Here'!$B$4+SUM($D$5:D148)-SUM($E$5:E148))</f>
+        <f aca="false">IF(AND(D148="",E148=""),"",'Start Here'!$B$4+SUM($D$5:D148)+SUM($E$5:E148))</f>
         <v/>
       </c>
       <c r="G148" s="5"/>
@@ -3126,7 +3127,7 @@
       <c r="D149" s="4"/>
       <c r="E149" s="4"/>
       <c r="F149" s="20" t="str">
-        <f aca="false">IF(AND(D149="",E149=""),"",'Start Here'!$B$4+SUM($D$5:D149)-SUM($E$5:E149))</f>
+        <f aca="false">IF(AND(D149="",E149=""),"",'Start Here'!$B$4+SUM($D$5:D149)+SUM($E$5:E149))</f>
         <v/>
       </c>
       <c r="G149" s="5"/>
@@ -3138,7 +3139,7 @@
       <c r="D150" s="4"/>
       <c r="E150" s="4"/>
       <c r="F150" s="20" t="str">
-        <f aca="false">IF(AND(D150="",E150=""),"",'Start Here'!$B$4+SUM($D$5:D150)-SUM($E$5:E150))</f>
+        <f aca="false">IF(AND(D150="",E150=""),"",'Start Here'!$B$4+SUM($D$5:D150)+SUM($E$5:E150))</f>
         <v/>
       </c>
       <c r="G150" s="5"/>
@@ -3150,7 +3151,7 @@
       <c r="D151" s="4"/>
       <c r="E151" s="4"/>
       <c r="F151" s="20" t="str">
-        <f aca="false">IF(AND(D151="",E151=""),"",'Start Here'!$B$4+SUM($D$5:D151)-SUM($E$5:E151))</f>
+        <f aca="false">IF(AND(D151="",E151=""),"",'Start Here'!$B$4+SUM($D$5:D151)+SUM($E$5:E151))</f>
         <v/>
       </c>
       <c r="G151" s="5"/>
@@ -3162,7 +3163,7 @@
       <c r="D152" s="4"/>
       <c r="E152" s="4"/>
       <c r="F152" s="20" t="str">
-        <f aca="false">IF(AND(D152="",E152=""),"",'Start Here'!$B$4+SUM($D$5:D152)-SUM($E$5:E152))</f>
+        <f aca="false">IF(AND(D152="",E152=""),"",'Start Here'!$B$4+SUM($D$5:D152)+SUM($E$5:E152))</f>
         <v/>
       </c>
       <c r="G152" s="5"/>
@@ -3174,7 +3175,7 @@
       <c r="D153" s="4"/>
       <c r="E153" s="4"/>
       <c r="F153" s="20" t="str">
-        <f aca="false">IF(AND(D153="",E153=""),"",'Start Here'!$B$4+SUM($D$5:D153)-SUM($E$5:E153))</f>
+        <f aca="false">IF(AND(D153="",E153=""),"",'Start Here'!$B$4+SUM($D$5:D153)+SUM($E$5:E153))</f>
         <v/>
       </c>
       <c r="G153" s="5"/>
@@ -3186,7 +3187,7 @@
       <c r="D154" s="4"/>
       <c r="E154" s="4"/>
       <c r="F154" s="20" t="str">
-        <f aca="false">IF(AND(D154="",E154=""),"",'Start Here'!$B$4+SUM($D$5:D154)-SUM($E$5:E154))</f>
+        <f aca="false">IF(AND(D154="",E154=""),"",'Start Here'!$B$4+SUM($D$5:D154)+SUM($E$5:E154))</f>
         <v/>
       </c>
       <c r="G154" s="5"/>
@@ -3198,7 +3199,7 @@
       <c r="D155" s="4"/>
       <c r="E155" s="4"/>
       <c r="F155" s="20" t="str">
-        <f aca="false">IF(AND(D155="",E155=""),"",'Start Here'!$B$4+SUM($D$5:D155)-SUM($E$5:E155))</f>
+        <f aca="false">IF(AND(D155="",E155=""),"",'Start Here'!$B$4+SUM($D$5:D155)+SUM($E$5:E155))</f>
         <v/>
       </c>
       <c r="G155" s="5"/>
@@ -3210,7 +3211,7 @@
       <c r="D156" s="4"/>
       <c r="E156" s="4"/>
       <c r="F156" s="20" t="str">
-        <f aca="false">IF(AND(D156="",E156=""),"",'Start Here'!$B$4+SUM($D$5:D156)-SUM($E$5:E156))</f>
+        <f aca="false">IF(AND(D156="",E156=""),"",'Start Here'!$B$4+SUM($D$5:D156)+SUM($E$5:E156))</f>
         <v/>
       </c>
       <c r="G156" s="5"/>
@@ -3222,7 +3223,7 @@
       <c r="D157" s="4"/>
       <c r="E157" s="4"/>
       <c r="F157" s="20" t="str">
-        <f aca="false">IF(AND(D157="",E157=""),"",'Start Here'!$B$4+SUM($D$5:D157)-SUM($E$5:E157))</f>
+        <f aca="false">IF(AND(D157="",E157=""),"",'Start Here'!$B$4+SUM($D$5:D157)+SUM($E$5:E157))</f>
         <v/>
       </c>
       <c r="G157" s="5"/>
@@ -3234,7 +3235,7 @@
       <c r="D158" s="4"/>
       <c r="E158" s="4"/>
       <c r="F158" s="20" t="str">
-        <f aca="false">IF(AND(D158="",E158=""),"",'Start Here'!$B$4+SUM($D$5:D158)-SUM($E$5:E158))</f>
+        <f aca="false">IF(AND(D158="",E158=""),"",'Start Here'!$B$4+SUM($D$5:D158)+SUM($E$5:E158))</f>
         <v/>
       </c>
       <c r="G158" s="5"/>
@@ -3246,7 +3247,7 @@
       <c r="D159" s="4"/>
       <c r="E159" s="4"/>
       <c r="F159" s="20" t="str">
-        <f aca="false">IF(AND(D159="",E159=""),"",'Start Here'!$B$4+SUM($D$5:D159)-SUM($E$5:E159))</f>
+        <f aca="false">IF(AND(D159="",E159=""),"",'Start Here'!$B$4+SUM($D$5:D159)+SUM($E$5:E159))</f>
         <v/>
       </c>
       <c r="G159" s="5"/>
@@ -3258,7 +3259,7 @@
       <c r="D160" s="4"/>
       <c r="E160" s="4"/>
       <c r="F160" s="20" t="str">
-        <f aca="false">IF(AND(D160="",E160=""),"",'Start Here'!$B$4+SUM($D$5:D160)-SUM($E$5:E160))</f>
+        <f aca="false">IF(AND(D160="",E160=""),"",'Start Here'!$B$4+SUM($D$5:D160)+SUM($E$5:E160))</f>
         <v/>
       </c>
       <c r="G160" s="5"/>
@@ -3270,7 +3271,7 @@
       <c r="D161" s="4"/>
       <c r="E161" s="4"/>
       <c r="F161" s="20" t="str">
-        <f aca="false">IF(AND(D161="",E161=""),"",'Start Here'!$B$4+SUM($D$5:D161)-SUM($E$5:E161))</f>
+        <f aca="false">IF(AND(D161="",E161=""),"",'Start Here'!$B$4+SUM($D$5:D161)+SUM($E$5:E161))</f>
         <v/>
       </c>
       <c r="G161" s="5"/>
@@ -3282,7 +3283,7 @@
       <c r="D162" s="4"/>
       <c r="E162" s="4"/>
       <c r="F162" s="20" t="str">
-        <f aca="false">IF(AND(D162="",E162=""),"",'Start Here'!$B$4+SUM($D$5:D162)-SUM($E$5:E162))</f>
+        <f aca="false">IF(AND(D162="",E162=""),"",'Start Here'!$B$4+SUM($D$5:D162)+SUM($E$5:E162))</f>
         <v/>
       </c>
       <c r="G162" s="5"/>
@@ -3294,7 +3295,7 @@
       <c r="D163" s="4"/>
       <c r="E163" s="4"/>
       <c r="F163" s="20" t="str">
-        <f aca="false">IF(AND(D163="",E163=""),"",'Start Here'!$B$4+SUM($D$5:D163)-SUM($E$5:E163))</f>
+        <f aca="false">IF(AND(D163="",E163=""),"",'Start Here'!$B$4+SUM($D$5:D163)+SUM($E$5:E163))</f>
         <v/>
       </c>
       <c r="G163" s="5"/>
@@ -3306,7 +3307,7 @@
       <c r="D164" s="4"/>
       <c r="E164" s="4"/>
       <c r="F164" s="20" t="str">
-        <f aca="false">IF(AND(D164="",E164=""),"",'Start Here'!$B$4+SUM($D$5:D164)-SUM($E$5:E164))</f>
+        <f aca="false">IF(AND(D164="",E164=""),"",'Start Here'!$B$4+SUM($D$5:D164)+SUM($E$5:E164))</f>
         <v/>
       </c>
       <c r="G164" s="5"/>
@@ -3318,7 +3319,7 @@
       <c r="D165" s="4"/>
       <c r="E165" s="4"/>
       <c r="F165" s="20" t="str">
-        <f aca="false">IF(AND(D165="",E165=""),"",'Start Here'!$B$4+SUM($D$5:D165)-SUM($E$5:E165))</f>
+        <f aca="false">IF(AND(D165="",E165=""),"",'Start Here'!$B$4+SUM($D$5:D165)+SUM($E$5:E165))</f>
         <v/>
       </c>
       <c r="G165" s="5"/>
@@ -3330,7 +3331,7 @@
       <c r="D166" s="4"/>
       <c r="E166" s="4"/>
       <c r="F166" s="20" t="str">
-        <f aca="false">IF(AND(D166="",E166=""),"",'Start Here'!$B$4+SUM($D$5:D166)-SUM($E$5:E166))</f>
+        <f aca="false">IF(AND(D166="",E166=""),"",'Start Here'!$B$4+SUM($D$5:D166)+SUM($E$5:E166))</f>
         <v/>
       </c>
       <c r="G166" s="5"/>
@@ -3342,7 +3343,7 @@
       <c r="D167" s="4"/>
       <c r="E167" s="4"/>
       <c r="F167" s="20" t="str">
-        <f aca="false">IF(AND(D167="",E167=""),"",'Start Here'!$B$4+SUM($D$5:D167)-SUM($E$5:E167))</f>
+        <f aca="false">IF(AND(D167="",E167=""),"",'Start Here'!$B$4+SUM($D$5:D167)+SUM($E$5:E167))</f>
         <v/>
       </c>
       <c r="G167" s="5"/>
@@ -3354,7 +3355,7 @@
       <c r="D168" s="4"/>
       <c r="E168" s="4"/>
       <c r="F168" s="20" t="str">
-        <f aca="false">IF(AND(D168="",E168=""),"",'Start Here'!$B$4+SUM($D$5:D168)-SUM($E$5:E168))</f>
+        <f aca="false">IF(AND(D168="",E168=""),"",'Start Here'!$B$4+SUM($D$5:D168)+SUM($E$5:E168))</f>
         <v/>
       </c>
       <c r="G168" s="5"/>
@@ -3366,7 +3367,7 @@
       <c r="D169" s="4"/>
       <c r="E169" s="4"/>
       <c r="F169" s="20" t="str">
-        <f aca="false">IF(AND(D169="",E169=""),"",'Start Here'!$B$4+SUM($D$5:D169)-SUM($E$5:E169))</f>
+        <f aca="false">IF(AND(D169="",E169=""),"",'Start Here'!$B$4+SUM($D$5:D169)+SUM($E$5:E169))</f>
         <v/>
       </c>
       <c r="G169" s="5"/>
@@ -3378,7 +3379,7 @@
       <c r="D170" s="4"/>
       <c r="E170" s="4"/>
       <c r="F170" s="20" t="str">
-        <f aca="false">IF(AND(D170="",E170=""),"",'Start Here'!$B$4+SUM($D$5:D170)-SUM($E$5:E170))</f>
+        <f aca="false">IF(AND(D170="",E170=""),"",'Start Here'!$B$4+SUM($D$5:D170)+SUM($E$5:E170))</f>
         <v/>
       </c>
       <c r="G170" s="5"/>
@@ -3390,7 +3391,7 @@
       <c r="D171" s="4"/>
       <c r="E171" s="4"/>
       <c r="F171" s="20" t="str">
-        <f aca="false">IF(AND(D171="",E171=""),"",'Start Here'!$B$4+SUM($D$5:D171)-SUM($E$5:E171))</f>
+        <f aca="false">IF(AND(D171="",E171=""),"",'Start Here'!$B$4+SUM($D$5:D171)+SUM($E$5:E171))</f>
         <v/>
       </c>
       <c r="G171" s="5"/>
@@ -3402,7 +3403,7 @@
       <c r="D172" s="4"/>
       <c r="E172" s="4"/>
       <c r="F172" s="20" t="str">
-        <f aca="false">IF(AND(D172="",E172=""),"",'Start Here'!$B$4+SUM($D$5:D172)-SUM($E$5:E172))</f>
+        <f aca="false">IF(AND(D172="",E172=""),"",'Start Here'!$B$4+SUM($D$5:D172)+SUM($E$5:E172))</f>
         <v/>
       </c>
       <c r="G172" s="5"/>
@@ -3414,7 +3415,7 @@
       <c r="D173" s="4"/>
       <c r="E173" s="4"/>
       <c r="F173" s="20" t="str">
-        <f aca="false">IF(AND(D173="",E173=""),"",'Start Here'!$B$4+SUM($D$5:D173)-SUM($E$5:E173))</f>
+        <f aca="false">IF(AND(D173="",E173=""),"",'Start Here'!$B$4+SUM($D$5:D173)+SUM($E$5:E173))</f>
         <v/>
       </c>
       <c r="G173" s="5"/>
@@ -3426,7 +3427,7 @@
       <c r="D174" s="4"/>
       <c r="E174" s="4"/>
       <c r="F174" s="20" t="str">
-        <f aca="false">IF(AND(D174="",E174=""),"",'Start Here'!$B$4+SUM($D$5:D174)-SUM($E$5:E174))</f>
+        <f aca="false">IF(AND(D174="",E174=""),"",'Start Here'!$B$4+SUM($D$5:D174)+SUM($E$5:E174))</f>
         <v/>
       </c>
       <c r="G174" s="5"/>
@@ -3438,7 +3439,7 @@
       <c r="D175" s="4"/>
       <c r="E175" s="4"/>
       <c r="F175" s="20" t="str">
-        <f aca="false">IF(AND(D175="",E175=""),"",'Start Here'!$B$4+SUM($D$5:D175)-SUM($E$5:E175))</f>
+        <f aca="false">IF(AND(D175="",E175=""),"",'Start Here'!$B$4+SUM($D$5:D175)+SUM($E$5:E175))</f>
         <v/>
       </c>
       <c r="G175" s="5"/>
@@ -3450,7 +3451,7 @@
       <c r="D176" s="4"/>
       <c r="E176" s="4"/>
       <c r="F176" s="20" t="str">
-        <f aca="false">IF(AND(D176="",E176=""),"",'Start Here'!$B$4+SUM($D$5:D176)-SUM($E$5:E176))</f>
+        <f aca="false">IF(AND(D176="",E176=""),"",'Start Here'!$B$4+SUM($D$5:D176)+SUM($E$5:E176))</f>
         <v/>
       </c>
       <c r="G176" s="5"/>
@@ -3462,7 +3463,7 @@
       <c r="D177" s="4"/>
       <c r="E177" s="4"/>
       <c r="F177" s="20" t="str">
-        <f aca="false">IF(AND(D177="",E177=""),"",'Start Here'!$B$4+SUM($D$5:D177)-SUM($E$5:E177))</f>
+        <f aca="false">IF(AND(D177="",E177=""),"",'Start Here'!$B$4+SUM($D$5:D177)+SUM($E$5:E177))</f>
         <v/>
       </c>
       <c r="G177" s="5"/>
@@ -3474,7 +3475,7 @@
       <c r="D178" s="4"/>
       <c r="E178" s="4"/>
       <c r="F178" s="20" t="str">
-        <f aca="false">IF(AND(D178="",E178=""),"",'Start Here'!$B$4+SUM($D$5:D178)-SUM($E$5:E178))</f>
+        <f aca="false">IF(AND(D178="",E178=""),"",'Start Here'!$B$4+SUM($D$5:D178)+SUM($E$5:E178))</f>
         <v/>
       </c>
       <c r="G178" s="5"/>
@@ -3486,7 +3487,7 @@
       <c r="D179" s="4"/>
       <c r="E179" s="4"/>
       <c r="F179" s="20" t="str">
-        <f aca="false">IF(AND(D179="",E179=""),"",'Start Here'!$B$4+SUM($D$5:D179)-SUM($E$5:E179))</f>
+        <f aca="false">IF(AND(D179="",E179=""),"",'Start Here'!$B$4+SUM($D$5:D179)+SUM($E$5:E179))</f>
         <v/>
       </c>
       <c r="G179" s="5"/>
@@ -3498,7 +3499,7 @@
       <c r="D180" s="4"/>
       <c r="E180" s="4"/>
       <c r="F180" s="20" t="str">
-        <f aca="false">IF(AND(D180="",E180=""),"",'Start Here'!$B$4+SUM($D$5:D180)-SUM($E$5:E180))</f>
+        <f aca="false">IF(AND(D180="",E180=""),"",'Start Here'!$B$4+SUM($D$5:D180)+SUM($E$5:E180))</f>
         <v/>
       </c>
       <c r="G180" s="5"/>
@@ -3510,7 +3511,7 @@
       <c r="D181" s="4"/>
       <c r="E181" s="4"/>
       <c r="F181" s="20" t="str">
-        <f aca="false">IF(AND(D181="",E181=""),"",'Start Here'!$B$4+SUM($D$5:D181)-SUM($E$5:E181))</f>
+        <f aca="false">IF(AND(D181="",E181=""),"",'Start Here'!$B$4+SUM($D$5:D181)+SUM($E$5:E181))</f>
         <v/>
       </c>
       <c r="G181" s="5"/>
@@ -3522,7 +3523,7 @@
       <c r="D182" s="4"/>
       <c r="E182" s="4"/>
       <c r="F182" s="20" t="str">
-        <f aca="false">IF(AND(D182="",E182=""),"",'Start Here'!$B$4+SUM($D$5:D182)-SUM($E$5:E182))</f>
+        <f aca="false">IF(AND(D182="",E182=""),"",'Start Here'!$B$4+SUM($D$5:D182)+SUM($E$5:E182))</f>
         <v/>
       </c>
       <c r="G182" s="5"/>
@@ -3534,7 +3535,7 @@
       <c r="D183" s="4"/>
       <c r="E183" s="4"/>
       <c r="F183" s="20" t="str">
-        <f aca="false">IF(AND(D183="",E183=""),"",'Start Here'!$B$4+SUM($D$5:D183)-SUM($E$5:E183))</f>
+        <f aca="false">IF(AND(D183="",E183=""),"",'Start Here'!$B$4+SUM($D$5:D183)+SUM($E$5:E183))</f>
         <v/>
       </c>
       <c r="G183" s="5"/>
@@ -3546,7 +3547,7 @@
       <c r="D184" s="4"/>
       <c r="E184" s="4"/>
       <c r="F184" s="20" t="str">
-        <f aca="false">IF(AND(D184="",E184=""),"",'Start Here'!$B$4+SUM($D$5:D184)-SUM($E$5:E184))</f>
+        <f aca="false">IF(AND(D184="",E184=""),"",'Start Here'!$B$4+SUM($D$5:D184)+SUM($E$5:E184))</f>
         <v/>
       </c>
       <c r="G184" s="5"/>
@@ -3558,7 +3559,7 @@
       <c r="D185" s="4"/>
       <c r="E185" s="4"/>
       <c r="F185" s="20" t="str">
-        <f aca="false">IF(AND(D185="",E185=""),"",'Start Here'!$B$4+SUM($D$5:D185)-SUM($E$5:E185))</f>
+        <f aca="false">IF(AND(D185="",E185=""),"",'Start Here'!$B$4+SUM($D$5:D185)+SUM($E$5:E185))</f>
         <v/>
       </c>
       <c r="G185" s="5"/>
@@ -3570,7 +3571,7 @@
       <c r="D186" s="4"/>
       <c r="E186" s="4"/>
       <c r="F186" s="20" t="str">
-        <f aca="false">IF(AND(D186="",E186=""),"",'Start Here'!$B$4+SUM($D$5:D186)-SUM($E$5:E186))</f>
+        <f aca="false">IF(AND(D186="",E186=""),"",'Start Here'!$B$4+SUM($D$5:D186)+SUM($E$5:E186))</f>
         <v/>
       </c>
       <c r="G186" s="5"/>
@@ -3582,7 +3583,7 @@
       <c r="D187" s="4"/>
       <c r="E187" s="4"/>
       <c r="F187" s="20" t="str">
-        <f aca="false">IF(AND(D187="",E187=""),"",'Start Here'!$B$4+SUM($D$5:D187)-SUM($E$5:E187))</f>
+        <f aca="false">IF(AND(D187="",E187=""),"",'Start Here'!$B$4+SUM($D$5:D187)+SUM($E$5:E187))</f>
         <v/>
       </c>
       <c r="G187" s="5"/>
@@ -3594,7 +3595,7 @@
       <c r="D188" s="4"/>
       <c r="E188" s="4"/>
       <c r="F188" s="20" t="str">
-        <f aca="false">IF(AND(D188="",E188=""),"",'Start Here'!$B$4+SUM($D$5:D188)-SUM($E$5:E188))</f>
+        <f aca="false">IF(AND(D188="",E188=""),"",'Start Here'!$B$4+SUM($D$5:D188)+SUM($E$5:E188))</f>
         <v/>
       </c>
       <c r="G188" s="5"/>
@@ -3606,7 +3607,7 @@
       <c r="D189" s="4"/>
       <c r="E189" s="4"/>
       <c r="F189" s="20" t="str">
-        <f aca="false">IF(AND(D189="",E189=""),"",'Start Here'!$B$4+SUM($D$5:D189)-SUM($E$5:E189))</f>
+        <f aca="false">IF(AND(D189="",E189=""),"",'Start Here'!$B$4+SUM($D$5:D189)+SUM($E$5:E189))</f>
         <v/>
       </c>
       <c r="G189" s="5"/>
@@ -3618,7 +3619,7 @@
       <c r="D190" s="4"/>
       <c r="E190" s="4"/>
       <c r="F190" s="20" t="str">
-        <f aca="false">IF(AND(D190="",E190=""),"",'Start Here'!$B$4+SUM($D$5:D190)-SUM($E$5:E190))</f>
+        <f aca="false">IF(AND(D190="",E190=""),"",'Start Here'!$B$4+SUM($D$5:D190)+SUM($E$5:E190))</f>
         <v/>
       </c>
       <c r="G190" s="5"/>
@@ -3630,7 +3631,7 @@
       <c r="D191" s="4"/>
       <c r="E191" s="4"/>
       <c r="F191" s="20" t="str">
-        <f aca="false">IF(AND(D191="",E191=""),"",'Start Here'!$B$4+SUM($D$5:D191)-SUM($E$5:E191))</f>
+        <f aca="false">IF(AND(D191="",E191=""),"",'Start Here'!$B$4+SUM($D$5:D191)+SUM($E$5:E191))</f>
         <v/>
       </c>
       <c r="G191" s="5"/>
@@ -3642,7 +3643,7 @@
       <c r="D192" s="4"/>
       <c r="E192" s="4"/>
       <c r="F192" s="20" t="str">
-        <f aca="false">IF(AND(D192="",E192=""),"",'Start Here'!$B$4+SUM($D$5:D192)-SUM($E$5:E192))</f>
+        <f aca="false">IF(AND(D192="",E192=""),"",'Start Here'!$B$4+SUM($D$5:D192)+SUM($E$5:E192))</f>
         <v/>
       </c>
       <c r="G192" s="5"/>
@@ -3654,7 +3655,7 @@
       <c r="D193" s="4"/>
       <c r="E193" s="4"/>
       <c r="F193" s="20" t="str">
-        <f aca="false">IF(AND(D193="",E193=""),"",'Start Here'!$B$4+SUM($D$5:D193)-SUM($E$5:E193))</f>
+        <f aca="false">IF(AND(D193="",E193=""),"",'Start Here'!$B$4+SUM($D$5:D193)+SUM($E$5:E193))</f>
         <v/>
       </c>
       <c r="G193" s="5"/>
@@ -3666,7 +3667,7 @@
       <c r="D194" s="4"/>
       <c r="E194" s="4"/>
       <c r="F194" s="20" t="str">
-        <f aca="false">IF(AND(D194="",E194=""),"",'Start Here'!$B$4+SUM($D$5:D194)-SUM($E$5:E194))</f>
+        <f aca="false">IF(AND(D194="",E194=""),"",'Start Here'!$B$4+SUM($D$5:D194)+SUM($E$5:E194))</f>
         <v/>
       </c>
       <c r="G194" s="5"/>
@@ -3678,7 +3679,7 @@
       <c r="D195" s="4"/>
       <c r="E195" s="4"/>
       <c r="F195" s="20" t="str">
-        <f aca="false">IF(AND(D195="",E195=""),"",'Start Here'!$B$4+SUM($D$5:D195)-SUM($E$5:E195))</f>
+        <f aca="false">IF(AND(D195="",E195=""),"",'Start Here'!$B$4+SUM($D$5:D195)+SUM($E$5:E195))</f>
         <v/>
       </c>
       <c r="G195" s="5"/>
@@ -3690,7 +3691,7 @@
       <c r="D196" s="4"/>
       <c r="E196" s="4"/>
       <c r="F196" s="20" t="str">
-        <f aca="false">IF(AND(D196="",E196=""),"",'Start Here'!$B$4+SUM($D$5:D196)-SUM($E$5:E196))</f>
+        <f aca="false">IF(AND(D196="",E196=""),"",'Start Here'!$B$4+SUM($D$5:D196)+SUM($E$5:E196))</f>
         <v/>
       </c>
       <c r="G196" s="5"/>
@@ -3702,7 +3703,7 @@
       <c r="D197" s="4"/>
       <c r="E197" s="4"/>
       <c r="F197" s="20" t="str">
-        <f aca="false">IF(AND(D197="",E197=""),"",'Start Here'!$B$4+SUM($D$5:D197)-SUM($E$5:E197))</f>
+        <f aca="false">IF(AND(D197="",E197=""),"",'Start Here'!$B$4+SUM($D$5:D197)+SUM($E$5:E197))</f>
         <v/>
       </c>
       <c r="G197" s="5"/>
@@ -3714,7 +3715,7 @@
       <c r="D198" s="4"/>
       <c r="E198" s="4"/>
       <c r="F198" s="20" t="str">
-        <f aca="false">IF(AND(D198="",E198=""),"",'Start Here'!$B$4+SUM($D$5:D198)-SUM($E$5:E198))</f>
+        <f aca="false">IF(AND(D198="",E198=""),"",'Start Here'!$B$4+SUM($D$5:D198)+SUM($E$5:E198))</f>
         <v/>
       </c>
       <c r="G198" s="5"/>
@@ -3726,7 +3727,7 @@
       <c r="D199" s="4"/>
       <c r="E199" s="4"/>
       <c r="F199" s="20" t="str">
-        <f aca="false">IF(AND(D199="",E199=""),"",'Start Here'!$B$4+SUM($D$5:D199)-SUM($E$5:E199))</f>
+        <f aca="false">IF(AND(D199="",E199=""),"",'Start Here'!$B$4+SUM($D$5:D199)+SUM($E$5:E199))</f>
         <v/>
       </c>
       <c r="G199" s="5"/>
@@ -3738,7 +3739,7 @@
       <c r="D200" s="4"/>
       <c r="E200" s="4"/>
       <c r="F200" s="20" t="str">
-        <f aca="false">IF(AND(D200="",E200=""),"",'Start Here'!$B$4+SUM($D$5:D200)-SUM($E$5:E200))</f>
+        <f aca="false">IF(AND(D200="",E200=""),"",'Start Here'!$B$4+SUM($D$5:D200)+SUM($E$5:E200))</f>
         <v/>
       </c>
       <c r="G200" s="5"/>
@@ -3750,7 +3751,7 @@
       <c r="D201" s="4"/>
       <c r="E201" s="4"/>
       <c r="F201" s="20" t="str">
-        <f aca="false">IF(AND(D201="",E201=""),"",'Start Here'!$B$4+SUM($D$5:D201)-SUM($E$5:E201))</f>
+        <f aca="false">IF(AND(D201="",E201=""),"",'Start Here'!$B$4+SUM($D$5:D201)+SUM($E$5:E201))</f>
         <v/>
       </c>
       <c r="G201" s="5"/>
@@ -3762,7 +3763,7 @@
       <c r="D202" s="4"/>
       <c r="E202" s="4"/>
       <c r="F202" s="20" t="str">
-        <f aca="false">IF(AND(D202="",E202=""),"",'Start Here'!$B$4+SUM($D$5:D202)-SUM($E$5:E202))</f>
+        <f aca="false">IF(AND(D202="",E202=""),"",'Start Here'!$B$4+SUM($D$5:D202)+SUM($E$5:E202))</f>
         <v/>
       </c>
       <c r="G202" s="5"/>
@@ -3774,7 +3775,7 @@
       <c r="D203" s="4"/>
       <c r="E203" s="4"/>
       <c r="F203" s="20" t="str">
-        <f aca="false">IF(AND(D203="",E203=""),"",'Start Here'!$B$4+SUM($D$5:D203)-SUM($E$5:E203))</f>
+        <f aca="false">IF(AND(D203="",E203=""),"",'Start Here'!$B$4+SUM($D$5:D203)+SUM($E$5:E203))</f>
         <v/>
       </c>
       <c r="G203" s="5"/>
@@ -3786,7 +3787,7 @@
       <c r="D204" s="4"/>
       <c r="E204" s="4"/>
       <c r="F204" s="20" t="str">
-        <f aca="false">IF(AND(D204="",E204=""),"",'Start Here'!$B$4+SUM($D$5:D204)-SUM($E$5:E204))</f>
+        <f aca="false">IF(AND(D204="",E204=""),"",'Start Here'!$B$4+SUM($D$5:D204)+SUM($E$5:E204))</f>
         <v/>
       </c>
       <c r="G204" s="5"/>
@@ -3798,7 +3799,7 @@
       <c r="D205" s="4"/>
       <c r="E205" s="4"/>
       <c r="F205" s="20" t="str">
-        <f aca="false">IF(AND(D205="",E205=""),"",'Start Here'!$B$4+SUM($D$5:D205)-SUM($E$5:E205))</f>
+        <f aca="false">IF(AND(D205="",E205=""),"",'Start Here'!$B$4+SUM($D$5:D205)+SUM($E$5:E205))</f>
         <v/>
       </c>
       <c r="G205" s="5"/>
@@ -3810,7 +3811,7 @@
       <c r="D206" s="4"/>
       <c r="E206" s="4"/>
       <c r="F206" s="20" t="str">
-        <f aca="false">IF(AND(D206="",E206=""),"",'Start Here'!$B$4+SUM($D$5:D206)-SUM($E$5:E206))</f>
+        <f aca="false">IF(AND(D206="",E206=""),"",'Start Here'!$B$4+SUM($D$5:D206)+SUM($E$5:E206))</f>
         <v/>
       </c>
       <c r="G206" s="5"/>
@@ -3822,7 +3823,7 @@
       <c r="D207" s="4"/>
       <c r="E207" s="4"/>
       <c r="F207" s="20" t="str">
-        <f aca="false">IF(AND(D207="",E207=""),"",'Start Here'!$B$4+SUM($D$5:D207)-SUM($E$5:E207))</f>
+        <f aca="false">IF(AND(D207="",E207=""),"",'Start Here'!$B$4+SUM($D$5:D207)+SUM($E$5:E207))</f>
         <v/>
       </c>
       <c r="G207" s="5"/>
@@ -3834,7 +3835,7 @@
       <c r="D208" s="4"/>
       <c r="E208" s="4"/>
       <c r="F208" s="20" t="str">
-        <f aca="false">IF(AND(D208="",E208=""),"",'Start Here'!$B$4+SUM($D$5:D208)-SUM($E$5:E208))</f>
+        <f aca="false">IF(AND(D208="",E208=""),"",'Start Here'!$B$4+SUM($D$5:D208)+SUM($E$5:E208))</f>
         <v/>
       </c>
       <c r="G208" s="5"/>
@@ -3846,7 +3847,7 @@
       <c r="D209" s="4"/>
       <c r="E209" s="4"/>
       <c r="F209" s="20" t="str">
-        <f aca="false">IF(AND(D209="",E209=""),"",'Start Here'!$B$4+SUM($D$5:D209)-SUM($E$5:E209))</f>
+        <f aca="false">IF(AND(D209="",E209=""),"",'Start Here'!$B$4+SUM($D$5:D209)+SUM($E$5:E209))</f>
         <v/>
       </c>
       <c r="G209" s="5"/>
@@ -3858,7 +3859,7 @@
       <c r="D210" s="4"/>
       <c r="E210" s="4"/>
       <c r="F210" s="20" t="str">
-        <f aca="false">IF(AND(D210="",E210=""),"",'Start Here'!$B$4+SUM($D$5:D210)-SUM($E$5:E210))</f>
+        <f aca="false">IF(AND(D210="",E210=""),"",'Start Here'!$B$4+SUM($D$5:D210)+SUM($E$5:E210))</f>
         <v/>
       </c>
       <c r="G210" s="5"/>
@@ -3870,7 +3871,7 @@
       <c r="D211" s="4"/>
       <c r="E211" s="4"/>
       <c r="F211" s="20" t="str">
-        <f aca="false">IF(AND(D211="",E211=""),"",'Start Here'!$B$4+SUM($D$5:D211)-SUM($E$5:E211))</f>
+        <f aca="false">IF(AND(D211="",E211=""),"",'Start Here'!$B$4+SUM($D$5:D211)+SUM($E$5:E211))</f>
         <v/>
       </c>
       <c r="G211" s="5"/>
@@ -3882,7 +3883,7 @@
       <c r="D212" s="4"/>
       <c r="E212" s="4"/>
       <c r="F212" s="20" t="str">
-        <f aca="false">IF(AND(D212="",E212=""),"",'Start Here'!$B$4+SUM($D$5:D212)-SUM($E$5:E212))</f>
+        <f aca="false">IF(AND(D212="",E212=""),"",'Start Here'!$B$4+SUM($D$5:D212)+SUM($E$5:E212))</f>
         <v/>
       </c>
       <c r="G212" s="5"/>
@@ -3894,7 +3895,7 @@
       <c r="D213" s="4"/>
       <c r="E213" s="4"/>
       <c r="F213" s="20" t="str">
-        <f aca="false">IF(AND(D213="",E213=""),"",'Start Here'!$B$4+SUM($D$5:D213)-SUM($E$5:E213))</f>
+        <f aca="false">IF(AND(D213="",E213=""),"",'Start Here'!$B$4+SUM($D$5:D213)+SUM($E$5:E213))</f>
         <v/>
       </c>
       <c r="G213" s="5"/>
@@ -3906,7 +3907,7 @@
       <c r="D214" s="4"/>
       <c r="E214" s="4"/>
       <c r="F214" s="20" t="str">
-        <f aca="false">IF(AND(D214="",E214=""),"",'Start Here'!$B$4+SUM($D$5:D214)-SUM($E$5:E214))</f>
+        <f aca="false">IF(AND(D214="",E214=""),"",'Start Here'!$B$4+SUM($D$5:D214)+SUM($E$5:E214))</f>
         <v/>
       </c>
       <c r="G214" s="5"/>
@@ -3918,7 +3919,7 @@
       <c r="D215" s="4"/>
       <c r="E215" s="4"/>
       <c r="F215" s="20" t="str">
-        <f aca="false">IF(AND(D215="",E215=""),"",'Start Here'!$B$4+SUM($D$5:D215)-SUM($E$5:E215))</f>
+        <f aca="false">IF(AND(D215="",E215=""),"",'Start Here'!$B$4+SUM($D$5:D215)+SUM($E$5:E215))</f>
         <v/>
       </c>
       <c r="G215" s="5"/>
@@ -3930,7 +3931,7 @@
       <c r="D216" s="4"/>
       <c r="E216" s="4"/>
       <c r="F216" s="20" t="str">
-        <f aca="false">IF(AND(D216="",E216=""),"",'Start Here'!$B$4+SUM($D$5:D216)-SUM($E$5:E216))</f>
+        <f aca="false">IF(AND(D216="",E216=""),"",'Start Here'!$B$4+SUM($D$5:D216)+SUM($E$5:E216))</f>
         <v/>
       </c>
       <c r="G216" s="5"/>
@@ -3942,7 +3943,7 @@
       <c r="D217" s="4"/>
       <c r="E217" s="4"/>
       <c r="F217" s="20" t="str">
-        <f aca="false">IF(AND(D217="",E217=""),"",'Start Here'!$B$4+SUM($D$5:D217)-SUM($E$5:E217))</f>
+        <f aca="false">IF(AND(D217="",E217=""),"",'Start Here'!$B$4+SUM($D$5:D217)+SUM($E$5:E217))</f>
         <v/>
       </c>
       <c r="G217" s="5"/>
@@ -3954,7 +3955,7 @@
       <c r="D218" s="4"/>
       <c r="E218" s="4"/>
       <c r="F218" s="20" t="str">
-        <f aca="false">IF(AND(D218="",E218=""),"",'Start Here'!$B$4+SUM($D$5:D218)-SUM($E$5:E218))</f>
+        <f aca="false">IF(AND(D218="",E218=""),"",'Start Here'!$B$4+SUM($D$5:D218)+SUM($E$5:E218))</f>
         <v/>
       </c>
       <c r="G218" s="5"/>
@@ -3966,7 +3967,7 @@
       <c r="D219" s="4"/>
       <c r="E219" s="4"/>
       <c r="F219" s="20" t="str">
-        <f aca="false">IF(AND(D219="",E219=""),"",'Start Here'!$B$4+SUM($D$5:D219)-SUM($E$5:E219))</f>
+        <f aca="false">IF(AND(D219="",E219=""),"",'Start Here'!$B$4+SUM($D$5:D219)+SUM($E$5:E219))</f>
         <v/>
       </c>
       <c r="G219" s="5"/>
@@ -3978,7 +3979,7 @@
       <c r="D220" s="4"/>
       <c r="E220" s="4"/>
       <c r="F220" s="20" t="str">
-        <f aca="false">IF(AND(D220="",E220=""),"",'Start Here'!$B$4+SUM($D$5:D220)-SUM($E$5:E220))</f>
+        <f aca="false">IF(AND(D220="",E220=""),"",'Start Here'!$B$4+SUM($D$5:D220)+SUM($E$5:E220))</f>
         <v/>
       </c>
       <c r="G220" s="5"/>
@@ -3990,7 +3991,7 @@
       <c r="D221" s="4"/>
       <c r="E221" s="4"/>
       <c r="F221" s="20" t="str">
-        <f aca="false">IF(AND(D221="",E221=""),"",'Start Here'!$B$4+SUM($D$5:D221)-SUM($E$5:E221))</f>
+        <f aca="false">IF(AND(D221="",E221=""),"",'Start Here'!$B$4+SUM($D$5:D221)+SUM($E$5:E221))</f>
         <v/>
       </c>
       <c r="G221" s="5"/>
@@ -4002,7 +4003,7 @@
       <c r="D222" s="4"/>
       <c r="E222" s="4"/>
       <c r="F222" s="20" t="str">
-        <f aca="false">IF(AND(D222="",E222=""),"",'Start Here'!$B$4+SUM($D$5:D222)-SUM($E$5:E222))</f>
+        <f aca="false">IF(AND(D222="",E222=""),"",'Start Here'!$B$4+SUM($D$5:D222)+SUM($E$5:E222))</f>
         <v/>
       </c>
       <c r="G222" s="5"/>
@@ -4014,7 +4015,7 @@
       <c r="D223" s="4"/>
       <c r="E223" s="4"/>
       <c r="F223" s="20" t="str">
-        <f aca="false">IF(AND(D223="",E223=""),"",'Start Here'!$B$4+SUM($D$5:D223)-SUM($E$5:E223))</f>
+        <f aca="false">IF(AND(D223="",E223=""),"",'Start Here'!$B$4+SUM($D$5:D223)+SUM($E$5:E223))</f>
         <v/>
       </c>
       <c r="G223" s="5"/>
@@ -4026,7 +4027,7 @@
       <c r="D224" s="4"/>
       <c r="E224" s="4"/>
       <c r="F224" s="20" t="str">
-        <f aca="false">IF(AND(D224="",E224=""),"",'Start Here'!$B$4+SUM($D$5:D224)-SUM($E$5:E224))</f>
+        <f aca="false">IF(AND(D224="",E224=""),"",'Start Here'!$B$4+SUM($D$5:D224)+SUM($E$5:E224))</f>
         <v/>
       </c>
       <c r="G224" s="5"/>
@@ -4038,7 +4039,7 @@
       <c r="D225" s="4"/>
       <c r="E225" s="4"/>
       <c r="F225" s="20" t="str">
-        <f aca="false">IF(AND(D225="",E225=""),"",'Start Here'!$B$4+SUM($D$5:D225)-SUM($E$5:E225))</f>
+        <f aca="false">IF(AND(D225="",E225=""),"",'Start Here'!$B$4+SUM($D$5:D225)+SUM($E$5:E225))</f>
         <v/>
       </c>
       <c r="G225" s="5"/>
@@ -4050,7 +4051,7 @@
       <c r="D226" s="4"/>
       <c r="E226" s="4"/>
       <c r="F226" s="20" t="str">
-        <f aca="false">IF(AND(D226="",E226=""),"",'Start Here'!$B$4+SUM($D$5:D226)-SUM($E$5:E226))</f>
+        <f aca="false">IF(AND(D226="",E226=""),"",'Start Here'!$B$4+SUM($D$5:D226)+SUM($E$5:E226))</f>
         <v/>
       </c>
       <c r="G226" s="5"/>
@@ -4062,7 +4063,7 @@
       <c r="D227" s="4"/>
       <c r="E227" s="4"/>
       <c r="F227" s="20" t="str">
-        <f aca="false">IF(AND(D227="",E227=""),"",'Start Here'!$B$4+SUM($D$5:D227)-SUM($E$5:E227))</f>
+        <f aca="false">IF(AND(D227="",E227=""),"",'Start Here'!$B$4+SUM($D$5:D227)+SUM($E$5:E227))</f>
         <v/>
       </c>
       <c r="G227" s="5"/>
@@ -4074,7 +4075,7 @@
       <c r="D228" s="4"/>
       <c r="E228" s="4"/>
       <c r="F228" s="20" t="str">
-        <f aca="false">IF(AND(D228="",E228=""),"",'Start Here'!$B$4+SUM($D$5:D228)-SUM($E$5:E228))</f>
+        <f aca="false">IF(AND(D228="",E228=""),"",'Start Here'!$B$4+SUM($D$5:D228)+SUM($E$5:E228))</f>
         <v/>
       </c>
       <c r="G228" s="5"/>
@@ -4086,7 +4087,7 @@
       <c r="D229" s="4"/>
       <c r="E229" s="4"/>
       <c r="F229" s="20" t="str">
-        <f aca="false">IF(AND(D229="",E229=""),"",'Start Here'!$B$4+SUM($D$5:D229)-SUM($E$5:E229))</f>
+        <f aca="false">IF(AND(D229="",E229=""),"",'Start Here'!$B$4+SUM($D$5:D229)+SUM($E$5:E229))</f>
         <v/>
       </c>
       <c r="G229" s="5"/>
@@ -4098,7 +4099,7 @@
       <c r="D230" s="4"/>
       <c r="E230" s="4"/>
       <c r="F230" s="20" t="str">
-        <f aca="false">IF(AND(D230="",E230=""),"",'Start Here'!$B$4+SUM($D$5:D230)-SUM($E$5:E230))</f>
+        <f aca="false">IF(AND(D230="",E230=""),"",'Start Here'!$B$4+SUM($D$5:D230)+SUM($E$5:E230))</f>
         <v/>
       </c>
       <c r="G230" s="5"/>
@@ -4110,7 +4111,7 @@
       <c r="D231" s="4"/>
       <c r="E231" s="4"/>
       <c r="F231" s="20" t="str">
-        <f aca="false">IF(AND(D231="",E231=""),"",'Start Here'!$B$4+SUM($D$5:D231)-SUM($E$5:E231))</f>
+        <f aca="false">IF(AND(D231="",E231=""),"",'Start Here'!$B$4+SUM($D$5:D231)+SUM($E$5:E231))</f>
         <v/>
       </c>
       <c r="G231" s="5"/>
@@ -4122,7 +4123,7 @@
       <c r="D232" s="4"/>
       <c r="E232" s="4"/>
       <c r="F232" s="20" t="str">
-        <f aca="false">IF(AND(D232="",E232=""),"",'Start Here'!$B$4+SUM($D$5:D232)-SUM($E$5:E232))</f>
+        <f aca="false">IF(AND(D232="",E232=""),"",'Start Here'!$B$4+SUM($D$5:D232)+SUM($E$5:E232))</f>
         <v/>
       </c>
       <c r="G232" s="5"/>
@@ -4134,7 +4135,7 @@
       <c r="D233" s="4"/>
       <c r="E233" s="4"/>
       <c r="F233" s="20" t="str">
-        <f aca="false">IF(AND(D233="",E233=""),"",'Start Here'!$B$4+SUM($D$5:D233)-SUM($E$5:E233))</f>
+        <f aca="false">IF(AND(D233="",E233=""),"",'Start Here'!$B$4+SUM($D$5:D233)+SUM($E$5:E233))</f>
         <v/>
       </c>
       <c r="G233" s="5"/>
@@ -4146,7 +4147,7 @@
       <c r="D234" s="4"/>
       <c r="E234" s="4"/>
       <c r="F234" s="20" t="str">
-        <f aca="false">IF(AND(D234="",E234=""),"",'Start Here'!$B$4+SUM($D$5:D234)-SUM($E$5:E234))</f>
+        <f aca="false">IF(AND(D234="",E234=""),"",'Start Here'!$B$4+SUM($D$5:D234)+SUM($E$5:E234))</f>
         <v/>
       </c>
       <c r="G234" s="5"/>
@@ -4158,7 +4159,7 @@
       <c r="D235" s="4"/>
       <c r="E235" s="4"/>
       <c r="F235" s="20" t="str">
-        <f aca="false">IF(AND(D235="",E235=""),"",'Start Here'!$B$4+SUM($D$5:D235)-SUM($E$5:E235))</f>
+        <f aca="false">IF(AND(D235="",E235=""),"",'Start Here'!$B$4+SUM($D$5:D235)+SUM($E$5:E235))</f>
         <v/>
       </c>
       <c r="G235" s="5"/>
@@ -4170,7 +4171,7 @@
       <c r="D236" s="4"/>
       <c r="E236" s="4"/>
       <c r="F236" s="20" t="str">
-        <f aca="false">IF(AND(D236="",E236=""),"",'Start Here'!$B$4+SUM($D$5:D236)-SUM($E$5:E236))</f>
+        <f aca="false">IF(AND(D236="",E236=""),"",'Start Here'!$B$4+SUM($D$5:D236)+SUM($E$5:E236))</f>
         <v/>
       </c>
       <c r="G236" s="5"/>
@@ -4182,7 +4183,7 @@
       <c r="D237" s="4"/>
       <c r="E237" s="4"/>
       <c r="F237" s="20" t="str">
-        <f aca="false">IF(AND(D237="",E237=""),"",'Start Here'!$B$4+SUM($D$5:D237)-SUM($E$5:E237))</f>
+        <f aca="false">IF(AND(D237="",E237=""),"",'Start Here'!$B$4+SUM($D$5:D237)+SUM($E$5:E237))</f>
         <v/>
       </c>
       <c r="G237" s="5"/>
@@ -4194,7 +4195,7 @@
       <c r="D238" s="4"/>
       <c r="E238" s="4"/>
       <c r="F238" s="20" t="str">
-        <f aca="false">IF(AND(D238="",E238=""),"",'Start Here'!$B$4+SUM($D$5:D238)-SUM($E$5:E238))</f>
+        <f aca="false">IF(AND(D238="",E238=""),"",'Start Here'!$B$4+SUM($D$5:D238)+SUM($E$5:E238))</f>
         <v/>
       </c>
       <c r="G238" s="5"/>
@@ -4206,7 +4207,7 @@
       <c r="D239" s="4"/>
       <c r="E239" s="4"/>
       <c r="F239" s="20" t="str">
-        <f aca="false">IF(AND(D239="",E239=""),"",'Start Here'!$B$4+SUM($D$5:D239)-SUM($E$5:E239))</f>
+        <f aca="false">IF(AND(D239="",E239=""),"",'Start Here'!$B$4+SUM($D$5:D239)+SUM($E$5:E239))</f>
         <v/>
       </c>
       <c r="G239" s="5"/>
@@ -4218,7 +4219,7 @@
       <c r="D240" s="4"/>
       <c r="E240" s="4"/>
       <c r="F240" s="20" t="str">
-        <f aca="false">IF(AND(D240="",E240=""),"",'Start Here'!$B$4+SUM($D$5:D240)-SUM($E$5:E240))</f>
+        <f aca="false">IF(AND(D240="",E240=""),"",'Start Here'!$B$4+SUM($D$5:D240)+SUM($E$5:E240))</f>
         <v/>
       </c>
       <c r="G240" s="5"/>
@@ -4230,7 +4231,7 @@
       <c r="D241" s="4"/>
       <c r="E241" s="4"/>
       <c r="F241" s="20" t="str">
-        <f aca="false">IF(AND(D241="",E241=""),"",'Start Here'!$B$4+SUM($D$5:D241)-SUM($E$5:E241))</f>
+        <f aca="false">IF(AND(D241="",E241=""),"",'Start Here'!$B$4+SUM($D$5:D241)+SUM($E$5:E241))</f>
         <v/>
       </c>
       <c r="G241" s="5"/>
@@ -4242,7 +4243,7 @@
       <c r="D242" s="4"/>
       <c r="E242" s="4"/>
       <c r="F242" s="20" t="str">
-        <f aca="false">IF(AND(D242="",E242=""),"",'Start Here'!$B$4+SUM($D$5:D242)-SUM($E$5:E242))</f>
+        <f aca="false">IF(AND(D242="",E242=""),"",'Start Here'!$B$4+SUM($D$5:D242)+SUM($E$5:E242))</f>
         <v/>
       </c>
       <c r="G242" s="5"/>
@@ -4254,7 +4255,7 @@
       <c r="D243" s="4"/>
       <c r="E243" s="4"/>
       <c r="F243" s="20" t="str">
-        <f aca="false">IF(AND(D243="",E243=""),"",'Start Here'!$B$4+SUM($D$5:D243)-SUM($E$5:E243))</f>
+        <f aca="false">IF(AND(D243="",E243=""),"",'Start Here'!$B$4+SUM($D$5:D243)+SUM($E$5:E243))</f>
         <v/>
       </c>
       <c r="G243" s="5"/>
@@ -4266,7 +4267,7 @@
       <c r="D244" s="4"/>
       <c r="E244" s="4"/>
       <c r="F244" s="20" t="str">
-        <f aca="false">IF(AND(D244="",E244=""),"",'Start Here'!$B$4+SUM($D$5:D244)-SUM($E$5:E244))</f>
+        <f aca="false">IF(AND(D244="",E244=""),"",'Start Here'!$B$4+SUM($D$5:D244)+SUM($E$5:E244))</f>
         <v/>
       </c>
       <c r="G244" s="5"/>
@@ -4278,7 +4279,7 @@
       <c r="D245" s="4"/>
       <c r="E245" s="4"/>
       <c r="F245" s="20" t="str">
-        <f aca="false">IF(AND(D245="",E245=""),"",'Start Here'!$B$4+SUM($D$5:D245)-SUM($E$5:E245))</f>
+        <f aca="false">IF(AND(D245="",E245=""),"",'Start Here'!$B$4+SUM($D$5:D245)+SUM($E$5:E245))</f>
         <v/>
       </c>
       <c r="G245" s="5"/>
@@ -4290,7 +4291,7 @@
       <c r="D246" s="4"/>
       <c r="E246" s="4"/>
       <c r="F246" s="20" t="str">
-        <f aca="false">IF(AND(D246="",E246=""),"",'Start Here'!$B$4+SUM($D$5:D246)-SUM($E$5:E246))</f>
+        <f aca="false">IF(AND(D246="",E246=""),"",'Start Here'!$B$4+SUM($D$5:D246)+SUM($E$5:E246))</f>
         <v/>
       </c>
       <c r="G246" s="5"/>
@@ -4302,7 +4303,7 @@
       <c r="D247" s="4"/>
       <c r="E247" s="4"/>
       <c r="F247" s="20" t="str">
-        <f aca="false">IF(AND(D247="",E247=""),"",'Start Here'!$B$4+SUM($D$5:D247)-SUM($E$5:E247))</f>
+        <f aca="false">IF(AND(D247="",E247=""),"",'Start Here'!$B$4+SUM($D$5:D247)+SUM($E$5:E247))</f>
         <v/>
       </c>
       <c r="G247" s="5"/>
@@ -4314,7 +4315,7 @@
       <c r="D248" s="4"/>
       <c r="E248" s="4"/>
       <c r="F248" s="20" t="str">
-        <f aca="false">IF(AND(D248="",E248=""),"",'Start Here'!$B$4+SUM($D$5:D248)-SUM($E$5:E248))</f>
+        <f aca="false">IF(AND(D248="",E248=""),"",'Start Here'!$B$4+SUM($D$5:D248)+SUM($E$5:E248))</f>
         <v/>
       </c>
       <c r="G248" s="5"/>
@@ -4326,7 +4327,7 @@
       <c r="D249" s="4"/>
       <c r="E249" s="4"/>
       <c r="F249" s="20" t="str">
-        <f aca="false">IF(AND(D249="",E249=""),"",'Start Here'!$B$4+SUM($D$5:D249)-SUM($E$5:E249))</f>
+        <f aca="false">IF(AND(D249="",E249=""),"",'Start Here'!$B$4+SUM($D$5:D249)+SUM($E$5:E249))</f>
         <v/>
       </c>
       <c r="G249" s="5"/>
@@ -4338,7 +4339,7 @@
       <c r="D250" s="4"/>
       <c r="E250" s="4"/>
       <c r="F250" s="20" t="str">
-        <f aca="false">IF(AND(D250="",E250=""),"",'Start Here'!$B$4+SUM($D$5:D250)-SUM($E$5:E250))</f>
+        <f aca="false">IF(AND(D250="",E250=""),"",'Start Here'!$B$4+SUM($D$5:D250)+SUM($E$5:E250))</f>
         <v/>
       </c>
       <c r="G250" s="5"/>
@@ -4350,7 +4351,7 @@
       <c r="D251" s="4"/>
       <c r="E251" s="4"/>
       <c r="F251" s="20" t="str">
-        <f aca="false">IF(AND(D251="",E251=""),"",'Start Here'!$B$4+SUM($D$5:D251)-SUM($E$5:E251))</f>
+        <f aca="false">IF(AND(D251="",E251=""),"",'Start Here'!$B$4+SUM($D$5:D251)+SUM($E$5:E251))</f>
         <v/>
       </c>
       <c r="G251" s="5"/>
@@ -4362,7 +4363,7 @@
       <c r="D252" s="4"/>
       <c r="E252" s="4"/>
       <c r="F252" s="20" t="str">
-        <f aca="false">IF(AND(D252="",E252=""),"",'Start Here'!$B$4+SUM($D$5:D252)-SUM($E$5:E252))</f>
+        <f aca="false">IF(AND(D252="",E252=""),"",'Start Here'!$B$4+SUM($D$5:D252)+SUM($E$5:E252))</f>
         <v/>
       </c>
       <c r="G252" s="5"/>
@@ -4374,7 +4375,7 @@
       <c r="D253" s="4"/>
       <c r="E253" s="4"/>
       <c r="F253" s="20" t="str">
-        <f aca="false">IF(AND(D253="",E253=""),"",'Start Here'!$B$4+SUM($D$5:D253)-SUM($E$5:E253))</f>
+        <f aca="false">IF(AND(D253="",E253=""),"",'Start Here'!$B$4+SUM($D$5:D253)+SUM($E$5:E253))</f>
         <v/>
       </c>
       <c r="G253" s="5"/>
@@ -4386,7 +4387,7 @@
       <c r="D254" s="4"/>
       <c r="E254" s="4"/>
       <c r="F254" s="20" t="str">
-        <f aca="false">IF(AND(D254="",E254=""),"",'Start Here'!$B$4+SUM($D$5:D254)-SUM($E$5:E254))</f>
+        <f aca="false">IF(AND(D254="",E254=""),"",'Start Here'!$B$4+SUM($D$5:D254)+SUM($E$5:E254))</f>
         <v/>
       </c>
       <c r="G254" s="5"/>
@@ -4398,7 +4399,7 @@
       <c r="D255" s="4"/>
       <c r="E255" s="4"/>
       <c r="F255" s="20" t="str">
-        <f aca="false">IF(AND(D255="",E255=""),"",'Start Here'!$B$4+SUM($D$5:D255)-SUM($E$5:E255))</f>
+        <f aca="false">IF(AND(D255="",E255=""),"",'Start Here'!$B$4+SUM($D$5:D255)+SUM($E$5:E255))</f>
         <v/>
       </c>
       <c r="G255" s="5"/>
@@ -4410,7 +4411,7 @@
       <c r="D256" s="4"/>
       <c r="E256" s="4"/>
       <c r="F256" s="20" t="str">
-        <f aca="false">IF(AND(D256="",E256=""),"",'Start Here'!$B$4+SUM($D$5:D256)-SUM($E$5:E256))</f>
+        <f aca="false">IF(AND(D256="",E256=""),"",'Start Here'!$B$4+SUM($D$5:D256)+SUM($E$5:E256))</f>
         <v/>
       </c>
       <c r="G256" s="5"/>
@@ -4422,7 +4423,7 @@
       <c r="D257" s="4"/>
       <c r="E257" s="4"/>
       <c r="F257" s="20" t="str">
-        <f aca="false">IF(AND(D257="",E257=""),"",'Start Here'!$B$4+SUM($D$5:D257)-SUM($E$5:E257))</f>
+        <f aca="false">IF(AND(D257="",E257=""),"",'Start Here'!$B$4+SUM($D$5:D257)+SUM($E$5:E257))</f>
         <v/>
       </c>
       <c r="G257" s="5"/>
@@ -4434,7 +4435,7 @@
       <c r="D258" s="4"/>
       <c r="E258" s="4"/>
       <c r="F258" s="20" t="str">
-        <f aca="false">IF(AND(D258="",E258=""),"",'Start Here'!$B$4+SUM($D$5:D258)-SUM($E$5:E258))</f>
+        <f aca="false">IF(AND(D258="",E258=""),"",'Start Here'!$B$4+SUM($D$5:D258)+SUM($E$5:E258))</f>
         <v/>
       </c>
       <c r="G258" s="5"/>
@@ -4446,7 +4447,7 @@
       <c r="D259" s="4"/>
       <c r="E259" s="4"/>
       <c r="F259" s="20" t="str">
-        <f aca="false">IF(AND(D259="",E259=""),"",'Start Here'!$B$4+SUM($D$5:D259)-SUM($E$5:E259))</f>
+        <f aca="false">IF(AND(D259="",E259=""),"",'Start Here'!$B$4+SUM($D$5:D259)+SUM($E$5:E259))</f>
         <v/>
       </c>
       <c r="G259" s="5"/>
@@ -4458,7 +4459,7 @@
       <c r="D260" s="4"/>
       <c r="E260" s="4"/>
       <c r="F260" s="20" t="str">
-        <f aca="false">IF(AND(D260="",E260=""),"",'Start Here'!$B$4+SUM($D$5:D260)-SUM($E$5:E260))</f>
+        <f aca="false">IF(AND(D260="",E260=""),"",'Start Here'!$B$4+SUM($D$5:D260)+SUM($E$5:E260))</f>
         <v/>
       </c>
       <c r="G260" s="5"/>
@@ -4470,7 +4471,7 @@
       <c r="D261" s="4"/>
       <c r="E261" s="4"/>
       <c r="F261" s="20" t="str">
-        <f aca="false">IF(AND(D261="",E261=""),"",'Start Here'!$B$4+SUM($D$5:D261)-SUM($E$5:E261))</f>
+        <f aca="false">IF(AND(D261="",E261=""),"",'Start Here'!$B$4+SUM($D$5:D261)+SUM($E$5:E261))</f>
         <v/>
       </c>
       <c r="G261" s="5"/>
@@ -4482,7 +4483,7 @@
       <c r="D262" s="4"/>
       <c r="E262" s="4"/>
       <c r="F262" s="20" t="str">
-        <f aca="false">IF(AND(D262="",E262=""),"",'Start Here'!$B$4+SUM($D$5:D262)-SUM($E$5:E262))</f>
+        <f aca="false">IF(AND(D262="",E262=""),"",'Start Here'!$B$4+SUM($D$5:D262)+SUM($E$5:E262))</f>
         <v/>
       </c>
       <c r="G262" s="5"/>
@@ -4494,7 +4495,7 @@
       <c r="D263" s="4"/>
       <c r="E263" s="4"/>
       <c r="F263" s="20" t="str">
-        <f aca="false">IF(AND(D263="",E263=""),"",'Start Here'!$B$4+SUM($D$5:D263)-SUM($E$5:E263))</f>
+        <f aca="false">IF(AND(D263="",E263=""),"",'Start Here'!$B$4+SUM($D$5:D263)+SUM($E$5:E263))</f>
         <v/>
       </c>
       <c r="G263" s="5"/>
@@ -4506,7 +4507,7 @@
       <c r="D264" s="4"/>
       <c r="E264" s="4"/>
       <c r="F264" s="20" t="str">
-        <f aca="false">IF(AND(D264="",E264=""),"",'Start Here'!$B$4+SUM($D$5:D264)-SUM($E$5:E264))</f>
+        <f aca="false">IF(AND(D264="",E264=""),"",'Start Here'!$B$4+SUM($D$5:D264)+SUM($E$5:E264))</f>
         <v/>
       </c>
       <c r="G264" s="5"/>
@@ -4518,7 +4519,7 @@
       <c r="D265" s="4"/>
       <c r="E265" s="4"/>
       <c r="F265" s="20" t="str">
-        <f aca="false">IF(AND(D265="",E265=""),"",'Start Here'!$B$4+SUM($D$5:D265)-SUM($E$5:E265))</f>
+        <f aca="false">IF(AND(D265="",E265=""),"",'Start Here'!$B$4+SUM($D$5:D265)+SUM($E$5:E265))</f>
         <v/>
       </c>
       <c r="G265" s="5"/>
@@ -4530,7 +4531,7 @@
       <c r="D266" s="4"/>
       <c r="E266" s="4"/>
       <c r="F266" s="20" t="str">
-        <f aca="false">IF(AND(D266="",E266=""),"",'Start Here'!$B$4+SUM($D$5:D266)-SUM($E$5:E266))</f>
+        <f aca="false">IF(AND(D266="",E266=""),"",'Start Here'!$B$4+SUM($D$5:D266)+SUM($E$5:E266))</f>
         <v/>
       </c>
       <c r="G266" s="5"/>
@@ -4542,7 +4543,7 @@
       <c r="D267" s="4"/>
       <c r="E267" s="4"/>
       <c r="F267" s="20" t="str">
-        <f aca="false">IF(AND(D267="",E267=""),"",'Start Here'!$B$4+SUM($D$5:D267)-SUM($E$5:E267))</f>
+        <f aca="false">IF(AND(D267="",E267=""),"",'Start Here'!$B$4+SUM($D$5:D267)+SUM($E$5:E267))</f>
         <v/>
       </c>
       <c r="G267" s="5"/>
@@ -4554,7 +4555,7 @@
       <c r="D268" s="4"/>
       <c r="E268" s="4"/>
       <c r="F268" s="20" t="str">
-        <f aca="false">IF(AND(D268="",E268=""),"",'Start Here'!$B$4+SUM($D$5:D268)-SUM($E$5:E268))</f>
+        <f aca="false">IF(AND(D268="",E268=""),"",'Start Here'!$B$4+SUM($D$5:D268)+SUM($E$5:E268))</f>
         <v/>
       </c>
       <c r="G268" s="5"/>
@@ -4566,7 +4567,7 @@
       <c r="D269" s="4"/>
       <c r="E269" s="4"/>
       <c r="F269" s="20" t="str">
-        <f aca="false">IF(AND(D269="",E269=""),"",'Start Here'!$B$4+SUM($D$5:D269)-SUM($E$5:E269))</f>
+        <f aca="false">IF(AND(D269="",E269=""),"",'Start Here'!$B$4+SUM($D$5:D269)+SUM($E$5:E269))</f>
         <v/>
       </c>
       <c r="G269" s="5"/>
@@ -4578,7 +4579,7 @@
       <c r="D270" s="4"/>
       <c r="E270" s="4"/>
       <c r="F270" s="20" t="str">
-        <f aca="false">IF(AND(D270="",E270=""),"",'Start Here'!$B$4+SUM($D$5:D270)-SUM($E$5:E270))</f>
+        <f aca="false">IF(AND(D270="",E270=""),"",'Start Here'!$B$4+SUM($D$5:D270)+SUM($E$5:E270))</f>
         <v/>
       </c>
       <c r="G270" s="5"/>
@@ -4590,7 +4591,7 @@
       <c r="D271" s="4"/>
       <c r="E271" s="4"/>
       <c r="F271" s="20" t="str">
-        <f aca="false">IF(AND(D271="",E271=""),"",'Start Here'!$B$4+SUM($D$5:D271)-SUM($E$5:E271))</f>
+        <f aca="false">IF(AND(D271="",E271=""),"",'Start Here'!$B$4+SUM($D$5:D271)+SUM($E$5:E271))</f>
         <v/>
       </c>
       <c r="G271" s="5"/>
@@ -4602,7 +4603,7 @@
       <c r="D272" s="4"/>
       <c r="E272" s="4"/>
       <c r="F272" s="20" t="str">
-        <f aca="false">IF(AND(D272="",E272=""),"",'Start Here'!$B$4+SUM($D$5:D272)-SUM($E$5:E272))</f>
+        <f aca="false">IF(AND(D272="",E272=""),"",'Start Here'!$B$4+SUM($D$5:D272)+SUM($E$5:E272))</f>
         <v/>
       </c>
       <c r="G272" s="5"/>
@@ -4614,7 +4615,7 @@
       <c r="D273" s="4"/>
       <c r="E273" s="4"/>
       <c r="F273" s="20" t="str">
-        <f aca="false">IF(AND(D273="",E273=""),"",'Start Here'!$B$4+SUM($D$5:D273)-SUM($E$5:E273))</f>
+        <f aca="false">IF(AND(D273="",E273=""),"",'Start Here'!$B$4+SUM($D$5:D273)+SUM($E$5:E273))</f>
         <v/>
       </c>
       <c r="G273" s="5"/>
@@ -4626,7 +4627,7 @@
       <c r="D274" s="4"/>
       <c r="E274" s="4"/>
       <c r="F274" s="20" t="str">
-        <f aca="false">IF(AND(D274="",E274=""),"",'Start Here'!$B$4+SUM($D$5:D274)-SUM($E$5:E274))</f>
+        <f aca="false">IF(AND(D274="",E274=""),"",'Start Here'!$B$4+SUM($D$5:D274)+SUM($E$5:E274))</f>
         <v/>
       </c>
       <c r="G274" s="5"/>
@@ -4638,7 +4639,7 @@
       <c r="D275" s="4"/>
       <c r="E275" s="4"/>
       <c r="F275" s="20" t="str">
-        <f aca="false">IF(AND(D275="",E275=""),"",'Start Here'!$B$4+SUM($D$5:D275)-SUM($E$5:E275))</f>
+        <f aca="false">IF(AND(D275="",E275=""),"",'Start Here'!$B$4+SUM($D$5:D275)+SUM($E$5:E275))</f>
         <v/>
       </c>
       <c r="G275" s="5"/>
@@ -4650,7 +4651,7 @@
       <c r="D276" s="4"/>
       <c r="E276" s="4"/>
       <c r="F276" s="20" t="str">
-        <f aca="false">IF(AND(D276="",E276=""),"",'Start Here'!$B$4+SUM($D$5:D276)-SUM($E$5:E276))</f>
+        <f aca="false">IF(AND(D276="",E276=""),"",'Start Here'!$B$4+SUM($D$5:D276)+SUM($E$5:E276))</f>
         <v/>
       </c>
       <c r="G276" s="5"/>
@@ -4662,7 +4663,7 @@
       <c r="D277" s="4"/>
       <c r="E277" s="4"/>
       <c r="F277" s="20" t="str">
-        <f aca="false">IF(AND(D277="",E277=""),"",'Start Here'!$B$4+SUM($D$5:D277)-SUM($E$5:E277))</f>
+        <f aca="false">IF(AND(D277="",E277=""),"",'Start Here'!$B$4+SUM($D$5:D277)+SUM($E$5:E277))</f>
         <v/>
       </c>
       <c r="G277" s="5"/>
@@ -4674,7 +4675,7 @@
       <c r="D278" s="4"/>
       <c r="E278" s="4"/>
       <c r="F278" s="20" t="str">
-        <f aca="false">IF(AND(D278="",E278=""),"",'Start Here'!$B$4+SUM($D$5:D278)-SUM($E$5:E278))</f>
+        <f aca="false">IF(AND(D278="",E278=""),"",'Start Here'!$B$4+SUM($D$5:D278)+SUM($E$5:E278))</f>
         <v/>
       </c>
       <c r="G278" s="5"/>
@@ -4686,7 +4687,7 @@
       <c r="D279" s="4"/>
       <c r="E279" s="4"/>
       <c r="F279" s="20" t="str">
-        <f aca="false">IF(AND(D279="",E279=""),"",'Start Here'!$B$4+SUM($D$5:D279)-SUM($E$5:E279))</f>
+        <f aca="false">IF(AND(D279="",E279=""),"",'Start Here'!$B$4+SUM($D$5:D279)+SUM($E$5:E279))</f>
         <v/>
       </c>
       <c r="G279" s="5"/>
@@ -4698,7 +4699,7 @@
       <c r="D280" s="4"/>
       <c r="E280" s="4"/>
       <c r="F280" s="20" t="str">
-        <f aca="false">IF(AND(D280="",E280=""),"",'Start Here'!$B$4+SUM($D$5:D280)-SUM($E$5:E280))</f>
+        <f aca="false">IF(AND(D280="",E280=""),"",'Start Here'!$B$4+SUM($D$5:D280)+SUM($E$5:E280))</f>
         <v/>
       </c>
       <c r="G280" s="5"/>
@@ -4710,7 +4711,7 @@
       <c r="D281" s="4"/>
       <c r="E281" s="4"/>
       <c r="F281" s="20" t="str">
-        <f aca="false">IF(AND(D281="",E281=""),"",'Start Here'!$B$4+SUM($D$5:D281)-SUM($E$5:E281))</f>
+        <f aca="false">IF(AND(D281="",E281=""),"",'Start Here'!$B$4+SUM($D$5:D281)+SUM($E$5:E281))</f>
         <v/>
       </c>
       <c r="G281" s="5"/>
@@ -4722,7 +4723,7 @@
       <c r="D282" s="4"/>
       <c r="E282" s="4"/>
       <c r="F282" s="20" t="str">
-        <f aca="false">IF(AND(D282="",E282=""),"",'Start Here'!$B$4+SUM($D$5:D282)-SUM($E$5:E282))</f>
+        <f aca="false">IF(AND(D282="",E282=""),"",'Start Here'!$B$4+SUM($D$5:D282)+SUM($E$5:E282))</f>
         <v/>
       </c>
       <c r="G282" s="5"/>
@@ -4734,7 +4735,7 @@
       <c r="D283" s="4"/>
       <c r="E283" s="4"/>
       <c r="F283" s="20" t="str">
-        <f aca="false">IF(AND(D283="",E283=""),"",'Start Here'!$B$4+SUM($D$5:D283)-SUM($E$5:E283))</f>
+        <f aca="false">IF(AND(D283="",E283=""),"",'Start Here'!$B$4+SUM($D$5:D283)+SUM($E$5:E283))</f>
         <v/>
       </c>
       <c r="G283" s="5"/>
@@ -4746,7 +4747,7 @@
       <c r="D284" s="4"/>
       <c r="E284" s="4"/>
       <c r="F284" s="20" t="str">
-        <f aca="false">IF(AND(D284="",E284=""),"",'Start Here'!$B$4+SUM($D$5:D284)-SUM($E$5:E284))</f>
+        <f aca="false">IF(AND(D284="",E284=""),"",'Start Here'!$B$4+SUM($D$5:D284)+SUM($E$5:E284))</f>
         <v/>
       </c>
       <c r="G284" s="5"/>
@@ -4758,7 +4759,7 @@
       <c r="D285" s="4"/>
       <c r="E285" s="4"/>
       <c r="F285" s="20" t="str">
-        <f aca="false">IF(AND(D285="",E285=""),"",'Start Here'!$B$4+SUM($D$5:D285)-SUM($E$5:E285))</f>
+        <f aca="false">IF(AND(D285="",E285=""),"",'Start Here'!$B$4+SUM($D$5:D285)+SUM($E$5:E285))</f>
         <v/>
       </c>
       <c r="G285" s="5"/>
@@ -4770,7 +4771,7 @@
       <c r="D286" s="4"/>
       <c r="E286" s="4"/>
       <c r="F286" s="20" t="str">
-        <f aca="false">IF(AND(D286="",E286=""),"",'Start Here'!$B$4+SUM($D$5:D286)-SUM($E$5:E286))</f>
+        <f aca="false">IF(AND(D286="",E286=""),"",'Start Here'!$B$4+SUM($D$5:D286)+SUM($E$5:E286))</f>
         <v/>
       </c>
       <c r="G286" s="5"/>
@@ -4782,7 +4783,7 @@
       <c r="D287" s="4"/>
       <c r="E287" s="4"/>
       <c r="F287" s="20" t="str">
-        <f aca="false">IF(AND(D287="",E287=""),"",'Start Here'!$B$4+SUM($D$5:D287)-SUM($E$5:E287))</f>
+        <f aca="false">IF(AND(D287="",E287=""),"",'Start Here'!$B$4+SUM($D$5:D287)+SUM($E$5:E287))</f>
         <v/>
       </c>
       <c r="G287" s="5"/>
@@ -4794,7 +4795,7 @@
       <c r="D288" s="4"/>
       <c r="E288" s="4"/>
       <c r="F288" s="20" t="str">
-        <f aca="false">IF(AND(D288="",E288=""),"",'Start Here'!$B$4+SUM($D$5:D288)-SUM($E$5:E288))</f>
+        <f aca="false">IF(AND(D288="",E288=""),"",'Start Here'!$B$4+SUM($D$5:D288)+SUM($E$5:E288))</f>
         <v/>
       </c>
       <c r="G288" s="5"/>
@@ -4806,7 +4807,7 @@
       <c r="D289" s="4"/>
       <c r="E289" s="4"/>
       <c r="F289" s="20" t="str">
-        <f aca="false">IF(AND(D289="",E289=""),"",'Start Here'!$B$4+SUM($D$5:D289)-SUM($E$5:E289))</f>
+        <f aca="false">IF(AND(D289="",E289=""),"",'Start Here'!$B$4+SUM($D$5:D289)+SUM($E$5:E289))</f>
         <v/>
       </c>
       <c r="G289" s="5"/>
@@ -4818,7 +4819,7 @@
       <c r="D290" s="4"/>
       <c r="E290" s="4"/>
       <c r="F290" s="20" t="str">
-        <f aca="false">IF(AND(D290="",E290=""),"",'Start Here'!$B$4+SUM($D$5:D290)-SUM($E$5:E290))</f>
+        <f aca="false">IF(AND(D290="",E290=""),"",'Start Here'!$B$4+SUM($D$5:D290)+SUM($E$5:E290))</f>
         <v/>
       </c>
       <c r="G290" s="5"/>
@@ -4830,7 +4831,7 @@
       <c r="D291" s="4"/>
       <c r="E291" s="4"/>
       <c r="F291" s="20" t="str">
-        <f aca="false">IF(AND(D291="",E291=""),"",'Start Here'!$B$4+SUM($D$5:D291)-SUM($E$5:E291))</f>
+        <f aca="false">IF(AND(D291="",E291=""),"",'Start Here'!$B$4+SUM($D$5:D291)+SUM($E$5:E291))</f>
         <v/>
       </c>
       <c r="G291" s="5"/>
@@ -4842,7 +4843,7 @@
       <c r="D292" s="4"/>
       <c r="E292" s="4"/>
       <c r="F292" s="20" t="str">
-        <f aca="false">IF(AND(D292="",E292=""),"",'Start Here'!$B$4+SUM($D$5:D292)-SUM($E$5:E292))</f>
+        <f aca="false">IF(AND(D292="",E292=""),"",'Start Here'!$B$4+SUM($D$5:D292)+SUM($E$5:E292))</f>
         <v/>
       </c>
       <c r="G292" s="5"/>
@@ -4854,7 +4855,7 @@
       <c r="D293" s="4"/>
       <c r="E293" s="4"/>
       <c r="F293" s="20" t="str">
-        <f aca="false">IF(AND(D293="",E293=""),"",'Start Here'!$B$4+SUM($D$5:D293)-SUM($E$5:E293))</f>
+        <f aca="false">IF(AND(D293="",E293=""),"",'Start Here'!$B$4+SUM($D$5:D293)+SUM($E$5:E293))</f>
         <v/>
       </c>
       <c r="G293" s="5"/>
@@ -4866,7 +4867,7 @@
       <c r="D294" s="4"/>
       <c r="E294" s="4"/>
       <c r="F294" s="20" t="str">
-        <f aca="false">IF(AND(D294="",E294=""),"",'Start Here'!$B$4+SUM($D$5:D294)-SUM($E$5:E294))</f>
+        <f aca="false">IF(AND(D294="",E294=""),"",'Start Here'!$B$4+SUM($D$5:D294)+SUM($E$5:E294))</f>
         <v/>
       </c>
       <c r="G294" s="5"/>
@@ -4878,7 +4879,7 @@
       <c r="D295" s="4"/>
       <c r="E295" s="4"/>
       <c r="F295" s="20" t="str">
-        <f aca="false">IF(AND(D295="",E295=""),"",'Start Here'!$B$4+SUM($D$5:D295)-SUM($E$5:E295))</f>
+        <f aca="false">IF(AND(D295="",E295=""),"",'Start Here'!$B$4+SUM($D$5:D295)+SUM($E$5:E295))</f>
         <v/>
       </c>
       <c r="G295" s="5"/>
@@ -4890,7 +4891,7 @@
       <c r="D296" s="4"/>
       <c r="E296" s="4"/>
       <c r="F296" s="20" t="str">
-        <f aca="false">IF(AND(D296="",E296=""),"",'Start Here'!$B$4+SUM($D$5:D296)-SUM($E$5:E296))</f>
+        <f aca="false">IF(AND(D296="",E296=""),"",'Start Here'!$B$4+SUM($D$5:D296)+SUM($E$5:E296))</f>
         <v/>
       </c>
       <c r="G296" s="5"/>
@@ -4902,7 +4903,7 @@
       <c r="D297" s="4"/>
       <c r="E297" s="4"/>
       <c r="F297" s="20" t="str">
-        <f aca="false">IF(AND(D297="",E297=""),"",'Start Here'!$B$4+SUM($D$5:D297)-SUM($E$5:E297))</f>
+        <f aca="false">IF(AND(D297="",E297=""),"",'Start Here'!$B$4+SUM($D$5:D297)+SUM($E$5:E297))</f>
         <v/>
       </c>
       <c r="G297" s="5"/>
@@ -4914,7 +4915,7 @@
       <c r="D298" s="4"/>
       <c r="E298" s="4"/>
       <c r="F298" s="20" t="str">
-        <f aca="false">IF(AND(D298="",E298=""),"",'Start Here'!$B$4+SUM($D$5:D298)-SUM($E$5:E298))</f>
+        <f aca="false">IF(AND(D298="",E298=""),"",'Start Here'!$B$4+SUM($D$5:D298)+SUM($E$5:E298))</f>
         <v/>
       </c>
       <c r="G298" s="5"/>
@@ -4926,7 +4927,7 @@
       <c r="D299" s="4"/>
       <c r="E299" s="4"/>
       <c r="F299" s="20" t="str">
-        <f aca="false">IF(AND(D299="",E299=""),"",'Start Here'!$B$4+SUM($D$5:D299)-SUM($E$5:E299))</f>
+        <f aca="false">IF(AND(D299="",E299=""),"",'Start Here'!$B$4+SUM($D$5:D299)+SUM($E$5:E299))</f>
         <v/>
       </c>
       <c r="G299" s="5"/>
@@ -4938,7 +4939,7 @@
       <c r="D300" s="4"/>
       <c r="E300" s="4"/>
       <c r="F300" s="20" t="str">
-        <f aca="false">IF(AND(D300="",E300=""),"",'Start Here'!$B$4+SUM($D$5:D300)-SUM($E$5:E300))</f>
+        <f aca="false">IF(AND(D300="",E300=""),"",'Start Here'!$B$4+SUM($D$5:D300)+SUM($E$5:E300))</f>
         <v/>
       </c>
       <c r="G300" s="5"/>
@@ -4950,7 +4951,7 @@
       <c r="D301" s="4"/>
       <c r="E301" s="4"/>
       <c r="F301" s="20" t="str">
-        <f aca="false">IF(AND(D301="",E301=""),"",'Start Here'!$B$4+SUM($D$5:D301)-SUM($E$5:E301))</f>
+        <f aca="false">IF(AND(D301="",E301=""),"",'Start Here'!$B$4+SUM($D$5:D301)+SUM($E$5:E301))</f>
         <v/>
       </c>
       <c r="G301" s="5"/>
@@ -4962,7 +4963,7 @@
       <c r="D302" s="4"/>
       <c r="E302" s="4"/>
       <c r="F302" s="20" t="str">
-        <f aca="false">IF(AND(D302="",E302=""),"",'Start Here'!$B$4+SUM($D$5:D302)-SUM($E$5:E302))</f>
+        <f aca="false">IF(AND(D302="",E302=""),"",'Start Here'!$B$4+SUM($D$5:D302)+SUM($E$5:E302))</f>
         <v/>
       </c>
       <c r="G302" s="5"/>
@@ -4974,7 +4975,7 @@
       <c r="D303" s="4"/>
       <c r="E303" s="4"/>
       <c r="F303" s="20" t="str">
-        <f aca="false">IF(AND(D303="",E303=""),"",'Start Here'!$B$4+SUM($D$5:D303)-SUM($E$5:E303))</f>
+        <f aca="false">IF(AND(D303="",E303=""),"",'Start Here'!$B$4+SUM($D$5:D303)+SUM($E$5:E303))</f>
         <v/>
       </c>
       <c r="G303" s="5"/>
@@ -4986,7 +4987,7 @@
       <c r="D304" s="4"/>
       <c r="E304" s="4"/>
       <c r="F304" s="20" t="str">
-        <f aca="false">IF(AND(D304="",E304=""),"",'Start Here'!$B$4+SUM($D$5:D304)-SUM($E$5:E304))</f>
+        <f aca="false">IF(AND(D304="",E304=""),"",'Start Here'!$B$4+SUM($D$5:D304)+SUM($E$5:E304))</f>
         <v/>
       </c>
       <c r="G304" s="5"/>
@@ -4998,7 +4999,7 @@
       <c r="D305" s="4"/>
       <c r="E305" s="4"/>
       <c r="F305" s="20" t="str">
-        <f aca="false">IF(AND(D305="",E305=""),"",'Start Here'!$B$4+SUM($D$5:D305)-SUM($E$5:E305))</f>
+        <f aca="false">IF(AND(D305="",E305=""),"",'Start Here'!$B$4+SUM($D$5:D305)+SUM($E$5:E305))</f>
         <v/>
       </c>
       <c r="G305" s="5"/>
@@ -5010,7 +5011,7 @@
       <c r="D306" s="4"/>
       <c r="E306" s="4"/>
       <c r="F306" s="20" t="str">
-        <f aca="false">IF(AND(D306="",E306=""),"",'Start Here'!$B$4+SUM($D$5:D306)-SUM($E$5:E306))</f>
+        <f aca="false">IF(AND(D306="",E306=""),"",'Start Here'!$B$4+SUM($D$5:D306)+SUM($E$5:E306))</f>
         <v/>
       </c>
       <c r="G306" s="5"/>
@@ -5022,7 +5023,7 @@
       <c r="D307" s="4"/>
       <c r="E307" s="4"/>
       <c r="F307" s="20" t="str">
-        <f aca="false">IF(AND(D307="",E307=""),"",'Start Here'!$B$4+SUM($D$5:D307)-SUM($E$5:E307))</f>
+        <f aca="false">IF(AND(D307="",E307=""),"",'Start Here'!$B$4+SUM($D$5:D307)+SUM($E$5:E307))</f>
         <v/>
       </c>
       <c r="G307" s="5"/>
@@ -5034,7 +5035,7 @@
       <c r="D308" s="4"/>
       <c r="E308" s="4"/>
       <c r="F308" s="20" t="str">
-        <f aca="false">IF(AND(D308="",E308=""),"",'Start Here'!$B$4+SUM($D$5:D308)-SUM($E$5:E308))</f>
+        <f aca="false">IF(AND(D308="",E308=""),"",'Start Here'!$B$4+SUM($D$5:D308)+SUM($E$5:E308))</f>
         <v/>
       </c>
       <c r="G308" s="5"/>
@@ -5046,7 +5047,7 @@
       <c r="D309" s="4"/>
       <c r="E309" s="4"/>
       <c r="F309" s="20" t="str">
-        <f aca="false">IF(AND(D309="",E309=""),"",'Start Here'!$B$4+SUM($D$5:D309)-SUM($E$5:E309))</f>
+        <f aca="false">IF(AND(D309="",E309=""),"",'Start Here'!$B$4+SUM($D$5:D309)+SUM($E$5:E309))</f>
         <v/>
       </c>
       <c r="G309" s="5"/>
@@ -5058,7 +5059,7 @@
       <c r="D310" s="4"/>
       <c r="E310" s="4"/>
       <c r="F310" s="20" t="str">
-        <f aca="false">IF(AND(D310="",E310=""),"",'Start Here'!$B$4+SUM($D$5:D310)-SUM($E$5:E310))</f>
+        <f aca="false">IF(AND(D310="",E310=""),"",'Start Here'!$B$4+SUM($D$5:D310)+SUM($E$5:E310))</f>
         <v/>
       </c>
       <c r="G310" s="5"/>
@@ -5070,7 +5071,7 @@
       <c r="D311" s="4"/>
       <c r="E311" s="4"/>
       <c r="F311" s="20" t="str">
-        <f aca="false">IF(AND(D311="",E311=""),"",'Start Here'!$B$4+SUM($D$5:D311)-SUM($E$5:E311))</f>
+        <f aca="false">IF(AND(D311="",E311=""),"",'Start Here'!$B$4+SUM($D$5:D311)+SUM($E$5:E311))</f>
         <v/>
       </c>
       <c r="G311" s="5"/>
@@ -5082,7 +5083,7 @@
       <c r="D312" s="4"/>
       <c r="E312" s="4"/>
       <c r="F312" s="20" t="str">
-        <f aca="false">IF(AND(D312="",E312=""),"",'Start Here'!$B$4+SUM($D$5:D312)-SUM($E$5:E312))</f>
+        <f aca="false">IF(AND(D312="",E312=""),"",'Start Here'!$B$4+SUM($D$5:D312)+SUM($E$5:E312))</f>
         <v/>
       </c>
       <c r="G312" s="5"/>
@@ -5094,7 +5095,7 @@
       <c r="D313" s="4"/>
       <c r="E313" s="4"/>
       <c r="F313" s="20" t="str">
-        <f aca="false">IF(AND(D313="",E313=""),"",'Start Here'!$B$4+SUM($D$5:D313)-SUM($E$5:E313))</f>
+        <f aca="false">IF(AND(D313="",E313=""),"",'Start Here'!$B$4+SUM($D$5:D313)+SUM($E$5:E313))</f>
         <v/>
       </c>
       <c r="G313" s="5"/>
@@ -5106,7 +5107,7 @@
       <c r="D314" s="4"/>
       <c r="E314" s="4"/>
       <c r="F314" s="20" t="str">
-        <f aca="false">IF(AND(D314="",E314=""),"",'Start Here'!$B$4+SUM($D$5:D314)-SUM($E$5:E314))</f>
+        <f aca="false">IF(AND(D314="",E314=""),"",'Start Here'!$B$4+SUM($D$5:D314)+SUM($E$5:E314))</f>
         <v/>
       </c>
       <c r="G314" s="5"/>
@@ -5118,7 +5119,7 @@
       <c r="D315" s="4"/>
       <c r="E315" s="4"/>
       <c r="F315" s="20" t="str">
-        <f aca="false">IF(AND(D315="",E315=""),"",'Start Here'!$B$4+SUM($D$5:D315)-SUM($E$5:E315))</f>
+        <f aca="false">IF(AND(D315="",E315=""),"",'Start Here'!$B$4+SUM($D$5:D315)+SUM($E$5:E315))</f>
         <v/>
       </c>
       <c r="G315" s="5"/>
@@ -5130,7 +5131,7 @@
       <c r="D316" s="4"/>
       <c r="E316" s="4"/>
       <c r="F316" s="20" t="str">
-        <f aca="false">IF(AND(D316="",E316=""),"",'Start Here'!$B$4+SUM($D$5:D316)-SUM($E$5:E316))</f>
+        <f aca="false">IF(AND(D316="",E316=""),"",'Start Here'!$B$4+SUM($D$5:D316)+SUM($E$5:E316))</f>
         <v/>
       </c>
       <c r="G316" s="5"/>
@@ -5142,7 +5143,7 @@
       <c r="D317" s="4"/>
       <c r="E317" s="4"/>
       <c r="F317" s="20" t="str">
-        <f aca="false">IF(AND(D317="",E317=""),"",'Start Here'!$B$4+SUM($D$5:D317)-SUM($E$5:E317))</f>
+        <f aca="false">IF(AND(D317="",E317=""),"",'Start Here'!$B$4+SUM($D$5:D317)+SUM($E$5:E317))</f>
         <v/>
       </c>
       <c r="G317" s="5"/>
@@ -5154,7 +5155,7 @@
       <c r="D318" s="4"/>
       <c r="E318" s="4"/>
       <c r="F318" s="20" t="str">
-        <f aca="false">IF(AND(D318="",E318=""),"",'Start Here'!$B$4+SUM($D$5:D318)-SUM($E$5:E318))</f>
+        <f aca="false">IF(AND(D318="",E318=""),"",'Start Here'!$B$4+SUM($D$5:D318)+SUM($E$5:E318))</f>
         <v/>
       </c>
       <c r="G318" s="5"/>
@@ -5166,7 +5167,7 @@
       <c r="D319" s="4"/>
       <c r="E319" s="4"/>
       <c r="F319" s="20" t="str">
-        <f aca="false">IF(AND(D319="",E319=""),"",'Start Here'!$B$4+SUM($D$5:D319)-SUM($E$5:E319))</f>
+        <f aca="false">IF(AND(D319="",E319=""),"",'Start Here'!$B$4+SUM($D$5:D319)+SUM($E$5:E319))</f>
         <v/>
       </c>
       <c r="G319" s="5"/>
@@ -5178,7 +5179,7 @@
       <c r="D320" s="4"/>
       <c r="E320" s="4"/>
       <c r="F320" s="20" t="str">
-        <f aca="false">IF(AND(D320="",E320=""),"",'Start Here'!$B$4+SUM($D$5:D320)-SUM($E$5:E320))</f>
+        <f aca="false">IF(AND(D320="",E320=""),"",'Start Here'!$B$4+SUM($D$5:D320)+SUM($E$5:E320))</f>
         <v/>
       </c>
       <c r="G320" s="5"/>
@@ -5190,7 +5191,7 @@
       <c r="D321" s="4"/>
       <c r="E321" s="4"/>
       <c r="F321" s="20" t="str">
-        <f aca="false">IF(AND(D321="",E321=""),"",'Start Here'!$B$4+SUM($D$5:D321)-SUM($E$5:E321))</f>
+        <f aca="false">IF(AND(D321="",E321=""),"",'Start Here'!$B$4+SUM($D$5:D321)+SUM($E$5:E321))</f>
         <v/>
       </c>
       <c r="G321" s="5"/>
@@ -5202,7 +5203,7 @@
       <c r="D322" s="4"/>
       <c r="E322" s="4"/>
       <c r="F322" s="20" t="str">
-        <f aca="false">IF(AND(D322="",E322=""),"",'Start Here'!$B$4+SUM($D$5:D322)-SUM($E$5:E322))</f>
+        <f aca="false">IF(AND(D322="",E322=""),"",'Start Here'!$B$4+SUM($D$5:D322)+SUM($E$5:E322))</f>
         <v/>
       </c>
       <c r="G322" s="5"/>
@@ -5214,7 +5215,7 @@
       <c r="D323" s="4"/>
       <c r="E323" s="4"/>
       <c r="F323" s="20" t="str">
-        <f aca="false">IF(AND(D323="",E323=""),"",'Start Here'!$B$4+SUM($D$5:D323)-SUM($E$5:E323))</f>
+        <f aca="false">IF(AND(D323="",E323=""),"",'Start Here'!$B$4+SUM($D$5:D323)+SUM($E$5:E323))</f>
         <v/>
       </c>
       <c r="G323" s="5"/>
@@ -5226,7 +5227,7 @@
       <c r="D324" s="4"/>
       <c r="E324" s="4"/>
       <c r="F324" s="20" t="str">
-        <f aca="false">IF(AND(D324="",E324=""),"",'Start Here'!$B$4+SUM($D$5:D324)-SUM($E$5:E324))</f>
+        <f aca="false">IF(AND(D324="",E324=""),"",'Start Here'!$B$4+SUM($D$5:D324)+SUM($E$5:E324))</f>
         <v/>
       </c>
       <c r="G324" s="5"/>
@@ -5238,7 +5239,7 @@
       <c r="D325" s="4"/>
       <c r="E325" s="4"/>
       <c r="F325" s="20" t="str">
-        <f aca="false">IF(AND(D325="",E325=""),"",'Start Here'!$B$4+SUM($D$5:D325)-SUM($E$5:E325))</f>
+        <f aca="false">IF(AND(D325="",E325=""),"",'Start Here'!$B$4+SUM($D$5:D325)+SUM($E$5:E325))</f>
         <v/>
       </c>
       <c r="G325" s="5"/>
@@ -5250,7 +5251,7 @@
       <c r="D326" s="4"/>
       <c r="E326" s="4"/>
       <c r="F326" s="20" t="str">
-        <f aca="false">IF(AND(D326="",E326=""),"",'Start Here'!$B$4+SUM($D$5:D326)-SUM($E$5:E326))</f>
+        <f aca="false">IF(AND(D326="",E326=""),"",'Start Here'!$B$4+SUM($D$5:D326)+SUM($E$5:E326))</f>
         <v/>
       </c>
       <c r="G326" s="5"/>
@@ -5262,7 +5263,7 @@
       <c r="D327" s="4"/>
       <c r="E327" s="4"/>
       <c r="F327" s="20" t="str">
-        <f aca="false">IF(AND(D327="",E327=""),"",'Start Here'!$B$4+SUM($D$5:D327)-SUM($E$5:E327))</f>
+        <f aca="false">IF(AND(D327="",E327=""),"",'Start Here'!$B$4+SUM($D$5:D327)+SUM($E$5:E327))</f>
         <v/>
       </c>
       <c r="G327" s="5"/>
@@ -5274,7 +5275,7 @@
       <c r="D328" s="4"/>
       <c r="E328" s="4"/>
       <c r="F328" s="20" t="str">
-        <f aca="false">IF(AND(D328="",E328=""),"",'Start Here'!$B$4+SUM($D$5:D328)-SUM($E$5:E328))</f>
+        <f aca="false">IF(AND(D328="",E328=""),"",'Start Here'!$B$4+SUM($D$5:D328)+SUM($E$5:E328))</f>
         <v/>
       </c>
       <c r="G328" s="5"/>
@@ -5286,7 +5287,7 @@
       <c r="D329" s="4"/>
       <c r="E329" s="4"/>
       <c r="F329" s="20" t="str">
-        <f aca="false">IF(AND(D329="",E329=""),"",'Start Here'!$B$4+SUM($D$5:D329)-SUM($E$5:E329))</f>
+        <f aca="false">IF(AND(D329="",E329=""),"",'Start Here'!$B$4+SUM($D$5:D329)+SUM($E$5:E329))</f>
         <v/>
       </c>
       <c r="G329" s="5"/>
@@ -5298,7 +5299,7 @@
       <c r="D330" s="4"/>
       <c r="E330" s="4"/>
       <c r="F330" s="20" t="str">
-        <f aca="false">IF(AND(D330="",E330=""),"",'Start Here'!$B$4+SUM($D$5:D330)-SUM($E$5:E330))</f>
+        <f aca="false">IF(AND(D330="",E330=""),"",'Start Here'!$B$4+SUM($D$5:D330)+SUM($E$5:E330))</f>
         <v/>
       </c>
       <c r="G330" s="5"/>
@@ -5310,7 +5311,7 @@
       <c r="D331" s="4"/>
       <c r="E331" s="4"/>
       <c r="F331" s="20" t="str">
-        <f aca="false">IF(AND(D331="",E331=""),"",'Start Here'!$B$4+SUM($D$5:D331)-SUM($E$5:E331))</f>
+        <f aca="false">IF(AND(D331="",E331=""),"",'Start Here'!$B$4+SUM($D$5:D331)+SUM($E$5:E331))</f>
         <v/>
       </c>
       <c r="G331" s="5"/>
@@ -5322,7 +5323,7 @@
       <c r="D332" s="4"/>
       <c r="E332" s="4"/>
       <c r="F332" s="20" t="str">
-        <f aca="false">IF(AND(D332="",E332=""),"",'Start Here'!$B$4+SUM($D$5:D332)-SUM($E$5:E332))</f>
+        <f aca="false">IF(AND(D332="",E332=""),"",'Start Here'!$B$4+SUM($D$5:D332)+SUM($E$5:E332))</f>
         <v/>
       </c>
       <c r="G332" s="5"/>
@@ -5334,7 +5335,7 @@
       <c r="D333" s="4"/>
       <c r="E333" s="4"/>
       <c r="F333" s="20" t="str">
-        <f aca="false">IF(AND(D333="",E333=""),"",'Start Here'!$B$4+SUM($D$5:D333)-SUM($E$5:E333))</f>
+        <f aca="false">IF(AND(D333="",E333=""),"",'Start Here'!$B$4+SUM($D$5:D333)+SUM($E$5:E333))</f>
         <v/>
       </c>
       <c r="G333" s="5"/>
@@ -5346,7 +5347,7 @@
       <c r="D334" s="4"/>
       <c r="E334" s="4"/>
       <c r="F334" s="20" t="str">
-        <f aca="false">IF(AND(D334="",E334=""),"",'Start Here'!$B$4+SUM($D$5:D334)-SUM($E$5:E334))</f>
+        <f aca="false">IF(AND(D334="",E334=""),"",'Start Here'!$B$4+SUM($D$5:D334)+SUM($E$5:E334))</f>
         <v/>
       </c>
       <c r="G334" s="5"/>
@@ -5358,7 +5359,7 @@
       <c r="D335" s="4"/>
       <c r="E335" s="4"/>
       <c r="F335" s="20" t="str">
-        <f aca="false">IF(AND(D335="",E335=""),"",'Start Here'!$B$4+SUM($D$5:D335)-SUM($E$5:E335))</f>
+        <f aca="false">IF(AND(D335="",E335=""),"",'Start Here'!$B$4+SUM($D$5:D335)+SUM($E$5:E335))</f>
         <v/>
       </c>
       <c r="G335" s="5"/>
@@ -5370,7 +5371,7 @@
       <c r="D336" s="4"/>
       <c r="E336" s="4"/>
       <c r="F336" s="20" t="str">
-        <f aca="false">IF(AND(D336="",E336=""),"",'Start Here'!$B$4+SUM($D$5:D336)-SUM($E$5:E336))</f>
+        <f aca="false">IF(AND(D336="",E336=""),"",'Start Here'!$B$4+SUM($D$5:D336)+SUM($E$5:E336))</f>
         <v/>
       </c>
       <c r="G336" s="5"/>
@@ -5382,7 +5383,7 @@
       <c r="D337" s="4"/>
       <c r="E337" s="4"/>
       <c r="F337" s="20" t="str">
-        <f aca="false">IF(AND(D337="",E337=""),"",'Start Here'!$B$4+SUM($D$5:D337)-SUM($E$5:E337))</f>
+        <f aca="false">IF(AND(D337="",E337=""),"",'Start Here'!$B$4+SUM($D$5:D337)+SUM($E$5:E337))</f>
         <v/>
       </c>
       <c r="G337" s="5"/>
@@ -5394,7 +5395,7 @@
       <c r="D338" s="4"/>
       <c r="E338" s="4"/>
       <c r="F338" s="20" t="str">
-        <f aca="false">IF(AND(D338="",E338=""),"",'Start Here'!$B$4+SUM($D$5:D338)-SUM($E$5:E338))</f>
+        <f aca="false">IF(AND(D338="",E338=""),"",'Start Here'!$B$4+SUM($D$5:D338)+SUM($E$5:E338))</f>
         <v/>
       </c>
       <c r="G338" s="5"/>
@@ -5406,7 +5407,7 @@
       <c r="D339" s="4"/>
       <c r="E339" s="4"/>
       <c r="F339" s="20" t="str">
-        <f aca="false">IF(AND(D339="",E339=""),"",'Start Here'!$B$4+SUM($D$5:D339)-SUM($E$5:E339))</f>
+        <f aca="false">IF(AND(D339="",E339=""),"",'Start Here'!$B$4+SUM($D$5:D339)+SUM($E$5:E339))</f>
         <v/>
       </c>
       <c r="G339" s="5"/>
@@ -5418,7 +5419,7 @@
       <c r="D340" s="4"/>
       <c r="E340" s="4"/>
       <c r="F340" s="20" t="str">
-        <f aca="false">IF(AND(D340="",E340=""),"",'Start Here'!$B$4+SUM($D$5:D340)-SUM($E$5:E340))</f>
+        <f aca="false">IF(AND(D340="",E340=""),"",'Start Here'!$B$4+SUM($D$5:D340)+SUM($E$5:E340))</f>
         <v/>
       </c>
       <c r="G340" s="5"/>
@@ -5430,7 +5431,7 @@
       <c r="D341" s="4"/>
       <c r="E341" s="4"/>
       <c r="F341" s="20" t="str">
-        <f aca="false">IF(AND(D341="",E341=""),"",'Start Here'!$B$4+SUM($D$5:D341)-SUM($E$5:E341))</f>
+        <f aca="false">IF(AND(D341="",E341=""),"",'Start Here'!$B$4+SUM($D$5:D341)+SUM($E$5:E341))</f>
         <v/>
       </c>
       <c r="G341" s="5"/>
@@ -5442,7 +5443,7 @@
       <c r="D342" s="4"/>
       <c r="E342" s="4"/>
       <c r="F342" s="20" t="str">
-        <f aca="false">IF(AND(D342="",E342=""),"",'Start Here'!$B$4+SUM($D$5:D342)-SUM($E$5:E342))</f>
+        <f aca="false">IF(AND(D342="",E342=""),"",'Start Here'!$B$4+SUM($D$5:D342)+SUM($E$5:E342))</f>
         <v/>
       </c>
       <c r="G342" s="5"/>
@@ -5454,7 +5455,7 @@
       <c r="D343" s="4"/>
       <c r="E343" s="4"/>
       <c r="F343" s="20" t="str">
-        <f aca="false">IF(AND(D343="",E343=""),"",'Start Here'!$B$4+SUM($D$5:D343)-SUM($E$5:E343))</f>
+        <f aca="false">IF(AND(D343="",E343=""),"",'Start Here'!$B$4+SUM($D$5:D343)+SUM($E$5:E343))</f>
         <v/>
       </c>
       <c r="G343" s="5"/>
@@ -5466,7 +5467,7 @@
       <c r="D344" s="4"/>
       <c r="E344" s="4"/>
       <c r="F344" s="20" t="str">
-        <f aca="false">IF(AND(D344="",E344=""),"",'Start Here'!$B$4+SUM($D$5:D344)-SUM($E$5:E344))</f>
+        <f aca="false">IF(AND(D344="",E344=""),"",'Start Here'!$B$4+SUM($D$5:D344)+SUM($E$5:E344))</f>
         <v/>
       </c>
       <c r="G344" s="5"/>
@@ -5478,7 +5479,7 @@
       <c r="D345" s="4"/>
       <c r="E345" s="4"/>
       <c r="F345" s="20" t="str">
-        <f aca="false">IF(AND(D345="",E345=""),"",'Start Here'!$B$4+SUM($D$5:D345)-SUM($E$5:E345))</f>
+        <f aca="false">IF(AND(D345="",E345=""),"",'Start Here'!$B$4+SUM($D$5:D345)+SUM($E$5:E345))</f>
         <v/>
       </c>
       <c r="G345" s="5"/>
@@ -5490,7 +5491,7 @@
       <c r="D346" s="4"/>
       <c r="E346" s="4"/>
       <c r="F346" s="20" t="str">
-        <f aca="false">IF(AND(D346="",E346=""),"",'Start Here'!$B$4+SUM($D$5:D346)-SUM($E$5:E346))</f>
+        <f aca="false">IF(AND(D346="",E346=""),"",'Start Here'!$B$4+SUM($D$5:D346)+SUM($E$5:E346))</f>
         <v/>
       </c>
       <c r="G346" s="5"/>
@@ -5502,7 +5503,7 @@
       <c r="D347" s="4"/>
       <c r="E347" s="4"/>
       <c r="F347" s="20" t="str">
-        <f aca="false">IF(AND(D347="",E347=""),"",'Start Here'!$B$4+SUM($D$5:D347)-SUM($E$5:E347))</f>
+        <f aca="false">IF(AND(D347="",E347=""),"",'Start Here'!$B$4+SUM($D$5:D347)+SUM($E$5:E347))</f>
         <v/>
       </c>
       <c r="G347" s="5"/>
@@ -5514,7 +5515,7 @@
       <c r="D348" s="4"/>
       <c r="E348" s="4"/>
       <c r="F348" s="20" t="str">
-        <f aca="false">IF(AND(D348="",E348=""),"",'Start Here'!$B$4+SUM($D$5:D348)-SUM($E$5:E348))</f>
+        <f aca="false">IF(AND(D348="",E348=""),"",'Start Here'!$B$4+SUM($D$5:D348)+SUM($E$5:E348))</f>
         <v/>
       </c>
       <c r="G348" s="5"/>
@@ -5526,7 +5527,7 @@
       <c r="D349" s="4"/>
       <c r="E349" s="4"/>
       <c r="F349" s="20" t="str">
-        <f aca="false">IF(AND(D349="",E349=""),"",'Start Here'!$B$4+SUM($D$5:D349)-SUM($E$5:E349))</f>
+        <f aca="false">IF(AND(D349="",E349=""),"",'Start Here'!$B$4+SUM($D$5:D349)+SUM($E$5:E349))</f>
         <v/>
       </c>
       <c r="G349" s="5"/>
@@ -5538,7 +5539,7 @@
       <c r="D350" s="4"/>
       <c r="E350" s="4"/>
       <c r="F350" s="20" t="str">
-        <f aca="false">IF(AND(D350="",E350=""),"",'Start Here'!$B$4+SUM($D$5:D350)-SUM($E$5:E350))</f>
+        <f aca="false">IF(AND(D350="",E350=""),"",'Start Here'!$B$4+SUM($D$5:D350)+SUM($E$5:E350))</f>
         <v/>
       </c>
       <c r="G350" s="5"/>
@@ -5550,7 +5551,7 @@
       <c r="D351" s="4"/>
       <c r="E351" s="4"/>
       <c r="F351" s="20" t="str">
-        <f aca="false">IF(AND(D351="",E351=""),"",'Start Here'!$B$4+SUM($D$5:D351)-SUM($E$5:E351))</f>
+        <f aca="false">IF(AND(D351="",E351=""),"",'Start Here'!$B$4+SUM($D$5:D351)+SUM($E$5:E351))</f>
         <v/>
       </c>
       <c r="G351" s="5"/>
@@ -5562,7 +5563,7 @@
       <c r="D352" s="4"/>
       <c r="E352" s="4"/>
       <c r="F352" s="20" t="str">
-        <f aca="false">IF(AND(D352="",E352=""),"",'Start Here'!$B$4+SUM($D$5:D352)-SUM($E$5:E352))</f>
+        <f aca="false">IF(AND(D352="",E352=""),"",'Start Here'!$B$4+SUM($D$5:D352)+SUM($E$5:E352))</f>
         <v/>
       </c>
       <c r="G352" s="5"/>
@@ -5574,7 +5575,7 @@
       <c r="D353" s="4"/>
       <c r="E353" s="4"/>
       <c r="F353" s="20" t="str">
-        <f aca="false">IF(AND(D353="",E353=""),"",'Start Here'!$B$4+SUM($D$5:D353)-SUM($E$5:E353))</f>
+        <f aca="false">IF(AND(D353="",E353=""),"",'Start Here'!$B$4+SUM($D$5:D353)+SUM($E$5:E353))</f>
         <v/>
       </c>
       <c r="G353" s="5"/>
@@ -5586,7 +5587,7 @@
       <c r="D354" s="4"/>
       <c r="E354" s="4"/>
       <c r="F354" s="20" t="str">
-        <f aca="false">IF(AND(D354="",E354=""),"",'Start Here'!$B$4+SUM($D$5:D354)-SUM($E$5:E354))</f>
+        <f aca="false">IF(AND(D354="",E354=""),"",'Start Here'!$B$4+SUM($D$5:D354)+SUM($E$5:E354))</f>
         <v/>
       </c>
       <c r="G354" s="5"/>
@@ -5598,7 +5599,7 @@
       <c r="D355" s="4"/>
       <c r="E355" s="4"/>
       <c r="F355" s="20" t="str">
-        <f aca="false">IF(AND(D355="",E355=""),"",'Start Here'!$B$4+SUM($D$5:D355)-SUM($E$5:E355))</f>
+        <f aca="false">IF(AND(D355="",E355=""),"",'Start Here'!$B$4+SUM($D$5:D355)+SUM($E$5:E355))</f>
         <v/>
       </c>
       <c r="G355" s="5"/>
@@ -5610,7 +5611,7 @@
       <c r="D356" s="4"/>
       <c r="E356" s="4"/>
       <c r="F356" s="20" t="str">
-        <f aca="false">IF(AND(D356="",E356=""),"",'Start Here'!$B$4+SUM($D$5:D356)-SUM($E$5:E356))</f>
+        <f aca="false">IF(AND(D356="",E356=""),"",'Start Here'!$B$4+SUM($D$5:D356)+SUM($E$5:E356))</f>
         <v/>
       </c>
       <c r="G356" s="5"/>
@@ -5622,7 +5623,7 @@
       <c r="D357" s="4"/>
       <c r="E357" s="4"/>
       <c r="F357" s="20" t="str">
-        <f aca="false">IF(AND(D357="",E357=""),"",'Start Here'!$B$4+SUM($D$5:D357)-SUM($E$5:E357))</f>
+        <f aca="false">IF(AND(D357="",E357=""),"",'Start Here'!$B$4+SUM($D$5:D357)+SUM($E$5:E357))</f>
         <v/>
       </c>
       <c r="G357" s="5"/>
@@ -5634,7 +5635,7 @@
       <c r="D358" s="4"/>
       <c r="E358" s="4"/>
       <c r="F358" s="20" t="str">
-        <f aca="false">IF(AND(D358="",E358=""),"",'Start Here'!$B$4+SUM($D$5:D358)-SUM($E$5:E358))</f>
+        <f aca="false">IF(AND(D358="",E358=""),"",'Start Here'!$B$4+SUM($D$5:D358)+SUM($E$5:E358))</f>
         <v/>
       </c>
       <c r="G358" s="5"/>
@@ -5646,7 +5647,7 @@
       <c r="D359" s="4"/>
       <c r="E359" s="4"/>
       <c r="F359" s="20" t="str">
-        <f aca="false">IF(AND(D359="",E359=""),"",'Start Here'!$B$4+SUM($D$5:D359)-SUM($E$5:E359))</f>
+        <f aca="false">IF(AND(D359="",E359=""),"",'Start Here'!$B$4+SUM($D$5:D359)+SUM($E$5:E359))</f>
         <v/>
       </c>
       <c r="G359" s="5"/>
@@ -5658,7 +5659,7 @@
       <c r="D360" s="4"/>
       <c r="E360" s="4"/>
       <c r="F360" s="20" t="str">
-        <f aca="false">IF(AND(D360="",E360=""),"",'Start Here'!$B$4+SUM($D$5:D360)-SUM($E$5:E360))</f>
+        <f aca="false">IF(AND(D360="",E360=""),"",'Start Here'!$B$4+SUM($D$5:D360)+SUM($E$5:E360))</f>
         <v/>
       </c>
       <c r="G360" s="5"/>
@@ -5670,7 +5671,7 @@
       <c r="D361" s="4"/>
       <c r="E361" s="4"/>
       <c r="F361" s="20" t="str">
-        <f aca="false">IF(AND(D361="",E361=""),"",'Start Here'!$B$4+SUM($D$5:D361)-SUM($E$5:E361))</f>
+        <f aca="false">IF(AND(D361="",E361=""),"",'Start Here'!$B$4+SUM($D$5:D361)+SUM($E$5:E361))</f>
         <v/>
       </c>
       <c r="G361" s="5"/>
@@ -5682,7 +5683,7 @@
       <c r="D362" s="4"/>
       <c r="E362" s="4"/>
       <c r="F362" s="20" t="str">
-        <f aca="false">IF(AND(D362="",E362=""),"",'Start Here'!$B$4+SUM($D$5:D362)-SUM($E$5:E362))</f>
+        <f aca="false">IF(AND(D362="",E362=""),"",'Start Here'!$B$4+SUM($D$5:D362)+SUM($E$5:E362))</f>
         <v/>
       </c>
       <c r="G362" s="5"/>
@@ -5694,7 +5695,7 @@
       <c r="D363" s="4"/>
       <c r="E363" s="4"/>
       <c r="F363" s="20" t="str">
-        <f aca="false">IF(AND(D363="",E363=""),"",'Start Here'!$B$4+SUM($D$5:D363)-SUM($E$5:E363))</f>
+        <f aca="false">IF(AND(D363="",E363=""),"",'Start Here'!$B$4+SUM($D$5:D363)+SUM($E$5:E363))</f>
         <v/>
       </c>
       <c r="G363" s="5"/>
@@ -5706,7 +5707,7 @@
       <c r="D364" s="4"/>
       <c r="E364" s="4"/>
       <c r="F364" s="20" t="str">
-        <f aca="false">IF(AND(D364="",E364=""),"",'Start Here'!$B$4+SUM($D$5:D364)-SUM($E$5:E364))</f>
+        <f aca="false">IF(AND(D364="",E364=""),"",'Start Here'!$B$4+SUM($D$5:D364)+SUM($E$5:E364))</f>
         <v/>
       </c>
       <c r="G364" s="5"/>
@@ -5718,7 +5719,7 @@
       <c r="D365" s="4"/>
       <c r="E365" s="4"/>
       <c r="F365" s="20" t="str">
-        <f aca="false">IF(AND(D365="",E365=""),"",'Start Here'!$B$4+SUM($D$5:D365)-SUM($E$5:E365))</f>
+        <f aca="false">IF(AND(D365="",E365=""),"",'Start Here'!$B$4+SUM($D$5:D365)+SUM($E$5:E365))</f>
         <v/>
       </c>
       <c r="G365" s="5"/>
@@ -5730,7 +5731,7 @@
       <c r="D366" s="4"/>
       <c r="E366" s="4"/>
       <c r="F366" s="20" t="str">
-        <f aca="false">IF(AND(D366="",E366=""),"",'Start Here'!$B$4+SUM($D$5:D366)-SUM($E$5:E366))</f>
+        <f aca="false">IF(AND(D366="",E366=""),"",'Start Here'!$B$4+SUM($D$5:D366)+SUM($E$5:E366))</f>
         <v/>
       </c>
       <c r="G366" s="5"/>
@@ -5742,7 +5743,7 @@
       <c r="D367" s="4"/>
       <c r="E367" s="4"/>
       <c r="F367" s="20" t="str">
-        <f aca="false">IF(AND(D367="",E367=""),"",'Start Here'!$B$4+SUM($D$5:D367)-SUM($E$5:E367))</f>
+        <f aca="false">IF(AND(D367="",E367=""),"",'Start Here'!$B$4+SUM($D$5:D367)+SUM($E$5:E367))</f>
         <v/>
       </c>
       <c r="G367" s="5"/>
@@ -5754,7 +5755,7 @@
       <c r="D368" s="4"/>
       <c r="E368" s="4"/>
       <c r="F368" s="20" t="str">
-        <f aca="false">IF(AND(D368="",E368=""),"",'Start Here'!$B$4+SUM($D$5:D368)-SUM($E$5:E368))</f>
+        <f aca="false">IF(AND(D368="",E368=""),"",'Start Here'!$B$4+SUM($D$5:D368)+SUM($E$5:E368))</f>
         <v/>
       </c>
       <c r="G368" s="5"/>
@@ -5766,7 +5767,7 @@
       <c r="D369" s="4"/>
       <c r="E369" s="4"/>
       <c r="F369" s="20" t="str">
-        <f aca="false">IF(AND(D369="",E369=""),"",'Start Here'!$B$4+SUM($D$5:D369)-SUM($E$5:E369))</f>
+        <f aca="false">IF(AND(D369="",E369=""),"",'Start Here'!$B$4+SUM($D$5:D369)+SUM($E$5:E369))</f>
         <v/>
       </c>
       <c r="G369" s="5"/>
@@ -5778,7 +5779,7 @@
       <c r="D370" s="4"/>
       <c r="E370" s="4"/>
       <c r="F370" s="20" t="str">
-        <f aca="false">IF(AND(D370="",E370=""),"",'Start Here'!$B$4+SUM($D$5:D370)-SUM($E$5:E370))</f>
+        <f aca="false">IF(AND(D370="",E370=""),"",'Start Here'!$B$4+SUM($D$5:D370)+SUM($E$5:E370))</f>
         <v/>
       </c>
       <c r="G370" s="5"/>
@@ -5790,7 +5791,7 @@
       <c r="D371" s="4"/>
       <c r="E371" s="4"/>
       <c r="F371" s="20" t="str">
-        <f aca="false">IF(AND(D371="",E371=""),"",'Start Here'!$B$4+SUM($D$5:D371)-SUM($E$5:E371))</f>
+        <f aca="false">IF(AND(D371="",E371=""),"",'Start Here'!$B$4+SUM($D$5:D371)+SUM($E$5:E371))</f>
         <v/>
       </c>
       <c r="G371" s="5"/>
@@ -5802,7 +5803,7 @@
       <c r="D372" s="4"/>
       <c r="E372" s="4"/>
       <c r="F372" s="20" t="str">
-        <f aca="false">IF(AND(D372="",E372=""),"",'Start Here'!$B$4+SUM($D$5:D372)-SUM($E$5:E372))</f>
+        <f aca="false">IF(AND(D372="",E372=""),"",'Start Here'!$B$4+SUM($D$5:D372)+SUM($E$5:E372))</f>
         <v/>
       </c>
       <c r="G372" s="5"/>
@@ -5814,7 +5815,7 @@
       <c r="D373" s="4"/>
       <c r="E373" s="4"/>
       <c r="F373" s="20" t="str">
-        <f aca="false">IF(AND(D373="",E373=""),"",'Start Here'!$B$4+SUM($D$5:D373)-SUM($E$5:E373))</f>
+        <f aca="false">IF(AND(D373="",E373=""),"",'Start Here'!$B$4+SUM($D$5:D373)+SUM($E$5:E373))</f>
         <v/>
       </c>
       <c r="G373" s="5"/>
@@ -5826,7 +5827,7 @@
       <c r="D374" s="4"/>
       <c r="E374" s="4"/>
       <c r="F374" s="20" t="str">
-        <f aca="false">IF(AND(D374="",E374=""),"",'Start Here'!$B$4+SUM($D$5:D374)-SUM($E$5:E374))</f>
+        <f aca="false">IF(AND(D374="",E374=""),"",'Start Here'!$B$4+SUM($D$5:D374)+SUM($E$5:E374))</f>
         <v/>
       </c>
       <c r="G374" s="5"/>
@@ -5838,7 +5839,7 @@
       <c r="D375" s="4"/>
       <c r="E375" s="4"/>
       <c r="F375" s="20" t="str">
-        <f aca="false">IF(AND(D375="",E375=""),"",'Start Here'!$B$4+SUM($D$5:D375)-SUM($E$5:E375))</f>
+        <f aca="false">IF(AND(D375="",E375=""),"",'Start Here'!$B$4+SUM($D$5:D375)+SUM($E$5:E375))</f>
         <v/>
       </c>
       <c r="G375" s="5"/>
@@ -5850,7 +5851,7 @@
       <c r="D376" s="4"/>
       <c r="E376" s="4"/>
       <c r="F376" s="20" t="str">
-        <f aca="false">IF(AND(D376="",E376=""),"",'Start Here'!$B$4+SUM($D$5:D376)-SUM($E$5:E376))</f>
+        <f aca="false">IF(AND(D376="",E376=""),"",'Start Here'!$B$4+SUM($D$5:D376)+SUM($E$5:E376))</f>
         <v/>
       </c>
       <c r="G376" s="5"/>
@@ -5862,7 +5863,7 @@
       <c r="D377" s="4"/>
       <c r="E377" s="4"/>
       <c r="F377" s="20" t="str">
-        <f aca="false">IF(AND(D377="",E377=""),"",'Start Here'!$B$4+SUM($D$5:D377)-SUM($E$5:E377))</f>
+        <f aca="false">IF(AND(D377="",E377=""),"",'Start Here'!$B$4+SUM($D$5:D377)+SUM($E$5:E377))</f>
         <v/>
       </c>
       <c r="G377" s="5"/>
@@ -5874,7 +5875,7 @@
       <c r="D378" s="4"/>
       <c r="E378" s="4"/>
       <c r="F378" s="20" t="str">
-        <f aca="false">IF(AND(D378="",E378=""),"",'Start Here'!$B$4+SUM($D$5:D378)-SUM($E$5:E378))</f>
+        <f aca="false">IF(AND(D378="",E378=""),"",'Start Here'!$B$4+SUM($D$5:D378)+SUM($E$5:E378))</f>
         <v/>
       </c>
       <c r="G378" s="5"/>
@@ -5886,7 +5887,7 @@
       <c r="D379" s="4"/>
       <c r="E379" s="4"/>
       <c r="F379" s="20" t="str">
-        <f aca="false">IF(AND(D379="",E379=""),"",'Start Here'!$B$4+SUM($D$5:D379)-SUM($E$5:E379))</f>
+        <f aca="false">IF(AND(D379="",E379=""),"",'Start Here'!$B$4+SUM($D$5:D379)+SUM($E$5:E379))</f>
         <v/>
       </c>
       <c r="G379" s="5"/>
@@ -5898,7 +5899,7 @@
       <c r="D380" s="4"/>
       <c r="E380" s="4"/>
       <c r="F380" s="20" t="str">
-        <f aca="false">IF(AND(D380="",E380=""),"",'Start Here'!$B$4+SUM($D$5:D380)-SUM($E$5:E380))</f>
+        <f aca="false">IF(AND(D380="",E380=""),"",'Start Here'!$B$4+SUM($D$5:D380)+SUM($E$5:E380))</f>
         <v/>
       </c>
       <c r="G380" s="5"/>
@@ -5910,7 +5911,7 @@
       <c r="D381" s="4"/>
       <c r="E381" s="4"/>
       <c r="F381" s="20" t="str">
-        <f aca="false">IF(AND(D381="",E381=""),"",'Start Here'!$B$4+SUM($D$5:D381)-SUM($E$5:E381))</f>
+        <f aca="false">IF(AND(D381="",E381=""),"",'Start Here'!$B$4+SUM($D$5:D381)+SUM($E$5:E381))</f>
         <v/>
       </c>
       <c r="G381" s="5"/>
@@ -5922,7 +5923,7 @@
       <c r="D382" s="4"/>
       <c r="E382" s="4"/>
       <c r="F382" s="20" t="str">
-        <f aca="false">IF(AND(D382="",E382=""),"",'Start Here'!$B$4+SUM($D$5:D382)-SUM($E$5:E382))</f>
+        <f aca="false">IF(AND(D382="",E382=""),"",'Start Here'!$B$4+SUM($D$5:D382)+SUM($E$5:E382))</f>
         <v/>
       </c>
       <c r="G382" s="5"/>
@@ -5934,7 +5935,7 @@
       <c r="D383" s="4"/>
       <c r="E383" s="4"/>
       <c r="F383" s="20" t="str">
-        <f aca="false">IF(AND(D383="",E383=""),"",'Start Here'!$B$4+SUM($D$5:D383)-SUM($E$5:E383))</f>
+        <f aca="false">IF(AND(D383="",E383=""),"",'Start Here'!$B$4+SUM($D$5:D383)+SUM($E$5:E383))</f>
         <v/>
       </c>
       <c r="G383" s="5"/>
@@ -5946,7 +5947,7 @@
       <c r="D384" s="4"/>
       <c r="E384" s="4"/>
       <c r="F384" s="20" t="str">
-        <f aca="false">IF(AND(D384="",E384=""),"",'Start Here'!$B$4+SUM($D$5:D384)-SUM($E$5:E384))</f>
+        <f aca="false">IF(AND(D384="",E384=""),"",'Start Here'!$B$4+SUM($D$5:D384)+SUM($E$5:E384))</f>
         <v/>
       </c>
       <c r="G384" s="5"/>
@@ -5958,7 +5959,7 @@
       <c r="D385" s="4"/>
       <c r="E385" s="4"/>
       <c r="F385" s="20" t="str">
-        <f aca="false">IF(AND(D385="",E385=""),"",'Start Here'!$B$4+SUM($D$5:D385)-SUM($E$5:E385))</f>
+        <f aca="false">IF(AND(D385="",E385=""),"",'Start Here'!$B$4+SUM($D$5:D385)+SUM($E$5:E385))</f>
         <v/>
       </c>
       <c r="G385" s="5"/>
@@ -5970,7 +5971,7 @@
       <c r="D386" s="4"/>
       <c r="E386" s="4"/>
       <c r="F386" s="20" t="str">
-        <f aca="false">IF(AND(D386="",E386=""),"",'Start Here'!$B$4+SUM($D$5:D386)-SUM($E$5:E386))</f>
+        <f aca="false">IF(AND(D386="",E386=""),"",'Start Here'!$B$4+SUM($D$5:D386)+SUM($E$5:E386))</f>
         <v/>
       </c>
       <c r="G386" s="5"/>
@@ -5982,7 +5983,7 @@
       <c r="D387" s="4"/>
       <c r="E387" s="4"/>
       <c r="F387" s="20" t="str">
-        <f aca="false">IF(AND(D387="",E387=""),"",'Start Here'!$B$4+SUM($D$5:D387)-SUM($E$5:E387))</f>
+        <f aca="false">IF(AND(D387="",E387=""),"",'Start Here'!$B$4+SUM($D$5:D387)+SUM($E$5:E387))</f>
         <v/>
       </c>
       <c r="G387" s="5"/>
@@ -5994,7 +5995,7 @@
       <c r="D388" s="4"/>
       <c r="E388" s="4"/>
       <c r="F388" s="20" t="str">
-        <f aca="false">IF(AND(D388="",E388=""),"",'Start Here'!$B$4+SUM($D$5:D388)-SUM($E$5:E388))</f>
+        <f aca="false">IF(AND(D388="",E388=""),"",'Start Here'!$B$4+SUM($D$5:D388)+SUM($E$5:E388))</f>
         <v/>
       </c>
       <c r="G388" s="5"/>
@@ -6006,7 +6007,7 @@
       <c r="D389" s="4"/>
       <c r="E389" s="4"/>
       <c r="F389" s="20" t="str">
-        <f aca="false">IF(AND(D389="",E389=""),"",'Start Here'!$B$4+SUM($D$5:D389)-SUM($E$5:E389))</f>
+        <f aca="false">IF(AND(D389="",E389=""),"",'Start Here'!$B$4+SUM($D$5:D389)+SUM($E$5:E389))</f>
         <v/>
       </c>
       <c r="G389" s="5"/>
@@ -6018,7 +6019,7 @@
       <c r="D390" s="4"/>
       <c r="E390" s="4"/>
       <c r="F390" s="20" t="str">
-        <f aca="false">IF(AND(D390="",E390=""),"",'Start Here'!$B$4+SUM($D$5:D390)-SUM($E$5:E390))</f>
+        <f aca="false">IF(AND(D390="",E390=""),"",'Start Here'!$B$4+SUM($D$5:D390)+SUM($E$5:E390))</f>
         <v/>
       </c>
       <c r="G390" s="5"/>
@@ -6030,7 +6031,7 @@
       <c r="D391" s="4"/>
       <c r="E391" s="4"/>
       <c r="F391" s="20" t="str">
-        <f aca="false">IF(AND(D391="",E391=""),"",'Start Here'!$B$4+SUM($D$5:D391)-SUM($E$5:E391))</f>
+        <f aca="false">IF(AND(D391="",E391=""),"",'Start Here'!$B$4+SUM($D$5:D391)+SUM($E$5:E391))</f>
         <v/>
       </c>
       <c r="G391" s="5"/>
@@ -6042,7 +6043,7 @@
       <c r="D392" s="4"/>
       <c r="E392" s="4"/>
       <c r="F392" s="20" t="str">
-        <f aca="false">IF(AND(D392="",E392=""),"",'Start Here'!$B$4+SUM($D$5:D392)-SUM($E$5:E392))</f>
+        <f aca="false">IF(AND(D392="",E392=""),"",'Start Here'!$B$4+SUM($D$5:D392)+SUM($E$5:E392))</f>
         <v/>
       </c>
       <c r="G392" s="5"/>
@@ -6054,7 +6055,7 @@
       <c r="D393" s="4"/>
       <c r="E393" s="4"/>
       <c r="F393" s="20" t="str">
-        <f aca="false">IF(AND(D393="",E393=""),"",'Start Here'!$B$4+SUM($D$5:D393)-SUM($E$5:E393))</f>
+        <f aca="false">IF(AND(D393="",E393=""),"",'Start Here'!$B$4+SUM($D$5:D393)+SUM($E$5:E393))</f>
         <v/>
       </c>
       <c r="G393" s="5"/>
@@ -6066,7 +6067,7 @@
       <c r="D394" s="4"/>
       <c r="E394" s="4"/>
       <c r="F394" s="20" t="str">
-        <f aca="false">IF(AND(D394="",E394=""),"",'Start Here'!$B$4+SUM($D$5:D394)-SUM($E$5:E394))</f>
+        <f aca="false">IF(AND(D394="",E394=""),"",'Start Here'!$B$4+SUM($D$5:D394)+SUM($E$5:E394))</f>
         <v/>
       </c>
       <c r="G394" s="5"/>
@@ -6078,7 +6079,7 @@
       <c r="D395" s="4"/>
       <c r="E395" s="4"/>
       <c r="F395" s="20" t="str">
-        <f aca="false">IF(AND(D395="",E395=""),"",'Start Here'!$B$4+SUM($D$5:D395)-SUM($E$5:E395))</f>
+        <f aca="false">IF(AND(D395="",E395=""),"",'Start Here'!$B$4+SUM($D$5:D395)+SUM($E$5:E395))</f>
         <v/>
       </c>
       <c r="G395" s="5"/>
@@ -6090,7 +6091,7 @@
       <c r="D396" s="4"/>
       <c r="E396" s="4"/>
       <c r="F396" s="20" t="str">
-        <f aca="false">IF(AND(D396="",E396=""),"",'Start Here'!$B$4+SUM($D$5:D396)-SUM($E$5:E396))</f>
+        <f aca="false">IF(AND(D396="",E396=""),"",'Start Here'!$B$4+SUM($D$5:D396)+SUM($E$5:E396))</f>
         <v/>
       </c>
       <c r="G396" s="5"/>
@@ -6102,7 +6103,7 @@
       <c r="D397" s="4"/>
       <c r="E397" s="4"/>
       <c r="F397" s="20" t="str">
-        <f aca="false">IF(AND(D397="",E397=""),"",'Start Here'!$B$4+SUM($D$5:D397)-SUM($E$5:E397))</f>
+        <f aca="false">IF(AND(D397="",E397=""),"",'Start Here'!$B$4+SUM($D$5:D397)+SUM($E$5:E397))</f>
         <v/>
       </c>
       <c r="G397" s="5"/>
@@ -6114,7 +6115,7 @@
       <c r="D398" s="4"/>
       <c r="E398" s="4"/>
       <c r="F398" s="20" t="str">
-        <f aca="false">IF(AND(D398="",E398=""),"",'Start Here'!$B$4+SUM($D$5:D398)-SUM($E$5:E398))</f>
+        <f aca="false">IF(AND(D398="",E398=""),"",'Start Here'!$B$4+SUM($D$5:D398)+SUM($E$5:E398))</f>
         <v/>
       </c>
       <c r="G398" s="5"/>
@@ -6126,7 +6127,7 @@
       <c r="D399" s="4"/>
       <c r="E399" s="4"/>
       <c r="F399" s="20" t="str">
-        <f aca="false">IF(AND(D399="",E399=""),"",'Start Here'!$B$4+SUM($D$5:D399)-SUM($E$5:E399))</f>
+        <f aca="false">IF(AND(D399="",E399=""),"",'Start Here'!$B$4+SUM($D$5:D399)+SUM($E$5:E399))</f>
         <v/>
       </c>
       <c r="G399" s="5"/>
@@ -6138,7 +6139,7 @@
       <c r="D400" s="4"/>
       <c r="E400" s="4"/>
       <c r="F400" s="20" t="str">
-        <f aca="false">IF(AND(D400="",E400=""),"",'Start Here'!$B$4+SUM($D$5:D400)-SUM($E$5:E400))</f>
+        <f aca="false">IF(AND(D400="",E400=""),"",'Start Here'!$B$4+SUM($D$5:D400)+SUM($E$5:E400))</f>
         <v/>
       </c>
       <c r="G400" s="5"/>
@@ -6150,7 +6151,7 @@
       <c r="D401" s="4"/>
       <c r="E401" s="4"/>
       <c r="F401" s="20" t="str">
-        <f aca="false">IF(AND(D401="",E401=""),"",'Start Here'!$B$4+SUM($D$5:D401)-SUM($E$5:E401))</f>
+        <f aca="false">IF(AND(D401="",E401=""),"",'Start Here'!$B$4+SUM($D$5:D401)+SUM($E$5:E401))</f>
         <v/>
       </c>
       <c r="G401" s="5"/>
@@ -6162,7 +6163,7 @@
       <c r="D402" s="4"/>
       <c r="E402" s="4"/>
       <c r="F402" s="20" t="str">
-        <f aca="false">IF(AND(D402="",E402=""),"",'Start Here'!$B$4+SUM($D$5:D402)-SUM($E$5:E402))</f>
+        <f aca="false">IF(AND(D402="",E402=""),"",'Start Here'!$B$4+SUM($D$5:D402)+SUM($E$5:E402))</f>
         <v/>
       </c>
       <c r="G402" s="5"/>
@@ -6174,7 +6175,7 @@
       <c r="D403" s="4"/>
       <c r="E403" s="4"/>
       <c r="F403" s="20" t="str">
-        <f aca="false">IF(AND(D403="",E403=""),"",'Start Here'!$B$4+SUM($D$5:D403)-SUM($E$5:E403))</f>
+        <f aca="false">IF(AND(D403="",E403=""),"",'Start Here'!$B$4+SUM($D$5:D403)+SUM($E$5:E403))</f>
         <v/>
       </c>
       <c r="G403" s="5"/>
@@ -6186,7 +6187,7 @@
       <c r="D404" s="4"/>
       <c r="E404" s="4"/>
       <c r="F404" s="20" t="str">
-        <f aca="false">IF(AND(D404="",E404=""),"",'Start Here'!$B$4+SUM($D$5:D404)-SUM($E$5:E404))</f>
+        <f aca="false">IF(AND(D404="",E404=""),"",'Start Here'!$B$4+SUM($D$5:D404)+SUM($E$5:E404))</f>
         <v/>
       </c>
       <c r="G404" s="5"/>
@@ -6198,7 +6199,7 @@
       <c r="D405" s="4"/>
       <c r="E405" s="4"/>
       <c r="F405" s="20" t="str">
-        <f aca="false">IF(AND(D405="",E405=""),"",'Start Here'!$B$4+SUM($D$5:D405)-SUM($E$5:E405))</f>
+        <f aca="false">IF(AND(D405="",E405=""),"",'Start Here'!$B$4+SUM($D$5:D405)+SUM($E$5:E405))</f>
         <v/>
       </c>
       <c r="G405" s="5"/>
@@ -6210,7 +6211,7 @@
       <c r="D406" s="4"/>
       <c r="E406" s="4"/>
       <c r="F406" s="20" t="str">
-        <f aca="false">IF(AND(D406="",E406=""),"",'Start Here'!$B$4+SUM($D$5:D406)-SUM($E$5:E406))</f>
+        <f aca="false">IF(AND(D406="",E406=""),"",'Start Here'!$B$4+SUM($D$5:D406)+SUM($E$5:E406))</f>
         <v/>
       </c>
       <c r="G406" s="5"/>
@@ -6222,7 +6223,7 @@
       <c r="D407" s="4"/>
       <c r="E407" s="4"/>
       <c r="F407" s="20" t="str">
-        <f aca="false">IF(AND(D407="",E407=""),"",'Start Here'!$B$4+SUM($D$5:D407)-SUM($E$5:E407))</f>
+        <f aca="false">IF(AND(D407="",E407=""),"",'Start Here'!$B$4+SUM($D$5:D407)+SUM($E$5:E407))</f>
         <v/>
       </c>
       <c r="G407" s="5"/>
@@ -6234,7 +6235,7 @@
       <c r="D408" s="4"/>
       <c r="E408" s="4"/>
       <c r="F408" s="20" t="str">
-        <f aca="false">IF(AND(D408="",E408=""),"",'Start Here'!$B$4+SUM($D$5:D408)-SUM($E$5:E408))</f>
+        <f aca="false">IF(AND(D408="",E408=""),"",'Start Here'!$B$4+SUM($D$5:D408)+SUM($E$5:E408))</f>
         <v/>
       </c>
       <c r="G408" s="5"/>
@@ -6246,7 +6247,7 @@
       <c r="D409" s="4"/>
       <c r="E409" s="4"/>
       <c r="F409" s="20" t="str">
-        <f aca="false">IF(AND(D409="",E409=""),"",'Start Here'!$B$4+SUM($D$5:D409)-SUM($E$5:E409))</f>
+        <f aca="false">IF(AND(D409="",E409=""),"",'Start Here'!$B$4+SUM($D$5:D409)+SUM($E$5:E409))</f>
         <v/>
       </c>
       <c r="G409" s="5"/>
@@ -6258,7 +6259,7 @@
       <c r="D410" s="4"/>
       <c r="E410" s="4"/>
       <c r="F410" s="20" t="str">
-        <f aca="false">IF(AND(D410="",E410=""),"",'Start Here'!$B$4+SUM($D$5:D410)-SUM($E$5:E410))</f>
+        <f aca="false">IF(AND(D410="",E410=""),"",'Start Here'!$B$4+SUM($D$5:D410)+SUM($E$5:E410))</f>
         <v/>
       </c>
       <c r="G410" s="5"/>
@@ -6270,7 +6271,7 @@
       <c r="D411" s="4"/>
       <c r="E411" s="4"/>
       <c r="F411" s="20" t="str">
-        <f aca="false">IF(AND(D411="",E411=""),"",'Start Here'!$B$4+SUM($D$5:D411)-SUM($E$5:E411))</f>
+        <f aca="false">IF(AND(D411="",E411=""),"",'Start Here'!$B$4+SUM($D$5:D411)+SUM($E$5:E411))</f>
         <v/>
       </c>
       <c r="G411" s="5"/>
@@ -6282,7 +6283,7 @@
       <c r="D412" s="4"/>
       <c r="E412" s="4"/>
       <c r="F412" s="20" t="str">
-        <f aca="false">IF(AND(D412="",E412=""),"",'Start Here'!$B$4+SUM($D$5:D412)-SUM($E$5:E412))</f>
+        <f aca="false">IF(AND(D412="",E412=""),"",'Start Here'!$B$4+SUM($D$5:D412)+SUM($E$5:E412))</f>
         <v/>
       </c>
       <c r="G412" s="5"/>
@@ -6294,7 +6295,7 @@
       <c r="D413" s="4"/>
       <c r="E413" s="4"/>
       <c r="F413" s="20" t="str">
-        <f aca="false">IF(AND(D413="",E413=""),"",'Start Here'!$B$4+SUM($D$5:D413)-SUM($E$5:E413))</f>
+        <f aca="false">IF(AND(D413="",E413=""),"",'Start Here'!$B$4+SUM($D$5:D413)+SUM($E$5:E413))</f>
         <v/>
       </c>
       <c r="G413" s="5"/>
@@ -6306,7 +6307,7 @@
       <c r="D414" s="4"/>
       <c r="E414" s="4"/>
       <c r="F414" s="20" t="str">
-        <f aca="false">IF(AND(D414="",E414=""),"",'Start Here'!$B$4+SUM($D$5:D414)-SUM($E$5:E414))</f>
+        <f aca="false">IF(AND(D414="",E414=""),"",'Start Here'!$B$4+SUM($D$5:D414)+SUM($E$5:E414))</f>
         <v/>
       </c>
       <c r="G414" s="5"/>
@@ -6318,7 +6319,7 @@
       <c r="D415" s="4"/>
       <c r="E415" s="4"/>
       <c r="F415" s="20" t="str">
-        <f aca="false">IF(AND(D415="",E415=""),"",'Start Here'!$B$4+SUM($D$5:D415)-SUM($E$5:E415))</f>
+        <f aca="false">IF(AND(D415="",E415=""),"",'Start Here'!$B$4+SUM($D$5:D415)+SUM($E$5:E415))</f>
         <v/>
       </c>
       <c r="G415" s="5"/>
@@ -6330,7 +6331,7 @@
       <c r="D416" s="4"/>
       <c r="E416" s="4"/>
       <c r="F416" s="20" t="str">
-        <f aca="false">IF(AND(D416="",E416=""),"",'Start Here'!$B$4+SUM($D$5:D416)-SUM($E$5:E416))</f>
+        <f aca="false">IF(AND(D416="",E416=""),"",'Start Here'!$B$4+SUM($D$5:D416)+SUM($E$5:E416))</f>
         <v/>
       </c>
       <c r="G416" s="5"/>
@@ -6342,7 +6343,7 @@
       <c r="D417" s="4"/>
       <c r="E417" s="4"/>
       <c r="F417" s="20" t="str">
-        <f aca="false">IF(AND(D417="",E417=""),"",'Start Here'!$B$4+SUM($D$5:D417)-SUM($E$5:E417))</f>
+        <f aca="false">IF(AND(D417="",E417=""),"",'Start Here'!$B$4+SUM($D$5:D417)+SUM($E$5:E417))</f>
         <v/>
       </c>
       <c r="G417" s="5"/>
@@ -6354,7 +6355,7 @@
       <c r="D418" s="4"/>
       <c r="E418" s="4"/>
       <c r="F418" s="20" t="str">
-        <f aca="false">IF(AND(D418="",E418=""),"",'Start Here'!$B$4+SUM($D$5:D418)-SUM($E$5:E418))</f>
+        <f aca="false">IF(AND(D418="",E418=""),"",'Start Here'!$B$4+SUM($D$5:D418)+SUM($E$5:E418))</f>
         <v/>
       </c>
       <c r="G418" s="5"/>
@@ -6366,7 +6367,7 @@
       <c r="D419" s="4"/>
       <c r="E419" s="4"/>
       <c r="F419" s="20" t="str">
-        <f aca="false">IF(AND(D419="",E419=""),"",'Start Here'!$B$4+SUM($D$5:D419)-SUM($E$5:E419))</f>
+        <f aca="false">IF(AND(D419="",E419=""),"",'Start Here'!$B$4+SUM($D$5:D419)+SUM($E$5:E419))</f>
         <v/>
       </c>
       <c r="G419" s="5"/>
@@ -6378,7 +6379,7 @@
       <c r="D420" s="4"/>
       <c r="E420" s="4"/>
       <c r="F420" s="20" t="str">
-        <f aca="false">IF(AND(D420="",E420=""),"",'Start Here'!$B$4+SUM($D$5:D420)-SUM($E$5:E420))</f>
+        <f aca="false">IF(AND(D420="",E420=""),"",'Start Here'!$B$4+SUM($D$5:D420)+SUM($E$5:E420))</f>
         <v/>
       </c>
       <c r="G420" s="5"/>
@@ -6390,7 +6391,7 @@
       <c r="D421" s="4"/>
       <c r="E421" s="4"/>
       <c r="F421" s="20" t="str">
-        <f aca="false">IF(AND(D421="",E421=""),"",'Start Here'!$B$4+SUM($D$5:D421)-SUM($E$5:E421))</f>
+        <f aca="false">IF(AND(D421="",E421=""),"",'Start Here'!$B$4+SUM($D$5:D421)+SUM($E$5:E421))</f>
         <v/>
       </c>
       <c r="G421" s="5"/>
@@ -6402,7 +6403,7 @@
       <c r="D422" s="4"/>
       <c r="E422" s="4"/>
       <c r="F422" s="20" t="str">
-        <f aca="false">IF(AND(D422="",E422=""),"",'Start Here'!$B$4+SUM($D$5:D422)-SUM($E$5:E422))</f>
+        <f aca="false">IF(AND(D422="",E422=""),"",'Start Here'!$B$4+SUM($D$5:D422)+SUM($E$5:E422))</f>
         <v/>
       </c>
       <c r="G422" s="5"/>
@@ -6414,7 +6415,7 @@
       <c r="D423" s="4"/>
       <c r="E423" s="4"/>
       <c r="F423" s="20" t="str">
-        <f aca="false">IF(AND(D423="",E423=""),"",'Start Here'!$B$4+SUM($D$5:D423)-SUM($E$5:E423))</f>
+        <f aca="false">IF(AND(D423="",E423=""),"",'Start Here'!$B$4+SUM($D$5:D423)+SUM($E$5:E423))</f>
         <v/>
       </c>
       <c r="G423" s="5"/>
@@ -6426,7 +6427,7 @@
       <c r="D424" s="4"/>
       <c r="E424" s="4"/>
       <c r="F424" s="20" t="str">
-        <f aca="false">IF(AND(D424="",E424=""),"",'Start Here'!$B$4+SUM($D$5:D424)-SUM($E$5:E424))</f>
+        <f aca="false">IF(AND(D424="",E424=""),"",'Start Here'!$B$4+SUM($D$5:D424)+SUM($E$5:E424))</f>
         <v/>
       </c>
       <c r="G424" s="5"/>
@@ -6438,7 +6439,7 @@
       <c r="D425" s="4"/>
       <c r="E425" s="4"/>
       <c r="F425" s="20" t="str">
-        <f aca="false">IF(AND(D425="",E425=""),"",'Start Here'!$B$4+SUM($D$5:D425)-SUM($E$5:E425))</f>
+        <f aca="false">IF(AND(D425="",E425=""),"",'Start Here'!$B$4+SUM($D$5:D425)+SUM($E$5:E425))</f>
         <v/>
       </c>
       <c r="G425" s="5"/>
@@ -6450,7 +6451,7 @@
       <c r="D426" s="4"/>
       <c r="E426" s="4"/>
       <c r="F426" s="20" t="str">
-        <f aca="false">IF(AND(D426="",E426=""),"",'Start Here'!$B$4+SUM($D$5:D426)-SUM($E$5:E426))</f>
+        <f aca="false">IF(AND(D426="",E426=""),"",'Start Here'!$B$4+SUM($D$5:D426)+SUM($E$5:E426))</f>
         <v/>
       </c>
       <c r="G426" s="5"/>
@@ -6462,7 +6463,7 @@
       <c r="D427" s="4"/>
       <c r="E427" s="4"/>
       <c r="F427" s="20" t="str">
-        <f aca="false">IF(AND(D427="",E427=""),"",'Start Here'!$B$4+SUM($D$5:D427)-SUM($E$5:E427))</f>
+        <f aca="false">IF(AND(D427="",E427=""),"",'Start Here'!$B$4+SUM($D$5:D427)+SUM($E$5:E427))</f>
         <v/>
       </c>
       <c r="G427" s="5"/>
@@ -6474,7 +6475,7 @@
       <c r="D428" s="4"/>
       <c r="E428" s="4"/>
       <c r="F428" s="20" t="str">
-        <f aca="false">IF(AND(D428="",E428=""),"",'Start Here'!$B$4+SUM($D$5:D428)-SUM($E$5:E428))</f>
+        <f aca="false">IF(AND(D428="",E428=""),"",'Start Here'!$B$4+SUM($D$5:D428)+SUM($E$5:E428))</f>
         <v/>
       </c>
       <c r="G428" s="5"/>
@@ -6486,7 +6487,7 @@
       <c r="D429" s="4"/>
       <c r="E429" s="4"/>
       <c r="F429" s="20" t="str">
-        <f aca="false">IF(AND(D429="",E429=""),"",'Start Here'!$B$4+SUM($D$5:D429)-SUM($E$5:E429))</f>
+        <f aca="false">IF(AND(D429="",E429=""),"",'Start Here'!$B$4+SUM($D$5:D429)+SUM($E$5:E429))</f>
         <v/>
       </c>
       <c r="G429" s="5"/>
@@ -6498,7 +6499,7 @@
       <c r="D430" s="4"/>
       <c r="E430" s="4"/>
       <c r="F430" s="20" t="str">
-        <f aca="false">IF(AND(D430="",E430=""),"",'Start Here'!$B$4+SUM($D$5:D430)-SUM($E$5:E430))</f>
+        <f aca="false">IF(AND(D430="",E430=""),"",'Start Here'!$B$4+SUM($D$5:D430)+SUM($E$5:E430))</f>
         <v/>
       </c>
       <c r="G430" s="5"/>
@@ -6510,7 +6511,7 @@
       <c r="D431" s="4"/>
       <c r="E431" s="4"/>
       <c r="F431" s="20" t="str">
-        <f aca="false">IF(AND(D431="",E431=""),"",'Start Here'!$B$4+SUM($D$5:D431)-SUM($E$5:E431))</f>
+        <f aca="false">IF(AND(D431="",E431=""),"",'Start Here'!$B$4+SUM($D$5:D431)+SUM($E$5:E431))</f>
         <v/>
       </c>
       <c r="G431" s="5"/>
@@ -6522,7 +6523,7 @@
       <c r="D432" s="4"/>
       <c r="E432" s="4"/>
       <c r="F432" s="20" t="str">
-        <f aca="false">IF(AND(D432="",E432=""),"",'Start Here'!$B$4+SUM($D$5:D432)-SUM($E$5:E432))</f>
+        <f aca="false">IF(AND(D432="",E432=""),"",'Start Here'!$B$4+SUM($D$5:D432)+SUM($E$5:E432))</f>
         <v/>
       </c>
       <c r="G432" s="5"/>
@@ -6534,7 +6535,7 @@
       <c r="D433" s="4"/>
       <c r="E433" s="4"/>
       <c r="F433" s="20" t="str">
-        <f aca="false">IF(AND(D433="",E433=""),"",'Start Here'!$B$4+SUM($D$5:D433)-SUM($E$5:E433))</f>
+        <f aca="false">IF(AND(D433="",E433=""),"",'Start Here'!$B$4+SUM($D$5:D433)+SUM($E$5:E433))</f>
         <v/>
       </c>
       <c r="G433" s="5"/>
@@ -6546,7 +6547,7 @@
       <c r="D434" s="4"/>
       <c r="E434" s="4"/>
       <c r="F434" s="20" t="str">
-        <f aca="false">IF(AND(D434="",E434=""),"",'Start Here'!$B$4+SUM($D$5:D434)-SUM($E$5:E434))</f>
+        <f aca="false">IF(AND(D434="",E434=""),"",'Start Here'!$B$4+SUM($D$5:D434)+SUM($E$5:E434))</f>
         <v/>
       </c>
       <c r="G434" s="5"/>
@@ -6558,7 +6559,7 @@
       <c r="D435" s="4"/>
       <c r="E435" s="4"/>
       <c r="F435" s="20" t="str">
-        <f aca="false">IF(AND(D435="",E435=""),"",'Start Here'!$B$4+SUM($D$5:D435)-SUM($E$5:E435))</f>
+        <f aca="false">IF(AND(D435="",E435=""),"",'Start Here'!$B$4+SUM($D$5:D435)+SUM($E$5:E435))</f>
         <v/>
       </c>
       <c r="G435" s="5"/>
@@ -6570,7 +6571,7 @@
       <c r="D436" s="4"/>
       <c r="E436" s="4"/>
       <c r="F436" s="20" t="str">
-        <f aca="false">IF(AND(D436="",E436=""),"",'Start Here'!$B$4+SUM($D$5:D436)-SUM($E$5:E436))</f>
+        <f aca="false">IF(AND(D436="",E436=""),"",'Start Here'!$B$4+SUM($D$5:D436)+SUM($E$5:E436))</f>
         <v/>
       </c>
       <c r="G436" s="5"/>
@@ -6582,7 +6583,7 @@
       <c r="D437" s="4"/>
       <c r="E437" s="4"/>
       <c r="F437" s="20" t="str">
-        <f aca="false">IF(AND(D437="",E437=""),"",'Start Here'!$B$4+SUM($D$5:D437)-SUM($E$5:E437))</f>
+        <f aca="false">IF(AND(D437="",E437=""),"",'Start Here'!$B$4+SUM($D$5:D437)+SUM($E$5:E437))</f>
         <v/>
       </c>
       <c r="G437" s="5"/>
@@ -6594,7 +6595,7 @@
       <c r="D438" s="4"/>
       <c r="E438" s="4"/>
       <c r="F438" s="20" t="str">
-        <f aca="false">IF(AND(D438="",E438=""),"",'Start Here'!$B$4+SUM($D$5:D438)-SUM($E$5:E438))</f>
+        <f aca="false">IF(AND(D438="",E438=""),"",'Start Here'!$B$4+SUM($D$5:D438)+SUM($E$5:E438))</f>
         <v/>
       </c>
       <c r="G438" s="5"/>
@@ -6606,7 +6607,7 @@
       <c r="D439" s="4"/>
       <c r="E439" s="4"/>
       <c r="F439" s="20" t="str">
-        <f aca="false">IF(AND(D439="",E439=""),"",'Start Here'!$B$4+SUM($D$5:D439)-SUM($E$5:E439))</f>
+        <f aca="false">IF(AND(D439="",E439=""),"",'Start Here'!$B$4+SUM($D$5:D439)+SUM($E$5:E439))</f>
         <v/>
       </c>
       <c r="G439" s="5"/>
@@ -6618,7 +6619,7 @@
       <c r="D440" s="4"/>
       <c r="E440" s="4"/>
       <c r="F440" s="20" t="str">
-        <f aca="false">IF(AND(D440="",E440=""),"",'Start Here'!$B$4+SUM($D$5:D440)-SUM($E$5:E440))</f>
+        <f aca="false">IF(AND(D440="",E440=""),"",'Start Here'!$B$4+SUM($D$5:D440)+SUM($E$5:E440))</f>
         <v/>
       </c>
       <c r="G440" s="5"/>
@@ -6630,7 +6631,7 @@
       <c r="D441" s="4"/>
       <c r="E441" s="4"/>
       <c r="F441" s="20" t="str">
-        <f aca="false">IF(AND(D441="",E441=""),"",'Start Here'!$B$4+SUM($D$5:D441)-SUM($E$5:E441))</f>
+        <f aca="false">IF(AND(D441="",E441=""),"",'Start Here'!$B$4+SUM($D$5:D441)+SUM($E$5:E441))</f>
         <v/>
       </c>
       <c r="G441" s="5"/>
@@ -6642,7 +6643,7 @@
       <c r="D442" s="4"/>
       <c r="E442" s="4"/>
       <c r="F442" s="20" t="str">
-        <f aca="false">IF(AND(D442="",E442=""),"",'Start Here'!$B$4+SUM($D$5:D442)-SUM($E$5:E442))</f>
+        <f aca="false">IF(AND(D442="",E442=""),"",'Start Here'!$B$4+SUM($D$5:D442)+SUM($E$5:E442))</f>
         <v/>
       </c>
       <c r="G442" s="5"/>
@@ -6654,7 +6655,7 @@
       <c r="D443" s="4"/>
       <c r="E443" s="4"/>
       <c r="F443" s="20" t="str">
-        <f aca="false">IF(AND(D443="",E443=""),"",'Start Here'!$B$4+SUM($D$5:D443)-SUM($E$5:E443))</f>
+        <f aca="false">IF(AND(D443="",E443=""),"",'Start Here'!$B$4+SUM($D$5:D443)+SUM($E$5:E443))</f>
         <v/>
       </c>
       <c r="G443" s="5"/>
@@ -6666,7 +6667,7 @@
       <c r="D444" s="4"/>
       <c r="E444" s="4"/>
       <c r="F444" s="20" t="str">
-        <f aca="false">IF(AND(D444="",E444=""),"",'Start Here'!$B$4+SUM($D$5:D444)-SUM($E$5:E444))</f>
+        <f aca="false">IF(AND(D444="",E444=""),"",'Start Here'!$B$4+SUM($D$5:D444)+SUM($E$5:E444))</f>
         <v/>
       </c>
       <c r="G444" s="5"/>
@@ -6678,7 +6679,7 @@
       <c r="D445" s="4"/>
       <c r="E445" s="4"/>
       <c r="F445" s="20" t="str">
-        <f aca="false">IF(AND(D445="",E445=""),"",'Start Here'!$B$4+SUM($D$5:D445)-SUM($E$5:E445))</f>
+        <f aca="false">IF(AND(D445="",E445=""),"",'Start Here'!$B$4+SUM($D$5:D445)+SUM($E$5:E445))</f>
         <v/>
       </c>
       <c r="G445" s="5"/>
@@ -6690,7 +6691,7 @@
       <c r="D446" s="4"/>
       <c r="E446" s="4"/>
       <c r="F446" s="20" t="str">
-        <f aca="false">IF(AND(D446="",E446=""),"",'Start Here'!$B$4+SUM($D$5:D446)-SUM($E$5:E446))</f>
+        <f aca="false">IF(AND(D446="",E446=""),"",'Start Here'!$B$4+SUM($D$5:D446)+SUM($E$5:E446))</f>
         <v/>
       </c>
       <c r="G446" s="5"/>
@@ -6702,7 +6703,7 @@
       <c r="D447" s="4"/>
       <c r="E447" s="4"/>
       <c r="F447" s="20" t="str">
-        <f aca="false">IF(AND(D447="",E447=""),"",'Start Here'!$B$4+SUM($D$5:D447)-SUM($E$5:E447))</f>
+        <f aca="false">IF(AND(D447="",E447=""),"",'Start Here'!$B$4+SUM($D$5:D447)+SUM($E$5:E447))</f>
         <v/>
       </c>
       <c r="G447" s="5"/>
@@ -6714,7 +6715,7 @@
       <c r="D448" s="4"/>
       <c r="E448" s="4"/>
       <c r="F448" s="20" t="str">
-        <f aca="false">IF(AND(D448="",E448=""),"",'Start Here'!$B$4+SUM($D$5:D448)-SUM($E$5:E448))</f>
+        <f aca="false">IF(AND(D448="",E448=""),"",'Start Here'!$B$4+SUM($D$5:D448)+SUM($E$5:E448))</f>
         <v/>
       </c>
       <c r="G448" s="5"/>
@@ -6726,7 +6727,7 @@
       <c r="D449" s="4"/>
       <c r="E449" s="4"/>
       <c r="F449" s="20" t="str">
-        <f aca="false">IF(AND(D449="",E449=""),"",'Start Here'!$B$4+SUM($D$5:D449)-SUM($E$5:E449))</f>
+        <f aca="false">IF(AND(D449="",E449=""),"",'Start Here'!$B$4+SUM($D$5:D449)+SUM($E$5:E449))</f>
         <v/>
       </c>
       <c r="G449" s="5"/>
@@ -6738,7 +6739,7 @@
       <c r="D450" s="4"/>
       <c r="E450" s="4"/>
       <c r="F450" s="20" t="str">
-        <f aca="false">IF(AND(D450="",E450=""),"",'Start Here'!$B$4+SUM($D$5:D450)-SUM($E$5:E450))</f>
+        <f aca="false">IF(AND(D450="",E450=""),"",'Start Here'!$B$4+SUM($D$5:D450)+SUM($E$5:E450))</f>
         <v/>
       </c>
       <c r="G450" s="5"/>
@@ -6750,7 +6751,7 @@
       <c r="D451" s="4"/>
       <c r="E451" s="4"/>
       <c r="F451" s="20" t="str">
-        <f aca="false">IF(AND(D451="",E451=""),"",'Start Here'!$B$4+SUM($D$5:D451)-SUM($E$5:E451))</f>
+        <f aca="false">IF(AND(D451="",E451=""),"",'Start Here'!$B$4+SUM($D$5:D451)+SUM($E$5:E451))</f>
         <v/>
       </c>
       <c r="G451" s="5"/>
@@ -6762,7 +6763,7 @@
       <c r="D452" s="4"/>
       <c r="E452" s="4"/>
       <c r="F452" s="20" t="str">
-        <f aca="false">IF(AND(D452="",E452=""),"",'Start Here'!$B$4+SUM($D$5:D452)-SUM($E$5:E452))</f>
+        <f aca="false">IF(AND(D452="",E452=""),"",'Start Here'!$B$4+SUM($D$5:D452)+SUM($E$5:E452))</f>
         <v/>
       </c>
       <c r="G452" s="5"/>
@@ -6774,7 +6775,7 @@
       <c r="D453" s="4"/>
       <c r="E453" s="4"/>
       <c r="F453" s="20" t="str">
-        <f aca="false">IF(AND(D453="",E453=""),"",'Start Here'!$B$4+SUM($D$5:D453)-SUM($E$5:E453))</f>
+        <f aca="false">IF(AND(D453="",E453=""),"",'Start Here'!$B$4+SUM($D$5:D453)+SUM($E$5:E453))</f>
         <v/>
       </c>
       <c r="G453" s="5"/>
@@ -6786,7 +6787,7 @@
       <c r="D454" s="4"/>
       <c r="E454" s="4"/>
       <c r="F454" s="20" t="str">
-        <f aca="false">IF(AND(D454="",E454=""),"",'Start Here'!$B$4+SUM($D$5:D454)-SUM($E$5:E454))</f>
+        <f aca="false">IF(AND(D454="",E454=""),"",'Start Here'!$B$4+SUM($D$5:D454)+SUM($E$5:E454))</f>
         <v/>
       </c>
       <c r="G454" s="5"/>
@@ -6798,7 +6799,7 @@
       <c r="D455" s="4"/>
       <c r="E455" s="4"/>
       <c r="F455" s="20" t="str">
-        <f aca="false">IF(AND(D455="",E455=""),"",'Start Here'!$B$4+SUM($D$5:D455)-SUM($E$5:E455))</f>
+        <f aca="false">IF(AND(D455="",E455=""),"",'Start Here'!$B$4+SUM($D$5:D455)+SUM($E$5:E455))</f>
         <v/>
       </c>
       <c r="G455" s="5"/>
@@ -6810,7 +6811,7 @@
       <c r="D456" s="4"/>
       <c r="E456" s="4"/>
       <c r="F456" s="20" t="str">
-        <f aca="false">IF(AND(D456="",E456=""),"",'Start Here'!$B$4+SUM($D$5:D456)-SUM($E$5:E456))</f>
+        <f aca="false">IF(AND(D456="",E456=""),"",'Start Here'!$B$4+SUM($D$5:D456)+SUM($E$5:E456))</f>
         <v/>
       </c>
       <c r="G456" s="5"/>
@@ -6822,7 +6823,7 @@
       <c r="D457" s="4"/>
       <c r="E457" s="4"/>
       <c r="F457" s="20" t="str">
-        <f aca="false">IF(AND(D457="",E457=""),"",'Start Here'!$B$4+SUM($D$5:D457)-SUM($E$5:E457))</f>
+        <f aca="false">IF(AND(D457="",E457=""),"",'Start Here'!$B$4+SUM($D$5:D457)+SUM($E$5:E457))</f>
         <v/>
       </c>
       <c r="G457" s="5"/>
@@ -6834,7 +6835,7 @@
       <c r="D458" s="4"/>
       <c r="E458" s="4"/>
       <c r="F458" s="20" t="str">
-        <f aca="false">IF(AND(D458="",E458=""),"",'Start Here'!$B$4+SUM($D$5:D458)-SUM($E$5:E458))</f>
+        <f aca="false">IF(AND(D458="",E458=""),"",'Start Here'!$B$4+SUM($D$5:D458)+SUM($E$5:E458))</f>
         <v/>
       </c>
       <c r="G458" s="5"/>
@@ -6846,7 +6847,7 @@
       <c r="D459" s="4"/>
       <c r="E459" s="4"/>
       <c r="F459" s="20" t="str">
-        <f aca="false">IF(AND(D459="",E459=""),"",'Start Here'!$B$4+SUM($D$5:D459)-SUM($E$5:E459))</f>
+        <f aca="false">IF(AND(D459="",E459=""),"",'Start Here'!$B$4+SUM($D$5:D459)+SUM($E$5:E459))</f>
         <v/>
       </c>
       <c r="G459" s="5"/>
@@ -6858,7 +6859,7 @@
       <c r="D460" s="4"/>
       <c r="E460" s="4"/>
       <c r="F460" s="20" t="str">
-        <f aca="false">IF(AND(D460="",E460=""),"",'Start Here'!$B$4+SUM($D$5:D460)-SUM($E$5:E460))</f>
+        <f aca="false">IF(AND(D460="",E460=""),"",'Start Here'!$B$4+SUM($D$5:D460)+SUM($E$5:E460))</f>
         <v/>
       </c>
       <c r="G460" s="5"/>
@@ -6870,7 +6871,7 @@
       <c r="D461" s="4"/>
       <c r="E461" s="4"/>
       <c r="F461" s="20" t="str">
-        <f aca="false">IF(AND(D461="",E461=""),"",'Start Here'!$B$4+SUM($D$5:D461)-SUM($E$5:E461))</f>
+        <f aca="false">IF(AND(D461="",E461=""),"",'Start Here'!$B$4+SUM($D$5:D461)+SUM($E$5:E461))</f>
         <v/>
       </c>
       <c r="G461" s="5"/>
@@ -6882,7 +6883,7 @@
       <c r="D462" s="4"/>
       <c r="E462" s="4"/>
       <c r="F462" s="20" t="str">
-        <f aca="false">IF(AND(D462="",E462=""),"",'Start Here'!$B$4+SUM($D$5:D462)-SUM($E$5:E462))</f>
+        <f aca="false">IF(AND(D462="",E462=""),"",'Start Here'!$B$4+SUM($D$5:D462)+SUM($E$5:E462))</f>
         <v/>
       </c>
       <c r="G462" s="5"/>
@@ -6894,7 +6895,7 @@
       <c r="D463" s="4"/>
       <c r="E463" s="4"/>
       <c r="F463" s="20" t="str">
-        <f aca="false">IF(AND(D463="",E463=""),"",'Start Here'!$B$4+SUM($D$5:D463)-SUM($E$5:E463))</f>
+        <f aca="false">IF(AND(D463="",E463=""),"",'Start Here'!$B$4+SUM($D$5:D463)+SUM($E$5:E463))</f>
         <v/>
       </c>
       <c r="G463" s="5"/>
@@ -6906,7 +6907,7 @@
       <c r="D464" s="4"/>
       <c r="E464" s="4"/>
       <c r="F464" s="20" t="str">
-        <f aca="false">IF(AND(D464="",E464=""),"",'Start Here'!$B$4+SUM($D$5:D464)-SUM($E$5:E464))</f>
+        <f aca="false">IF(AND(D464="",E464=""),"",'Start Here'!$B$4+SUM($D$5:D464)+SUM($E$5:E464))</f>
         <v/>
       </c>
       <c r="G464" s="5"/>
@@ -6918,7 +6919,7 @@
       <c r="D465" s="4"/>
       <c r="E465" s="4"/>
       <c r="F465" s="20" t="str">
-        <f aca="false">IF(AND(D465="",E465=""),"",'Start Here'!$B$4+SUM($D$5:D465)-SUM($E$5:E465))</f>
+        <f aca="false">IF(AND(D465="",E465=""),"",'Start Here'!$B$4+SUM($D$5:D465)+SUM($E$5:E465))</f>
         <v/>
       </c>
       <c r="G465" s="5"/>
@@ -6930,7 +6931,7 @@
       <c r="D466" s="4"/>
       <c r="E466" s="4"/>
       <c r="F466" s="20" t="str">
-        <f aca="false">IF(AND(D466="",E466=""),"",'Start Here'!$B$4+SUM($D$5:D466)-SUM($E$5:E466))</f>
+        <f aca="false">IF(AND(D466="",E466=""),"",'Start Here'!$B$4+SUM($D$5:D466)+SUM($E$5:E466))</f>
         <v/>
       </c>
       <c r="G466" s="5"/>
@@ -6942,7 +6943,7 @@
       <c r="D467" s="4"/>
       <c r="E467" s="4"/>
       <c r="F467" s="20" t="str">
-        <f aca="false">IF(AND(D467="",E467=""),"",'Start Here'!$B$4+SUM($D$5:D467)-SUM($E$5:E467))</f>
+        <f aca="false">IF(AND(D467="",E467=""),"",'Start Here'!$B$4+SUM($D$5:D467)+SUM($E$5:E467))</f>
         <v/>
       </c>
       <c r="G467" s="5"/>
@@ -6954,7 +6955,7 @@
       <c r="D468" s="4"/>
       <c r="E468" s="4"/>
       <c r="F468" s="20" t="str">
-        <f aca="false">IF(AND(D468="",E468=""),"",'Start Here'!$B$4+SUM($D$5:D468)-SUM($E$5:E468))</f>
+        <f aca="false">IF(AND(D468="",E468=""),"",'Start Here'!$B$4+SUM($D$5:D468)+SUM($E$5:E468))</f>
         <v/>
       </c>
       <c r="G468" s="5"/>
@@ -6966,7 +6967,7 @@
       <c r="D469" s="4"/>
       <c r="E469" s="4"/>
       <c r="F469" s="20" t="str">
-        <f aca="false">IF(AND(D469="",E469=""),"",'Start Here'!$B$4+SUM($D$5:D469)-SUM($E$5:E469))</f>
+        <f aca="false">IF(AND(D469="",E469=""),"",'Start Here'!$B$4+SUM($D$5:D469)+SUM($E$5:E469))</f>
         <v/>
       </c>
       <c r="G469" s="5"/>
@@ -6978,7 +6979,7 @@
       <c r="D470" s="4"/>
       <c r="E470" s="4"/>
       <c r="F470" s="20" t="str">
-        <f aca="false">IF(AND(D470="",E470=""),"",'Start Here'!$B$4+SUM($D$5:D470)-SUM($E$5:E470))</f>
+        <f aca="false">IF(AND(D470="",E470=""),"",'Start Here'!$B$4+SUM($D$5:D470)+SUM($E$5:E470))</f>
         <v/>
       </c>
       <c r="G470" s="5"/>
@@ -6990,7 +6991,7 @@
       <c r="D471" s="4"/>
       <c r="E471" s="4"/>
       <c r="F471" s="20" t="str">
-        <f aca="false">IF(AND(D471="",E471=""),"",'Start Here'!$B$4+SUM($D$5:D471)-SUM($E$5:E471))</f>
+        <f aca="false">IF(AND(D471="",E471=""),"",'Start Here'!$B$4+SUM($D$5:D471)+SUM($E$5:E471))</f>
         <v/>
       </c>
       <c r="G471" s="5"/>
@@ -7002,7 +7003,7 @@
       <c r="D472" s="4"/>
       <c r="E472" s="4"/>
       <c r="F472" s="20" t="str">
-        <f aca="false">IF(AND(D472="",E472=""),"",'Start Here'!$B$4+SUM($D$5:D472)-SUM($E$5:E472))</f>
+        <f aca="false">IF(AND(D472="",E472=""),"",'Start Here'!$B$4+SUM($D$5:D472)+SUM($E$5:E472))</f>
         <v/>
       </c>
       <c r="G472" s="5"/>
@@ -7014,7 +7015,7 @@
       <c r="D473" s="4"/>
       <c r="E473" s="4"/>
       <c r="F473" s="20" t="str">
-        <f aca="false">IF(AND(D473="",E473=""),"",'Start Here'!$B$4+SUM($D$5:D473)-SUM($E$5:E473))</f>
+        <f aca="false">IF(AND(D473="",E473=""),"",'Start Here'!$B$4+SUM($D$5:D473)+SUM($E$5:E473))</f>
         <v/>
       </c>
       <c r="G473" s="5"/>
@@ -7026,7 +7027,7 @@
       <c r="D474" s="4"/>
       <c r="E474" s="4"/>
       <c r="F474" s="20" t="str">
-        <f aca="false">IF(AND(D474="",E474=""),"",'Start Here'!$B$4+SUM($D$5:D474)-SUM($E$5:E474))</f>
+        <f aca="false">IF(AND(D474="",E474=""),"",'Start Here'!$B$4+SUM($D$5:D474)+SUM($E$5:E474))</f>
         <v/>
       </c>
       <c r="G474" s="5"/>
@@ -7038,7 +7039,7 @@
       <c r="D475" s="4"/>
       <c r="E475" s="4"/>
       <c r="F475" s="20" t="str">
-        <f aca="false">IF(AND(D475="",E475=""),"",'Start Here'!$B$4+SUM($D$5:D475)-SUM($E$5:E475))</f>
+        <f aca="false">IF(AND(D475="",E475=""),"",'Start Here'!$B$4+SUM($D$5:D475)+SUM($E$5:E475))</f>
         <v/>
       </c>
       <c r="G475" s="5"/>
@@ -7050,7 +7051,7 @@
       <c r="D476" s="4"/>
       <c r="E476" s="4"/>
       <c r="F476" s="20" t="str">
-        <f aca="false">IF(AND(D476="",E476=""),"",'Start Here'!$B$4+SUM($D$5:D476)-SUM($E$5:E476))</f>
+        <f aca="false">IF(AND(D476="",E476=""),"",'Start Here'!$B$4+SUM($D$5:D476)+SUM($E$5:E476))</f>
         <v/>
       </c>
       <c r="G476" s="5"/>
@@ -7062,7 +7063,7 @@
       <c r="D477" s="4"/>
       <c r="E477" s="4"/>
       <c r="F477" s="20" t="str">
-        <f aca="false">IF(AND(D477="",E477=""),"",'Start Here'!$B$4+SUM($D$5:D477)-SUM($E$5:E477))</f>
+        <f aca="false">IF(AND(D477="",E477=""),"",'Start Here'!$B$4+SUM($D$5:D477)+SUM($E$5:E477))</f>
         <v/>
       </c>
       <c r="G477" s="5"/>
@@ -7074,7 +7075,7 @@
       <c r="D478" s="4"/>
       <c r="E478" s="4"/>
       <c r="F478" s="20" t="str">
-        <f aca="false">IF(AND(D478="",E478=""),"",'Start Here'!$B$4+SUM($D$5:D478)-SUM($E$5:E478))</f>
+        <f aca="false">IF(AND(D478="",E478=""),"",'Start Here'!$B$4+SUM($D$5:D478)+SUM($E$5:E478))</f>
         <v/>
       </c>
       <c r="G478" s="5"/>
@@ -7086,7 +7087,7 @@
       <c r="D479" s="4"/>
       <c r="E479" s="4"/>
       <c r="F479" s="20" t="str">
-        <f aca="false">IF(AND(D479="",E479=""),"",'Start Here'!$B$4+SUM($D$5:D479)-SUM($E$5:E479))</f>
+        <f aca="false">IF(AND(D479="",E479=""),"",'Start Here'!$B$4+SUM($D$5:D479)+SUM($E$5:E479))</f>
         <v/>
       </c>
       <c r="G479" s="5"/>
@@ -7098,7 +7099,7 @@
       <c r="D480" s="4"/>
       <c r="E480" s="4"/>
       <c r="F480" s="20" t="str">
-        <f aca="false">IF(AND(D480="",E480=""),"",'Start Here'!$B$4+SUM($D$5:D480)-SUM($E$5:E480))</f>
+        <f aca="false">IF(AND(D480="",E480=""),"",'Start Here'!$B$4+SUM($D$5:D480)+SUM($E$5:E480))</f>
         <v/>
       </c>
       <c r="G480" s="5"/>
@@ -7110,7 +7111,7 @@
       <c r="D481" s="4"/>
       <c r="E481" s="4"/>
       <c r="F481" s="20" t="str">
-        <f aca="false">IF(AND(D481="",E481=""),"",'Start Here'!$B$4+SUM($D$5:D481)-SUM($E$5:E481))</f>
+        <f aca="false">IF(AND(D481="",E481=""),"",'Start Here'!$B$4+SUM($D$5:D481)+SUM($E$5:E481))</f>
         <v/>
       </c>
       <c r="G481" s="5"/>
@@ -7122,7 +7123,7 @@
       <c r="D482" s="4"/>
       <c r="E482" s="4"/>
       <c r="F482" s="20" t="str">
-        <f aca="false">IF(AND(D482="",E482=""),"",'Start Here'!$B$4+SUM($D$5:D482)-SUM($E$5:E482))</f>
+        <f aca="false">IF(AND(D482="",E482=""),"",'Start Here'!$B$4+SUM($D$5:D482)+SUM($E$5:E482))</f>
         <v/>
       </c>
       <c r="G482" s="5"/>
@@ -7134,7 +7135,7 @@
       <c r="D483" s="4"/>
       <c r="E483" s="4"/>
       <c r="F483" s="20" t="str">
-        <f aca="false">IF(AND(D483="",E483=""),"",'Start Here'!$B$4+SUM($D$5:D483)-SUM($E$5:E483))</f>
+        <f aca="false">IF(AND(D483="",E483=""),"",'Start Here'!$B$4+SUM($D$5:D483)+SUM($E$5:E483))</f>
         <v/>
       </c>
       <c r="G483" s="5"/>
@@ -7146,7 +7147,7 @@
       <c r="D484" s="4"/>
       <c r="E484" s="4"/>
       <c r="F484" s="20" t="str">
-        <f aca="false">IF(AND(D484="",E484=""),"",'Start Here'!$B$4+SUM($D$5:D484)-SUM($E$5:E484))</f>
+        <f aca="false">IF(AND(D484="",E484=""),"",'Start Here'!$B$4+SUM($D$5:D484)+SUM($E$5:E484))</f>
         <v/>
       </c>
       <c r="G484" s="5"/>
@@ -7158,7 +7159,7 @@
       <c r="D485" s="4"/>
       <c r="E485" s="4"/>
       <c r="F485" s="20" t="str">
-        <f aca="false">IF(AND(D485="",E485=""),"",'Start Here'!$B$4+SUM($D$5:D485)-SUM($E$5:E485))</f>
+        <f aca="false">IF(AND(D485="",E485=""),"",'Start Here'!$B$4+SUM($D$5:D485)+SUM($E$5:E485))</f>
         <v/>
       </c>
       <c r="G485" s="5"/>
@@ -7170,7 +7171,7 @@
       <c r="D486" s="4"/>
       <c r="E486" s="4"/>
       <c r="F486" s="20" t="str">
-        <f aca="false">IF(AND(D486="",E486=""),"",'Start Here'!$B$4+SUM($D$5:D486)-SUM($E$5:E486))</f>
+        <f aca="false">IF(AND(D486="",E486=""),"",'Start Here'!$B$4+SUM($D$5:D486)+SUM($E$5:E486))</f>
         <v/>
       </c>
       <c r="G486" s="5"/>
@@ -7182,7 +7183,7 @@
       <c r="D487" s="4"/>
       <c r="E487" s="4"/>
       <c r="F487" s="20" t="str">
-        <f aca="false">IF(AND(D487="",E487=""),"",'Start Here'!$B$4+SUM($D$5:D487)-SUM($E$5:E487))</f>
+        <f aca="false">IF(AND(D487="",E487=""),"",'Start Here'!$B$4+SUM($D$5:D487)+SUM($E$5:E487))</f>
         <v/>
       </c>
       <c r="G487" s="5"/>
@@ -7194,7 +7195,7 @@
       <c r="D488" s="4"/>
       <c r="E488" s="4"/>
       <c r="F488" s="20" t="str">
-        <f aca="false">IF(AND(D488="",E488=""),"",'Start Here'!$B$4+SUM($D$5:D488)-SUM($E$5:E488))</f>
+        <f aca="false">IF(AND(D488="",E488=""),"",'Start Here'!$B$4+SUM($D$5:D488)+SUM($E$5:E488))</f>
         <v/>
       </c>
       <c r="G488" s="5"/>
@@ -7206,7 +7207,7 @@
       <c r="D489" s="4"/>
       <c r="E489" s="4"/>
       <c r="F489" s="20" t="str">
-        <f aca="false">IF(AND(D489="",E489=""),"",'Start Here'!$B$4+SUM($D$5:D489)-SUM($E$5:E489))</f>
+        <f aca="false">IF(AND(D489="",E489=""),"",'Start Here'!$B$4+SUM($D$5:D489)+SUM($E$5:E489))</f>
         <v/>
       </c>
       <c r="G489" s="5"/>
@@ -7218,7 +7219,7 @@
       <c r="D490" s="4"/>
       <c r="E490" s="4"/>
       <c r="F490" s="20" t="str">
-        <f aca="false">IF(AND(D490="",E490=""),"",'Start Here'!$B$4+SUM($D$5:D490)-SUM($E$5:E490))</f>
+        <f aca="false">IF(AND(D490="",E490=""),"",'Start Here'!$B$4+SUM($D$5:D490)+SUM($E$5:E490))</f>
         <v/>
       </c>
       <c r="G490" s="5"/>
@@ -7230,7 +7231,7 @@
       <c r="D491" s="4"/>
       <c r="E491" s="4"/>
       <c r="F491" s="20" t="str">
-        <f aca="false">IF(AND(D491="",E491=""),"",'Start Here'!$B$4+SUM($D$5:D491)-SUM($E$5:E491))</f>
+        <f aca="false">IF(AND(D491="",E491=""),"",'Start Here'!$B$4+SUM($D$5:D491)+SUM($E$5:E491))</f>
         <v/>
       </c>
       <c r="G491" s="5"/>
@@ -7242,7 +7243,7 @@
       <c r="D492" s="4"/>
       <c r="E492" s="4"/>
       <c r="F492" s="20" t="str">
-        <f aca="false">IF(AND(D492="",E492=""),"",'Start Here'!$B$4+SUM($D$5:D492)-SUM($E$5:E492))</f>
+        <f aca="false">IF(AND(D492="",E492=""),"",'Start Here'!$B$4+SUM($D$5:D492)+SUM($E$5:E492))</f>
         <v/>
       </c>
       <c r="G492" s="5"/>
@@ -7254,7 +7255,7 @@
       <c r="D493" s="4"/>
       <c r="E493" s="4"/>
       <c r="F493" s="20" t="str">
-        <f aca="false">IF(AND(D493="",E493=""),"",'Start Here'!$B$4+SUM($D$5:D493)-SUM($E$5:E493))</f>
+        <f aca="false">IF(AND(D493="",E493=""),"",'Start Here'!$B$4+SUM($D$5:D493)+SUM($E$5:E493))</f>
         <v/>
       </c>
       <c r="G493" s="5"/>
@@ -7266,7 +7267,7 @@
       <c r="D494" s="4"/>
       <c r="E494" s="4"/>
       <c r="F494" s="20" t="str">
-        <f aca="false">IF(AND(D494="",E494=""),"",'Start Here'!$B$4+SUM($D$5:D494)-SUM($E$5:E494))</f>
+        <f aca="false">IF(AND(D494="",E494=""),"",'Start Here'!$B$4+SUM($D$5:D494)+SUM($E$5:E494))</f>
         <v/>
       </c>
       <c r="G494" s="5"/>
@@ -7278,7 +7279,7 @@
       <c r="D495" s="4"/>
       <c r="E495" s="4"/>
       <c r="F495" s="20" t="str">
-        <f aca="false">IF(AND(D495="",E495=""),"",'Start Here'!$B$4+SUM($D$5:D495)-SUM($E$5:E495))</f>
+        <f aca="false">IF(AND(D495="",E495=""),"",'Start Here'!$B$4+SUM($D$5:D495)+SUM($E$5:E495))</f>
         <v/>
       </c>
       <c r="G495" s="5"/>
@@ -7290,7 +7291,7 @@
       <c r="D496" s="4"/>
       <c r="E496" s="4"/>
       <c r="F496" s="20" t="str">
-        <f aca="false">IF(AND(D496="",E496=""),"",'Start Here'!$B$4+SUM($D$5:D496)-SUM($E$5:E496))</f>
+        <f aca="false">IF(AND(D496="",E496=""),"",'Start Here'!$B$4+SUM($D$5:D496)+SUM($E$5:E496))</f>
         <v/>
       </c>
       <c r="G496" s="5"/>
@@ -7302,7 +7303,7 @@
       <c r="D497" s="4"/>
       <c r="E497" s="4"/>
       <c r="F497" s="20" t="str">
-        <f aca="false">IF(AND(D497="",E497=""),"",'Start Here'!$B$4+SUM($D$5:D497)-SUM($E$5:E497))</f>
+        <f aca="false">IF(AND(D497="",E497=""),"",'Start Here'!$B$4+SUM($D$5:D497)+SUM($E$5:E497))</f>
         <v/>
       </c>
       <c r="G497" s="5"/>
@@ -7314,7 +7315,7 @@
       <c r="D498" s="4"/>
       <c r="E498" s="4"/>
       <c r="F498" s="20" t="str">
-        <f aca="false">IF(AND(D498="",E498=""),"",'Start Here'!$B$4+SUM($D$5:D498)-SUM($E$5:E498))</f>
+        <f aca="false">IF(AND(D498="",E498=""),"",'Start Here'!$B$4+SUM($D$5:D498)+SUM($E$5:E498))</f>
         <v/>
       </c>
       <c r="G498" s="5"/>
@@ -7326,7 +7327,7 @@
       <c r="D499" s="4"/>
       <c r="E499" s="4"/>
       <c r="F499" s="20" t="str">
-        <f aca="false">IF(AND(D499="",E499=""),"",'Start Here'!$B$4+SUM($D$5:D499)-SUM($E$5:E499))</f>
+        <f aca="false">IF(AND(D499="",E499=""),"",'Start Here'!$B$4+SUM($D$5:D499)+SUM($E$5:E499))</f>
         <v/>
       </c>
       <c r="G499" s="5"/>
@@ -7338,7 +7339,7 @@
       <c r="D500" s="4"/>
       <c r="E500" s="4"/>
       <c r="F500" s="20" t="str">
-        <f aca="false">IF(AND(D500="",E500=""),"",'Start Here'!$B$4+SUM($D$5:D500)-SUM($E$5:E500))</f>
+        <f aca="false">IF(AND(D500="",E500=""),"",'Start Here'!$B$4+SUM($D$5:D500)+SUM($E$5:E500))</f>
         <v/>
       </c>
       <c r="G500" s="5"/>
@@ -7350,7 +7351,7 @@
       <c r="D501" s="4"/>
       <c r="E501" s="4"/>
       <c r="F501" s="20" t="str">
-        <f aca="false">IF(AND(D501="",E501=""),"",'Start Here'!$B$4+SUM($D$5:D501)-SUM($E$5:E501))</f>
+        <f aca="false">IF(AND(D501="",E501=""),"",'Start Here'!$B$4+SUM($D$5:D501)+SUM($E$5:E501))</f>
         <v/>
       </c>
       <c r="G501" s="5"/>
@@ -7362,7 +7363,7 @@
       <c r="D502" s="4"/>
       <c r="E502" s="4"/>
       <c r="F502" s="20" t="str">
-        <f aca="false">IF(AND(D502="",E502=""),"",'Start Here'!$B$4+SUM($D$5:D502)-SUM($E$5:E502))</f>
+        <f aca="false">IF(AND(D502="",E502=""),"",'Start Here'!$B$4+SUM($D$5:D502)+SUM($E$5:E502))</f>
         <v/>
       </c>
       <c r="G502" s="5"/>
@@ -7374,7 +7375,7 @@
       <c r="D503" s="4"/>
       <c r="E503" s="4"/>
       <c r="F503" s="20" t="str">
-        <f aca="false">IF(AND(D503="",E503=""),"",'Start Here'!$B$4+SUM($D$5:D503)-SUM($E$5:E503))</f>
+        <f aca="false">IF(AND(D503="",E503=""),"",'Start Here'!$B$4+SUM($D$5:D503)+SUM($E$5:E503))</f>
         <v/>
       </c>
       <c r="G503" s="5"/>
@@ -7386,7 +7387,7 @@
       <c r="D504" s="4"/>
       <c r="E504" s="4"/>
       <c r="F504" s="20" t="str">
-        <f aca="false">IF(AND(D504="",E504=""),"",'Start Here'!$B$4+SUM($D$5:D504)-SUM($E$5:E504))</f>
+        <f aca="false">IF(AND(D504="",E504=""),"",'Start Here'!$B$4+SUM($D$5:D504)+SUM($E$5:E504))</f>
         <v/>
       </c>
       <c r="G504" s="5"/>
@@ -7397,12 +7398,16 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C504" type="list">
       <formula1>'Start Here'!$A$17:$A$33</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Enter a positive number" errorStyle="stop" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:E504" type="decimal">
+    <dataValidation allowBlank="true" error="Money In must be a positive number" errorStyle="stop" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D504" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Money Out must be a negative number, e.g. -200" errorStyle="stop" operator="lessThanOrEqual" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E504" type="decimal">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>